<commit_message>
Podcast w piśmie do MKiDN, zaślepka karty oceny, pomysły z nocy
Karta oceny: plik zamieniony na jednozdaniową zaślepkę kierującą do
Załącznika nr 1 Regulaminu. Dotąd ta sama treść stała pod dwoma adresami.

Pismo i nota dla MKiDN: podcast dopisany jako czwarte działanie, z dwoma
cyklami - "Pierwszy raz" i "NAIstolatek". Kluczowe jest zdanie, że
przedmiotem odcinka nie są odpowiedzi AI, lecz kolejne pytanie człowieka.
Odcinki z nastolatkami za pisemną zgodą opiekunów, z możliwością jej
wycofania przed publikacją.

Budżet Antologii: produkcja podcastu wraz z honorarium prowadzącego jako
pozycja DO WYCENY oraz 72 godziny koordynacji przy 24 odcinkach.
Przy okazji naprawione formuły, które po wstawieniu wiersza wskazywały
na sąsiednie pozycje. Antologia 277 550 -> 298 142 zł netto.

Koncepcja: pomysły z 26.10.2026 zapisane jako nierozstrzygnięte.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="237">
   <si>
     <t xml:space="preserve">Budżet pierwszej edycji Nagrody Konstela</t>
   </si>
@@ -473,6 +473,9 @@
     <t xml:space="preserve">generowanie stron z kopii, nawigacja, tryb redakcji fragmentów</t>
   </si>
   <si>
+    <t xml:space="preserve">Koordynacja podcastu: goście, terminy, publikacja</t>
+  </si>
+  <si>
     <t xml:space="preserve">Powołanie fundacji-organizatora</t>
   </si>
   <si>
@@ -485,6 +488,9 @@
     <t xml:space="preserve">sześć obszarów, w tym licencja i archiwum; obowiązkowa przed naborem</t>
   </si>
   <si>
+    <t xml:space="preserve">sześć obszarów, w tym licencja i archiwum; kwota z zapasem wobec ofert kancelarii</t>
+  </si>
+  <si>
     <t xml:space="preserve">Domeny, poczta, hosting, magazyn kopii archiwalnych</t>
   </si>
   <si>
@@ -539,6 +545,18 @@
     <t xml:space="preserve">Dostęp do narzędzi AI, bez których 937 godzin pracy organizatora nie jest wykonalne; rzędu 2,5 tys. zł miesięcznie</t>
   </si>
   <si>
+    <t xml:space="preserve">Rejestracja znaku towarowego Konstela w EUIPO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jedna klasa, ochrona w całej Unii; opłaty urzędowe około 850 euro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produkcja podcastu wraz z honorarium prowadzącego (24 odcinki)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO WYCENY - nagranie, montaż, dźwięk, wersja wideo i dystrybucja; honorarium prowadzącego nieustalone</t>
+  </si>
+  <si>
     <t xml:space="preserve">Marża (od pracy i kosztów, bez nagród)</t>
   </si>
   <si>
@@ -609,6 +627,21 @@
   </si>
   <si>
     <t xml:space="preserve">DO WYCENY - zależy od miejsca gali, które nie jest wybrane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obsługa prawna plebiscytu (netto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO WYCENY - zakres plebiscytowy nie był objęty wyceną z 22.10.2026; osobne zlecenie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">odrębne zlecenie na pytania plebiscytowe; kwota z zapasem wobec ofert kancelarii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dojazd i nocleg dziesięciu finalistów na galę (netto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO WYCENY - udział czołowej trójki obowiązkowy (§ 14 regulaminu plebiscytu), pokrycie dla całej dziesiątki</t>
   </si>
   <si>
     <t xml:space="preserve">Koszty twarde bez nagród</t>
@@ -858,7 +891,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -885,6 +918,10 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -943,6 +980,18 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -955,8 +1004,8 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -1292,7 +1341,7 @@
       <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="3"/>
@@ -1308,7 +1357,7 @@
       <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <f aca="false">'Budżet Nagrody'!$D$39</f>
         <v>561684.8</v>
       </c>
@@ -1325,9 +1374,9 @@
       <c r="B7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="7" t="n">
-        <f aca="false">'Budżet Antologii'!$D$35</f>
-        <v>271700</v>
+      <c r="C7" s="8" t="n">
+        <f aca="false">'Budżet Antologii'!$D$38</f>
+        <v>298142</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
@@ -1342,8 +1391,8 @@
       <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7" t="n">
-        <f aca="false">'Budżet Plebiscytu'!$D$30</f>
+      <c r="C8" s="8" t="n">
+        <f aca="false">'Budżet Plebiscytu'!$D$32</f>
         <v>256616</v>
       </c>
       <c r="D8" s="3"/>
@@ -1359,7 +1408,7 @@
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="8" t="n">
         <f aca="false">'Budżet Akademii'!$D$27</f>
         <v>49280</v>
       </c>
@@ -1369,9 +1418,9 @@
         <v>14</v>
       </c>
       <c r="B10" s="3"/>
-      <c r="C10" s="8" t="n">
-        <f aca="false">'Budżet Nagrody'!$D$39+'Budżet Antologii'!$D$35+'Budżet Plebiscytu'!$D$30+'Budżet Akademii'!$D$27</f>
-        <v>1139280.8</v>
+      <c r="C10" s="9" t="n">
+        <f aca="false">'Budżet Nagrody'!$D$39+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$32+'Budżet Akademii'!$D$27</f>
+        <v>1165722.8</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -1415,10 +1464,10 @@
       <c r="A14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <v>220</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>18</v>
       </c>
       <c r="D14" s="3"/>
@@ -1431,10 +1480,10 @@
       <c r="A15" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="11" t="s">
         <v>20</v>
       </c>
       <c r="D15" s="3"/>
@@ -1447,10 +1496,10 @@
       <c r="A16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <v>300000</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="11" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="3"/>
@@ -1463,10 +1512,10 @@
       <c r="A17" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <v>10000</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="11" t="s">
         <v>24</v>
       </c>
       <c r="D17" s="3"/>
@@ -1479,10 +1528,10 @@
       <c r="A18" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B18" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>26</v>
       </c>
       <c r="D18" s="3"/>
@@ -1495,10 +1544,10 @@
       <c r="A19" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B19" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="11" t="s">
         <v>28</v>
       </c>
       <c r="D19" s="3"/>
@@ -1511,10 +1560,10 @@
       <c r="A20" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B20" s="10" t="n">
         <v>35000</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>30</v>
       </c>
       <c r="D20" s="3"/>
@@ -1527,10 +1576,10 @@
       <c r="A21" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B21" s="10" t="n">
         <v>4000</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="11" t="s">
         <v>32</v>
       </c>
       <c r="D21" s="3"/>
@@ -1543,10 +1592,10 @@
       <c r="A22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B22" s="10" t="n">
         <v>7500</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>34</v>
       </c>
       <c r="D22" s="3"/>
@@ -1559,10 +1608,10 @@
       <c r="A23" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B23" s="9" t="n">
+      <c r="B23" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="11" t="s">
         <v>36</v>
       </c>
       <c r="D23" s="3"/>
@@ -1575,10 +1624,10 @@
       <c r="A24" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="9" t="n">
+      <c r="B24" s="10" t="n">
         <v>80000</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="11" t="s">
         <v>38</v>
       </c>
       <c r="D24" s="3"/>
@@ -1591,10 +1640,10 @@
       <c r="A25" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B25" s="10" t="n">
         <v>3000</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="11" t="s">
         <v>40</v>
       </c>
       <c r="D25" s="3"/>
@@ -1607,10 +1656,10 @@
       <c r="A26" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="11" t="n">
+      <c r="B26" s="12" t="n">
         <v>0.12</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="11" t="s">
         <v>42</v>
       </c>
       <c r="D26" s="3"/>
@@ -1623,10 +1672,10 @@
       <c r="A27" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="11" t="n">
+      <c r="B27" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="11" t="s">
         <v>44</v>
       </c>
       <c r="D27" s="3"/>
@@ -1639,10 +1688,10 @@
       <c r="A28" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="11" t="n">
+      <c r="B28" s="12" t="n">
         <v>0.12</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="11" t="s">
         <v>42</v>
       </c>
       <c r="D28" s="3"/>
@@ -1655,10 +1704,10 @@
       <c r="A29" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B29" s="11" t="n">
+      <c r="B29" s="12" t="n">
         <v>0.23</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="11" t="s">
         <v>47</v>
       </c>
       <c r="D29" s="3"/>
@@ -1671,10 +1720,10 @@
       <c r="A30" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B30" s="11" t="n">
+      <c r="B30" s="12" t="n">
         <v>0.1</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="11" t="s">
         <v>49</v>
       </c>
       <c r="D30" s="3"/>
@@ -1785,17 +1834,17 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12" t="s">
+      <c r="A41" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B42" s="9" t="n">
+      <c r="B42" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -1806,7 +1855,7 @@
       <c r="A43" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B43" s="13" t="n">
+      <c r="B43" s="14" t="n">
         <v>500</v>
       </c>
       <c r="C43" s="3" t="s">
@@ -1817,7 +1866,7 @@
       <c r="A44" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B44" s="13" t="n">
+      <c r="B44" s="14" t="n">
         <v>2500</v>
       </c>
       <c r="C44" s="3" t="s">
@@ -1828,7 +1877,7 @@
       <c r="A45" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B45" s="9" t="n">
+      <c r="B45" s="10" t="n">
         <v>15</v>
       </c>
       <c r="C45" s="3" t="s">
@@ -1839,7 +1888,7 @@
       <c r="A46" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B46" s="9" t="n">
+      <c r="B46" s="10" t="n">
         <v>20</v>
       </c>
       <c r="C46" s="3" t="s">
@@ -2007,16 +2056,16 @@
       <c r="A6" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>76</v>
       </c>
       <c r="F6" s="6" t="s">
@@ -2026,264 +2075,264 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="16" t="n">
         <v>60</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$15/60</f>
         <v>60</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="18" t="n">
         <f aca="false">D7*Wyjaśnienia!$B$14</f>
         <v>13200</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="11" t="s">
         <v>79</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$15/60</f>
         <v>24</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="18" t="n">
         <f aca="false">D8*Wyjaśnienia!$B$14</f>
         <v>5280</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>81</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$15/60</f>
         <v>50</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="18" t="n">
         <f aca="false">D9*Wyjaśnienia!$B$14</f>
         <v>11000</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>83</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="17" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$15/60</f>
         <v>23</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="18" t="n">
         <f aca="false">D10*Wyjaśnienia!$B$14</f>
         <v>5060</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>85</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="17" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$15/60</f>
         <v>20</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="18" t="n">
         <f aca="false">D11*Wyjaśnienia!$B$14</f>
         <v>4400</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="11" t="s">
         <v>87</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="17" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$15/60</f>
         <v>20</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="18" t="n">
         <f aca="false">D12*Wyjaśnienia!$B$14</f>
         <v>4400</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>89</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="17" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$15/60</f>
         <v>40</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="18" t="n">
         <f aca="false">D13*Wyjaśnienia!$B$14</f>
         <v>8800</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>91</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="17" t="n">
         <f aca="false">B14+C14*Wyjaśnienia!$B$15/60</f>
         <v>25</v>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="18" t="n">
         <f aca="false">D14*Wyjaśnienia!$B$14</f>
         <v>5500</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="11" t="s">
         <v>93</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B15" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="17" t="n">
         <f aca="false">B15+C15*Wyjaśnienia!$B$15/60</f>
         <v>45</v>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="18" t="n">
         <f aca="false">D15*Wyjaśnienia!$B$14</f>
         <v>9900</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" s="11" t="s">
         <v>95</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="16" t="n">
+      <c r="D16" s="17" t="n">
         <f aca="false">B16+C16*Wyjaśnienia!$B$15/60</f>
         <v>25</v>
       </c>
-      <c r="E16" s="17" t="n">
+      <c r="E16" s="18" t="n">
         <f aca="false">D16*Wyjaśnienia!$B$14</f>
         <v>5500</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="11" t="s">
         <v>97</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="B17" s="15" t="n">
+      <c r="B17" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="C17" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="16" t="n">
+      <c r="D17" s="17" t="n">
         <f aca="false">B17+C17*Wyjaśnienia!$B$15/60</f>
         <v>40</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="18" t="n">
         <f aca="false">D17*Wyjaśnienia!$B$14</f>
         <v>8800</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="11" t="s">
         <v>99</v>
       </c>
       <c r="G17" s="3"/>
@@ -2295,11 +2344,11 @@
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
-      <c r="D18" s="18" t="n">
+      <c r="D18" s="19" t="n">
         <f aca="false">SUM(D7:D17)</f>
         <v>372</v>
       </c>
-      <c r="E18" s="8" t="n">
+      <c r="E18" s="9" t="n">
         <f aca="false">SUM(E7:E17)</f>
         <v>81840</v>
       </c>
@@ -2333,13 +2382,13 @@
       <c r="A21" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>76</v>
       </c>
       <c r="E21" s="6" t="s">
@@ -2350,20 +2399,20 @@
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="B22" s="19" t="n">
+      <c r="B22" s="20" t="n">
         <v>8000</v>
       </c>
-      <c r="C22" s="15" t="n">
+      <c r="C22" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="18" t="n">
         <f aca="false">B22*C22</f>
         <v>8000</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="11" t="s">
         <v>105</v>
       </c>
       <c r="F22" s="3"/>
@@ -2371,20 +2420,20 @@
       <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="B23" s="19" t="n">
+      <c r="B23" s="20" t="n">
         <v>1500</v>
       </c>
-      <c r="C23" s="15" t="n">
+      <c r="C23" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="D23" s="18" t="n">
         <f aca="false">B23*C23</f>
         <v>1500</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" s="11" t="s">
         <v>107</v>
       </c>
       <c r="F23" s="3"/>
@@ -2392,20 +2441,20 @@
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B24" s="19" t="n">
+      <c r="B24" s="20" t="n">
         <v>1200</v>
       </c>
-      <c r="C24" s="15" t="n">
+      <c r="C24" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="18" t="n">
         <f aca="false">B24*C24</f>
         <v>1200</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" s="11" t="s">
         <v>109</v>
       </c>
       <c r="F24" s="3"/>
@@ -2413,20 +2462,20 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="B25" s="19" t="n">
+      <c r="B25" s="20" t="n">
         <v>4000</v>
       </c>
-      <c r="C25" s="15" t="n">
+      <c r="C25" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="17" t="n">
+      <c r="D25" s="18" t="n">
         <f aca="false">B25*C25</f>
         <v>4000</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" s="11" t="s">
         <v>111</v>
       </c>
       <c r="F25" s="3"/>
@@ -2434,20 +2483,20 @@
       <c r="H25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="B26" s="19" t="n">
+      <c r="B26" s="20" t="n">
         <v>1500</v>
       </c>
-      <c r="C26" s="15" t="n">
+      <c r="C26" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="18" t="n">
         <f aca="false">B26*C26</f>
         <v>1500</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="11" t="s">
         <v>113</v>
       </c>
       <c r="F26" s="3"/>
@@ -2455,20 +2504,20 @@
       <c r="H26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="B27" s="19" t="n">
+      <c r="B27" s="20" t="n">
         <v>250</v>
       </c>
-      <c r="C27" s="15" t="n">
+      <c r="C27" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="18" t="n">
         <f aca="false">B27*C27</f>
         <v>250</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" s="11" t="s">
         <v>115</v>
       </c>
       <c r="F27" s="3"/>
@@ -2476,20 +2525,20 @@
       <c r="H27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="B28" s="19" t="n">
+      <c r="B28" s="20" t="n">
         <v>32000</v>
       </c>
-      <c r="C28" s="15" t="n">
+      <c r="C28" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="18" t="n">
         <f aca="false">B28*C28</f>
         <v>32000</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" s="11" t="s">
         <v>117</v>
       </c>
       <c r="F28" s="3" t="s">
@@ -2499,20 +2548,20 @@
       <c r="H28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="B29" s="19" t="n">
+      <c r="B29" s="20" t="n">
         <v>15000</v>
       </c>
-      <c r="C29" s="15" t="n">
+      <c r="C29" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="18" t="n">
         <f aca="false">B29*C29</f>
         <v>15000</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" s="11" t="s">
         <v>120</v>
       </c>
       <c r="F29" s="3"/>
@@ -2520,20 +2569,20 @@
       <c r="H29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="B30" s="19" t="n">
+      <c r="B30" s="20" t="n">
         <v>8000</v>
       </c>
-      <c r="C30" s="15" t="n">
+      <c r="C30" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="18" t="n">
         <f aca="false">B30*C30</f>
         <v>8000</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="11" t="s">
         <v>122</v>
       </c>
       <c r="F30" s="3"/>
@@ -2541,20 +2590,20 @@
       <c r="H30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
+      <c r="A31" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="B31" s="19" t="n">
+      <c r="B31" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="15" t="n">
+      <c r="C31" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D31" s="17" t="n">
+      <c r="D31" s="18" t="n">
         <f aca="false">B31*C31</f>
         <v>0</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="11" t="s">
         <v>124</v>
       </c>
       <c r="F31" s="3"/>
@@ -2567,7 +2616,7 @@
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
-      <c r="D32" s="8" t="n">
+      <c r="D32" s="9" t="n">
         <f aca="false">SUM(D22:D31)</f>
         <v>71450</v>
       </c>
@@ -2599,12 +2648,12 @@
       <c r="H34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="s">
+      <c r="A35" s="15" t="s">
         <v>127</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
-      <c r="D35" s="17" t="n">
+      <c r="D35" s="18" t="n">
         <f aca="false">Wyjaśnienia!$B$16+Wyjaśnienia!$B$17*Wyjaśnienia!$B$18</f>
         <v>390000</v>
       </c>
@@ -2614,12 +2663,12 @@
       <c r="H35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
+      <c r="A36" s="15" t="s">
         <v>128</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
-      <c r="D36" s="7" t="n">
+      <c r="D36" s="8" t="n">
         <f aca="false">E18</f>
         <v>81840</v>
       </c>
@@ -2629,12 +2678,12 @@
       <c r="H36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="s">
+      <c r="A37" s="15" t="s">
         <v>129</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
-      <c r="D37" s="7" t="n">
+      <c r="D37" s="8" t="n">
         <f aca="false">D32</f>
         <v>71450</v>
       </c>
@@ -2644,12 +2693,12 @@
       <c r="H37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14" t="s">
+      <c r="A38" s="15" t="s">
         <v>130</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
-      <c r="D38" s="7" t="n">
+      <c r="D38" s="8" t="n">
         <f aca="false">(D36+D37)*Wyjaśnienia!$B$26</f>
         <v>18394.8</v>
       </c>
@@ -2664,7 +2713,7 @@
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
-      <c r="D39" s="8" t="n">
+      <c r="D39" s="9" t="n">
         <f aca="false">SUM(D35:D38)</f>
         <v>561684.8</v>
       </c>
@@ -2674,12 +2723,12 @@
       <c r="H39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14" t="s">
+      <c r="A40" s="15" t="s">
         <v>132</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
-      <c r="D40" s="7" t="n">
+      <c r="D40" s="8" t="n">
         <f aca="false">D39*Wyjaśnienia!$B$29</f>
         <v>129187.504</v>
       </c>
@@ -2694,7 +2743,7 @@
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
-      <c r="D41" s="20" t="n">
+      <c r="D41" s="21" t="n">
         <f aca="false">D39+D40</f>
         <v>690872.304</v>
       </c>
@@ -2864,16 +2913,16 @@
       <c r="A6" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>76</v>
       </c>
       <c r="F6" s="6" t="s">
@@ -2883,311 +2932,312 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$15/60</f>
         <v>45</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="18" t="n">
         <f aca="false">D7*Wyjaśnienia!$B$14</f>
         <v>9900</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="11" t="s">
         <v>136</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="15" t="s">
         <v>137</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$15/60</f>
         <v>40</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="18" t="n">
         <f aca="false">D8*Wyjaśnienia!$B$14</f>
         <v>8800</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>138</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$15/60</f>
         <v>30</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="18" t="n">
         <f aca="false">D9*Wyjaśnienia!$B$14</f>
         <v>6600</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="11" t="s">
         <v>140</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="17" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$15/60</f>
         <v>50</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="18" t="n">
         <f aca="false">D10*Wyjaśnienia!$B$14</f>
         <v>11000</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="11" t="s">
         <v>142</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="17" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$15/60</f>
         <v>25</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="18" t="n">
         <f aca="false">D11*Wyjaśnienia!$B$14</f>
         <v>5500</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" s="11" t="s">
         <v>144</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="16" t="n">
         <v>160</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="17" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$15/60</f>
         <v>160</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="18" t="n">
         <f aca="false">D12*Wyjaśnienia!$B$14</f>
         <v>35200</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="11" t="s">
         <v>146</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="17" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$15/60</f>
         <v>50</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="18" t="n">
         <f aca="false">D13*Wyjaśnienia!$B$14</f>
         <v>11000</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="11" t="s">
         <v>148</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>72</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="17" t="n">
+        <f aca="false">B14+C14*Wyjaśnienia!$B$15/60</f>
+        <v>72</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <f aca="false">D14*Wyjaśnienia!$B$14</f>
+        <v>15840</v>
+      </c>
+      <c r="F14" s="11"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="18" t="n">
-        <f aca="false">SUM(D7:D13)</f>
-        <v>400</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <f aca="false">SUM(E7:E13)</f>
-        <v>88000</v>
-      </c>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="D15" s="19" t="n">
+        <f aca="false">SUM(D7:D14)</f>
+        <v>472</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <f aca="false">SUM(E7:E14)</f>
+        <v>103840</v>
+      </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="F17" s="3"/>
+      <c r="A17" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="B18" s="19" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C18" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="17" t="n">
-        <f aca="false">B18*C18</f>
-        <v>3000</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>150</v>
+      <c r="A18" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>77</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <f aca="false">B19*C19</f>
+        <v>3000</v>
+      </c>
+      <c r="E19" s="11" t="s">
         <v>151</v>
-      </c>
-      <c r="B19" s="19" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C19" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="17" t="n">
-        <f aca="false">B19*C19</f>
-        <v>6000</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>152</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="B20" s="20" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C20" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="18" t="n">
+        <f aca="false">B20*C20</f>
+        <v>6000</v>
+      </c>
+      <c r="E20" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="B20" s="19" t="n">
-        <v>10000</v>
-      </c>
-      <c r="C20" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="17" t="n">
-        <f aca="false">B20*C20</f>
-        <v>10000</v>
-      </c>
-      <c r="E20" s="10" t="s">
+      <c r="F20" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="B21" s="19" t="n">
-        <v>40000</v>
-      </c>
-      <c r="C21" s="15" t="n">
+      <c r="B21" s="20" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C21" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="D21" s="18" t="n">
         <f aca="false">B21*C21</f>
-        <v>40000</v>
-      </c>
-      <c r="E21" s="10" t="s">
+        <v>10000</v>
+      </c>
+      <c r="E21" s="11" t="s">
         <v>156</v>
       </c>
       <c r="F21" s="3"/>
@@ -3195,20 +3245,20 @@
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="B22" s="19" t="n">
-        <v>4000</v>
-      </c>
-      <c r="C22" s="15" t="n">
+      <c r="B22" s="20" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C22" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="18" t="n">
         <f aca="false">B22*C22</f>
-        <v>4000</v>
-      </c>
-      <c r="E22" s="10" t="s">
+        <v>40000</v>
+      </c>
+      <c r="E22" s="11" t="s">
         <v>158</v>
       </c>
       <c r="F22" s="3"/>
@@ -3216,20 +3266,20 @@
       <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="B23" s="19" t="n">
-        <v>3000</v>
-      </c>
-      <c r="C23" s="15" t="n">
+      <c r="B23" s="20" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C23" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="D23" s="18" t="n">
         <f aca="false">B23*C23</f>
-        <v>3000</v>
-      </c>
-      <c r="E23" s="10" t="s">
+        <v>4000</v>
+      </c>
+      <c r="E23" s="11" t="s">
         <v>160</v>
       </c>
       <c r="F23" s="3"/>
@@ -3237,20 +3287,20 @@
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="B24" s="19" t="n">
-        <v>4000</v>
-      </c>
-      <c r="C24" s="15" t="n">
+      <c r="B24" s="20" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C24" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="18" t="n">
         <f aca="false">B24*C24</f>
-        <v>4000</v>
-      </c>
-      <c r="E24" s="10" t="s">
+        <v>3000</v>
+      </c>
+      <c r="E24" s="11" t="s">
         <v>162</v>
       </c>
       <c r="F24" s="3"/>
@@ -3258,20 +3308,20 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="B25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="15" t="n">
+      <c r="B25" s="20" t="n">
+        <v>4000</v>
+      </c>
+      <c r="C25" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="17" t="n">
+      <c r="D25" s="18" t="n">
         <f aca="false">B25*C25</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="10" t="s">
+        <v>4000</v>
+      </c>
+      <c r="E25" s="11" t="s">
         <v>164</v>
       </c>
       <c r="F25" s="3"/>
@@ -3279,20 +3329,20 @@
       <c r="H25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="B26" s="19" t="n">
-        <v>15000</v>
-      </c>
-      <c r="C26" s="15" t="n">
+      <c r="B26" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="18" t="n">
         <f aca="false">B26*C26</f>
-        <v>15000</v>
-      </c>
-      <c r="E26" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="E26" s="11" t="s">
         <v>166</v>
       </c>
       <c r="F26" s="3"/>
@@ -3300,20 +3350,20 @@
       <c r="H26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
+      <c r="A27" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="B27" s="19" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C27" s="15" t="n">
+      <c r="B27" s="20" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C27" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="18" t="n">
         <f aca="false">B27*C27</f>
-        <v>6000</v>
-      </c>
-      <c r="E27" s="10" t="s">
+        <v>15000</v>
+      </c>
+      <c r="E27" s="11" t="s">
         <v>168</v>
       </c>
       <c r="F27" s="3"/>
@@ -3321,20 +3371,20 @@
       <c r="H27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
+      <c r="A28" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="B28" s="19" t="n">
-        <v>30000</v>
-      </c>
-      <c r="C28" s="15" t="n">
+      <c r="B28" s="20" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C28" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="18" t="n">
         <f aca="false">B28*C28</f>
-        <v>30000</v>
-      </c>
-      <c r="E28" s="10" t="s">
+        <v>6000</v>
+      </c>
+      <c r="E28" s="11" t="s">
         <v>170</v>
       </c>
       <c r="F28" s="3"/>
@@ -3342,51 +3392,72 @@
       <c r="H28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="8" t="n">
-        <f aca="false">SUM(D18:D28)</f>
-        <v>121000</v>
-      </c>
-      <c r="E29" s="3"/>
+      <c r="A29" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C29" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="18" t="n">
+        <f aca="false">B29*C29</f>
+        <v>30000</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>172</v>
+      </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
+      <c r="A30" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <f aca="false">B30*C30</f>
+        <v>4500</v>
+      </c>
+      <c r="F30" s="22" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
+      <c r="A31" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <f aca="false">B31*C31</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F31" s="22"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="14" t="s">
-        <v>128</v>
+      <c r="A32" s="6" t="s">
+        <v>125</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
-      <c r="D32" s="7" t="n">
-        <f aca="false">E14</f>
-        <v>88000</v>
+      <c r="D32" s="9" t="n">
+        <f aca="false">SUM(D19:D31)</f>
+        <v>125500</v>
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
@@ -3394,44 +3465,36 @@
       <c r="H32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="7" t="n">
-        <f aca="false">D29</f>
-        <v>121000</v>
-      </c>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="24"/>
+      <c r="C33" s="24"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="7" t="n">
-        <f aca="false">(D32+D33)*Wyjaśnienia!$B$27</f>
-        <v>62700</v>
-      </c>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
+      <c r="A34" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
-        <v>131</v>
+      <c r="A35" s="15" t="s">
+        <v>128</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="8" t="n">
-        <f aca="false">SUM(D32:D34)</f>
-        <v>271700</v>
+        <f aca="false">E15</f>
+        <v>103840</v>
       </c>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
@@ -3439,14 +3502,14 @@
       <c r="H35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
-        <v>132</v>
+      <c r="A36" s="15" t="s">
+        <v>129</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
-      <c r="D36" s="7" t="n">
-        <f aca="false">D35*Wyjaśnienia!$B$29</f>
-        <v>62491</v>
+      <c r="D36" s="8" t="n">
+        <f aca="false">D32</f>
+        <v>125500</v>
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -3454,23 +3517,65 @@
       <c r="H36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
-        <v>133</v>
+      <c r="A37" s="15" t="s">
+        <v>177</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
-      <c r="D37" s="20" t="n">
-        <f aca="false">D35+D36</f>
-        <v>334191</v>
+      <c r="D37" s="8" t="n">
+        <f aca="false">(D35+D36)*Wyjaśnienia!$B$27</f>
+        <v>68802</v>
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="9" t="n">
+        <f aca="false">SUM(D35:D37)</f>
+        <v>298142</v>
+      </c>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="8" t="n">
+        <f aca="false">D38*Wyjaśnienia!$B$29</f>
+        <v>68572.66</v>
+      </c>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="21" t="n">
+        <f aca="false">D38+D39</f>
+        <v>366714.66</v>
+      </c>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+    </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3537,13 +3642,14 @@
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A34:F34"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3585,7 +3691,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -3633,16 +3739,16 @@
       <c r="A6" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>76</v>
       </c>
       <c r="F6" s="6" t="s">
@@ -3652,121 +3758,121 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="B7" s="15" t="n">
+      <c r="A7" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="17" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$19/60</f>
         <v>25</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="18" t="n">
         <f aca="false">D7*Wyjaśnienia!$B$14</f>
         <v>5500</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>174</v>
+      <c r="F7" s="11" t="s">
+        <v>180</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="B8" s="15" t="n">
+      <c r="A8" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="B8" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$19/60</f>
         <v>40</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="18" t="n">
         <f aca="false">D8*Wyjaśnienia!$B$14</f>
         <v>8800</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>176</v>
+      <c r="F8" s="11" t="s">
+        <v>182</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="15" t="n">
+      <c r="A9" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="B9" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$19/60</f>
         <v>30</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="18" t="n">
         <f aca="false">D9*Wyjaśnienia!$B$14</f>
         <v>6600</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>178</v>
+      <c r="F9" s="11" t="s">
+        <v>184</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="B10" s="15" t="n">
+      <c r="A10" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="B10" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="17" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$19/60</f>
         <v>20</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="18" t="n">
         <f aca="false">D10*Wyjaśnienia!$B$14</f>
         <v>4400</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>180</v>
+      <c r="F10" s="11" t="s">
+        <v>186</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="B11" s="15" t="n">
+      <c r="A11" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="B11" s="16" t="n">
         <v>50</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="17" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$19/60</f>
         <v>50</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="18" t="n">
         <f aca="false">D11*Wyjaśnienia!$B$14</f>
         <v>11000</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>182</v>
+      <c r="F11" s="11" t="s">
+        <v>188</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -3777,11 +3883,11 @@
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="19" t="n">
         <f aca="false">SUM(D7:D11)</f>
         <v>165</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="9" t="n">
         <f aca="false">SUM(E7:E11)</f>
         <v>36300</v>
       </c>
@@ -3815,13 +3921,13 @@
       <c r="A15" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="7" t="s">
         <v>76</v>
       </c>
       <c r="E15" s="6" t="s">
@@ -3832,234 +3938,244 @@
       <c r="H15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="B16" s="17" t="n">
+      <c r="A16" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" s="18" t="n">
         <f aca="false">Wyjaśnienia!$B$20</f>
         <v>35000</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="18" t="n">
         <f aca="false">B16*C16</f>
         <v>35000</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>184</v>
+      <c r="E16" s="11" t="s">
+        <v>190</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="B17" s="17" t="n">
+      <c r="A17" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" s="18" t="n">
         <f aca="false">Wyjaśnienia!$B$21</f>
         <v>4000</v>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="C17" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="D17" s="18" t="n">
         <f aca="false">B17*C17</f>
         <v>4000</v>
       </c>
-      <c r="E17" s="10" t="s">
-        <v>186</v>
+      <c r="E17" s="11" t="s">
+        <v>192</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="B18" s="17" t="n">
+      <c r="A18" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="B18" s="18" t="n">
         <f aca="false">Wyjaśnienia!$B$22</f>
         <v>7500</v>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C18" s="17" t="n">
         <f aca="false">Wyjaśnienia!$B$23</f>
         <v>10</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="18" t="n">
         <f aca="false">B18*C18</f>
         <v>75000</v>
       </c>
-      <c r="E18" s="10" t="s">
-        <v>188</v>
+      <c r="E18" s="11" t="s">
+        <v>194</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="17" t="n">
+      <c r="B19" s="18" t="n">
         <f aca="false">Wyjaśnienia!$B$24</f>
         <v>80000</v>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="C19" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="D19" s="18" t="n">
         <f aca="false">B19*C19</f>
         <v>80000</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>189</v>
+      <c r="E19" s="11" t="s">
+        <v>195</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="18" t="n">
         <f aca="false">Wyjaśnienia!$B$25</f>
         <v>3000</v>
       </c>
-      <c r="C20" s="15" t="n">
+      <c r="C20" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="18" t="n">
         <f aca="false">B20*C20</f>
         <v>3000</v>
       </c>
-      <c r="E20" s="10" t="s">
-        <v>190</v>
+      <c r="E20" s="11" t="s">
+        <v>196</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
-        <v>191</v>
-      </c>
-      <c r="B21" s="19" t="n">
+      <c r="A21" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="B21" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="C21" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="D21" s="18" t="n">
         <f aca="false">B21*C21</f>
         <v>0</v>
       </c>
-      <c r="E21" s="10" t="s">
-        <v>192</v>
+      <c r="E21" s="11" t="s">
+        <v>198</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="B22" s="19" t="n">
+      <c r="A22" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="B22" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="15" t="n">
+      <c r="C22" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="18" t="n">
         <f aca="false">B22*C22</f>
         <v>0</v>
       </c>
-      <c r="E22" s="10" t="s">
-        <v>194</v>
+      <c r="E22" s="11" t="s">
+        <v>200</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <f aca="false">B23*C23</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="F23" s="22" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="22" t="s">
+        <v>204</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <f aca="false">B24*C24</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F24" s="22"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="8" t="n">
-        <f aca="false">SUM(D16:D22)</f>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="19" t="n">
+        <f aca="false">SUM(D16:D24)</f>
         <v>197000</v>
       </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="24"/>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="17" t="n">
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="18" t="n">
         <f aca="false">Wyjaśnienia!$B$20+Wyjaśnienia!$B$21</f>
         <v>39000</v>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="7" t="n">
-        <f aca="false">E12</f>
-        <v>36300</v>
-      </c>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="7" t="n">
-        <f aca="false">D23-D26</f>
-        <v>158000</v>
       </c>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
@@ -4067,14 +4183,14 @@
       <c r="H28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="14" t="s">
-        <v>130</v>
+      <c r="A29" s="15" t="s">
+        <v>128</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
-      <c r="D29" s="7" t="n">
-        <f aca="false">(D27+D28)*Wyjaśnienia!$B$28</f>
-        <v>23316</v>
+      <c r="D29" s="8" t="n">
+        <f aca="false">E12</f>
+        <v>36300</v>
       </c>
       <c r="E29" s="3"/>
       <c r="F29" s="3"/>
@@ -4082,14 +4198,14 @@
       <c r="H29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>131</v>
+      <c r="A30" s="15" t="s">
+        <v>206</v>
       </c>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="8" t="n">
-        <f aca="false">SUM(D26:D29)</f>
-        <v>256616</v>
+        <f aca="false">D25-D28</f>
+        <v>158000</v>
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
@@ -4097,14 +4213,14 @@
       <c r="H30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="14" t="s">
-        <v>132</v>
+      <c r="A31" s="15" t="s">
+        <v>130</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
-      <c r="D31" s="7" t="n">
-        <f aca="false">D30*Wyjaśnienia!$B$29</f>
-        <v>59021.68</v>
+      <c r="D31" s="8" t="n">
+        <f aca="false">(D29+D30)*Wyjaśnienia!$B$28</f>
+        <v>23316</v>
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
@@ -4113,21 +4229,49 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
-      <c r="D32" s="20" t="n">
-        <f aca="false">D30+D31</f>
-        <v>315637.68</v>
+      <c r="D32" s="9" t="n">
+        <f aca="false">SUM(D28:D31)</f>
+        <v>256616</v>
       </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="8" t="n">
+        <f aca="false">D32*Wyjaśnienia!$B$29</f>
+        <v>59021.68</v>
+      </c>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="21" t="n">
+        <f aca="false">D32+D33</f>
+        <v>315637.68</v>
+      </c>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+    </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -4200,13 +4344,14 @@
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A25:F25"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A27:F27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4235,533 +4380,533 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
-        <v>196</v>
-      </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
+      <c r="A2" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
-        <v>197</v>
-      </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="A3" s="26" t="s">
+        <v>208</v>
+      </c>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
+      <c r="A5" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="23" t="s">
-        <v>199</v>
-      </c>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="23" t="s">
+      <c r="B6" s="28" t="s">
+        <v>210</v>
+      </c>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="27" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="B7" s="25" t="n">
+      <c r="A7" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="B7" s="29" t="n">
         <f aca="false">Wyjaśnienia!$B$15</f>
         <v>150</v>
       </c>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24" t="s">
-        <v>201</v>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
-        <v>202</v>
-      </c>
-      <c r="B8" s="25" t="n">
+      <c r="A8" s="22" t="s">
+        <v>213</v>
+      </c>
+      <c r="B8" s="29" t="n">
         <f aca="false">Wyjaśnienia!$B$42</f>
         <v>2</v>
       </c>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24" t="s">
-        <v>203</v>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="B9" s="26" t="n">
+      <c r="A9" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="B9" s="30" t="n">
         <f aca="false">B7*B8</f>
         <v>300</v>
       </c>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>206</v>
-      </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
+      <c r="A11" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="23" t="s">
-        <v>207</v>
-      </c>
-      <c r="C12" s="23" t="s">
+      <c r="B12" s="28" t="s">
+        <v>218</v>
+      </c>
+      <c r="C12" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="24"/>
-      <c r="F12" s="23" t="s">
+      <c r="E12" s="22"/>
+      <c r="F12" s="27" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="B13" s="27" t="n">
+      <c r="A13" s="22" t="s">
+        <v>219</v>
+      </c>
+      <c r="B13" s="31" t="n">
         <f aca="false">Wyjaśnienia!$B$44</f>
         <v>2500</v>
       </c>
-      <c r="C13" s="25" t="n">
+      <c r="C13" s="29" t="n">
         <f aca="false">Wyjaśnienia!$B$45</f>
         <v>15</v>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D13" s="31" t="n">
         <f aca="false">B13*C13</f>
         <v>37500</v>
       </c>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24" t="s">
-        <v>209</v>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
-        <v>210</v>
-      </c>
-      <c r="B14" s="27" t="n">
+      <c r="A14" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="B14" s="31" t="n">
         <f aca="false">Wyjaśnienia!$B$43</f>
         <v>500</v>
       </c>
-      <c r="C14" s="25" t="n">
+      <c r="C14" s="29" t="n">
         <f aca="false">ROUNDUP(B9/100,0)</f>
         <v>3</v>
       </c>
-      <c r="D14" s="27" t="n">
+      <c r="D14" s="31" t="n">
         <f aca="false">B14*C14</f>
         <v>1500</v>
       </c>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24" t="s">
-        <v>211</v>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="28" t="n">
+      <c r="A15" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="32" t="n">
         <f aca="false">SUM(D13:D14)</f>
         <v>39000</v>
       </c>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="28" t="s">
         <v>102</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="D18" s="23" t="s">
+      <c r="D18" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="E18" s="24"/>
-      <c r="F18" s="23" t="s">
+      <c r="E18" s="22"/>
+      <c r="F18" s="27" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24" t="s">
-        <v>213</v>
-      </c>
-      <c r="B19" s="29" t="n">
+      <c r="A19" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="B19" s="33" t="n">
         <v>2000</v>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C19" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="27" t="n">
+      <c r="D19" s="31" t="n">
         <f aca="false">B19*C19</f>
         <v>2000</v>
       </c>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24" t="s">
-        <v>214</v>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="24" t="s">
-        <v>215</v>
-      </c>
-      <c r="B20" s="29" t="n">
+      <c r="A20" s="22" t="s">
+        <v>226</v>
+      </c>
+      <c r="B20" s="33" t="n">
         <v>3000</v>
       </c>
-      <c r="C20" s="24" t="n">
+      <c r="C20" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="27" t="n">
+      <c r="D20" s="31" t="n">
         <f aca="false">B20*C20</f>
         <v>3000</v>
       </c>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24" t="s">
-        <v>216</v>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="27" t="s">
         <v>125</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="28" t="n">
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="32" t="n">
         <f aca="false">SUM(D19:D20)</f>
         <v>5000</v>
       </c>
-      <c r="E21" s="24"/>
-      <c r="F21" s="24"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24"/>
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="24" t="s">
-        <v>217</v>
-      </c>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="27" t="n">
+      <c r="A24" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="31" t="n">
         <f aca="false">D15</f>
         <v>39000</v>
       </c>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="24" t="s">
+      <c r="A25" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="27" t="n">
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="31" t="n">
         <f aca="false">D21</f>
         <v>5000</v>
       </c>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="24" t="s">
-        <v>218</v>
-      </c>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="27" t="n">
+      <c r="A26" s="22" t="s">
+        <v>229</v>
+      </c>
+      <c r="B26" s="22"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="31" t="n">
         <f aca="false">(D24+D25)*Wyjaśnienia!$B$26</f>
         <v>5280</v>
       </c>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
+      <c r="A27" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="28" t="n">
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="32" t="n">
         <f aca="false">SUM(D24:D26)</f>
         <v>49280</v>
       </c>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="24" t="s">
+      <c r="A28" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="27" t="n">
+      <c r="B28" s="22"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="31" t="n">
         <f aca="false">D27*Wyjaśnienia!$B$29</f>
         <v>11334.4</v>
       </c>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="23" t="s">
+      <c r="A29" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="28" t="n">
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="32" t="n">
         <f aca="false">D27+D28</f>
         <v>60614.4</v>
       </c>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="24"/>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="22"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
+      <c r="A31" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
+      <c r="A32" s="26" t="s">
+        <v>231</v>
+      </c>
+      <c r="B32" s="26"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="26"/>
+      <c r="F32" s="26"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
-        <v>221</v>
-      </c>
-      <c r="B33" s="23" t="s">
-        <v>222</v>
-      </c>
-      <c r="C33" s="23" t="s">
-        <v>223</v>
-      </c>
-      <c r="D33" s="23" t="s">
-        <v>224</v>
-      </c>
-      <c r="E33" s="23" t="s">
-        <v>225</v>
-      </c>
-      <c r="F33" s="24"/>
+      <c r="A33" s="28" t="s">
+        <v>232</v>
+      </c>
+      <c r="B33" s="28" t="s">
+        <v>233</v>
+      </c>
+      <c r="C33" s="28" t="s">
+        <v>234</v>
+      </c>
+      <c r="D33" s="28" t="s">
+        <v>235</v>
+      </c>
+      <c r="E33" s="28" t="s">
+        <v>236</v>
+      </c>
+      <c r="F33" s="22"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="n">
+      <c r="A34" s="29" t="n">
         <v>150</v>
       </c>
-      <c r="B34" s="25" t="n">
+      <c r="B34" s="29" t="n">
         <f aca="false">A34*Wyjaśnienia!$B$42</f>
         <v>300</v>
       </c>
-      <c r="C34" s="25" t="n">
+      <c r="C34" s="29" t="n">
         <f aca="false">ROUNDUP(B34/100,0)</f>
         <v>3</v>
       </c>
-      <c r="D34" s="27" t="n">
+      <c r="D34" s="31" t="n">
         <f aca="false">C34*Wyjaśnienia!$B$43</f>
         <v>1500</v>
       </c>
-      <c r="E34" s="25" t="n">
+      <c r="E34" s="29" t="n">
         <f aca="false">ROUNDUP(A34/Wyjaśnienia!$B$46,0)</f>
         <v>8</v>
       </c>
-      <c r="F34" s="24"/>
+      <c r="F34" s="22"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="25" t="n">
+      <c r="A35" s="29" t="n">
         <v>1000</v>
       </c>
-      <c r="B35" s="25" t="n">
+      <c r="B35" s="29" t="n">
         <f aca="false">A35*Wyjaśnienia!$B$42</f>
         <v>2000</v>
       </c>
-      <c r="C35" s="25" t="n">
+      <c r="C35" s="29" t="n">
         <f aca="false">ROUNDUP(B35/100,0)</f>
         <v>20</v>
       </c>
-      <c r="D35" s="27" t="n">
+      <c r="D35" s="31" t="n">
         <f aca="false">C35*Wyjaśnienia!$B$43</f>
         <v>10000</v>
       </c>
-      <c r="E35" s="25" t="n">
+      <c r="E35" s="29" t="n">
         <f aca="false">ROUNDUP(A35/Wyjaśnienia!$B$46,0)</f>
         <v>50</v>
       </c>
-      <c r="F35" s="24"/>
+      <c r="F35" s="22"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="25" t="n">
+      <c r="A36" s="29" t="n">
         <v>10000</v>
       </c>
-      <c r="B36" s="25" t="n">
+      <c r="B36" s="29" t="n">
         <f aca="false">A36*Wyjaśnienia!$B$42</f>
         <v>20000</v>
       </c>
-      <c r="C36" s="25" t="n">
+      <c r="C36" s="29" t="n">
         <f aca="false">ROUNDUP(B36/100,0)</f>
         <v>200</v>
       </c>
-      <c r="D36" s="27" t="n">
+      <c r="D36" s="31" t="n">
         <f aca="false">C36*Wyjaśnienia!$B$43</f>
         <v>100000</v>
       </c>
-      <c r="E36" s="25" t="n">
+      <c r="E36" s="29" t="n">
         <f aca="false">ROUNDUP(A36/Wyjaśnienia!$B$46,0)</f>
         <v>500</v>
       </c>
-      <c r="F36" s="24"/>
+      <c r="F36" s="22"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="n">
+      <c r="A37" s="29" t="n">
         <v>100000</v>
       </c>
-      <c r="B37" s="25" t="n">
+      <c r="B37" s="29" t="n">
         <f aca="false">A37*Wyjaśnienia!$B$42</f>
         <v>200000</v>
       </c>
-      <c r="C37" s="25" t="n">
+      <c r="C37" s="29" t="n">
         <f aca="false">ROUNDUP(B37/100,0)</f>
         <v>2000</v>
       </c>
-      <c r="D37" s="27" t="n">
+      <c r="D37" s="31" t="n">
         <f aca="false">C37*Wyjaśnienia!$B$43</f>
         <v>1000000</v>
       </c>
-      <c r="E37" s="25" t="n">
+      <c r="E37" s="29" t="n">
         <f aca="false">ROUNDUP(A37/Wyjaśnienia!$B$46,0)</f>
         <v>5000</v>
       </c>
-      <c r="F37" s="24"/>
+      <c r="F37" s="22"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="25" t="n">
+      <c r="A38" s="29" t="n">
         <v>1000000</v>
       </c>
-      <c r="B38" s="25" t="n">
+      <c r="B38" s="29" t="n">
         <f aca="false">A38*Wyjaśnienia!$B$42</f>
         <v>2000000</v>
       </c>
-      <c r="C38" s="25" t="n">
+      <c r="C38" s="29" t="n">
         <f aca="false">ROUNDUP(B38/100,0)</f>
         <v>20000</v>
       </c>
-      <c r="D38" s="27" t="n">
+      <c r="D38" s="31" t="n">
         <f aca="false">C38*Wyjaśnienia!$B$43</f>
         <v>10000000</v>
       </c>
-      <c r="E38" s="25" t="n">
+      <c r="E38" s="29" t="n">
         <f aca="false">ROUNDUP(A38/Wyjaśnienia!$B$46,0)</f>
         <v>50000</v>
       </c>
-      <c r="F38" s="24"/>
+      <c r="F38" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
Honoraria jury plakatu wracaja na DO USTALENIA
Pozycja stala na 14 500 zl jako 5 osob razy 10 godzin razy 290 zl, czyli
stawka Kapituly. To jest wlasciwa miara przy ocenie rozmow, bo tam
placimy za przeczytanie stu piecdziesieciu zgloszen. Przy jurorze,
ktorego udzial sam jest wartoscia dla konkursu, iloczyn godzin i stawki
nie mierzy tego, co kupujemy, a 2 900 zl za przewodniczenie jury brzmi
gorzej niz brak propozycji. Warunki ustali rozmowa z przewodniczacym.

Kotwica zostaje widoczna w Wyjasnieniach i w uwagach do pozycji: 5 osob
po 10 godzin po 290 zl dalaby 14 500 zl.

Budzet plakatu spada z 171 736 na 155 496 zl netto, rezerwa z 8 436 na
6 696. Suma pozycji, o ktore pytamy MKiDN, z 428 352 na 412 112 zl, a
liczba pozycji czekajacych na wycene w tej grupie z trzech na cztery.
Razem wszystkie budzety: 1 321 218,80 zl.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Liczba jurorów plakatu</t>
   </si>
   <si>
-    <t xml:space="preserve">Składu jeszcze nie ma. Przy trzech pozycja spada do 8,7 tys., przy siedmiu rośnie do 20,3 tys.</t>
+    <t xml:space="preserve">Kotwica, nie decyzja: pozycja honorariów w Budżecie Plakatu stoi na zerze jako DO USTALENIA, do rozmowy z przewodniczącym jury.</t>
   </si>
   <si>
     <t xml:space="preserve">Godzin oceny na jurora</t>
@@ -786,7 +786,7 @@
     <t xml:space="preserve">Honoraria jury plakatu za ocenę (netto)</t>
   </si>
   <si>
-    <t xml:space="preserve">stawka Kapituły, 10 h na jurora, skład pięcioosobowy</t>
+    <t xml:space="preserve">DO USTALENIA - stawka godzinowa jest przy nazwisku złym narzędziem; kotwica z Wyjaśnień (5 osób x 10 h x 290 zł) dałaby 14 500 zł</t>
   </si>
   <si>
     <t xml:space="preserve">Transport oryginałów w obie strony (netto)</t>
@@ -1619,7 +1619,7 @@
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'Budżet Plakatu'!$D$34</f>
-        <v>171736</v>
+        <v>155496</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C11" s="11" t="n">
         <f aca="false">'Budżet Nagrody'!$D$39+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$32+'Budżet Plakatu'!$D$34+'Budżet Akademii'!$D$27</f>
-        <v>1337458.8</v>
+        <v>1321218.8</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -5001,17 +5001,15 @@
       <c r="A21" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="B21" s="8" t="n">
-        <f aca="false">Wyjaśnienia!$B$55*Wyjaśnienia!$B$54</f>
-        <v>2900</v>
+      <c r="B21" s="16" t="n">
+        <v>0</v>
       </c>
       <c r="C21" s="30" t="n">
-        <f aca="false">Wyjaśnienia!$B$53</f>
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D21" s="8" t="n">
         <f aca="false">B21*C21</f>
-        <v>14500</v>
+        <v>0</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>253</v>
@@ -5116,7 +5114,7 @@
       </c>
       <c r="D27" s="11" t="n">
         <f aca="false">SUM(D18:D26)</f>
-        <v>121500</v>
+        <v>107000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5153,7 +5151,7 @@
       </c>
       <c r="D32" s="8" t="n">
         <f aca="false">D27-D30</f>
-        <v>28500</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5162,7 +5160,7 @@
       </c>
       <c r="D33" s="8" t="n">
         <f aca="false">(D31+D32)*Wyjaśnienia!$B$59</f>
-        <v>8436</v>
+        <v>6696</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5171,7 +5169,7 @@
       </c>
       <c r="D34" s="11" t="n">
         <f aca="false">SUM(D30:D33)</f>
-        <v>171736</v>
+        <v>155496</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5180,7 +5178,7 @@
       </c>
       <c r="D35" s="8" t="n">
         <f aca="false">D34*Wyjaśnienia!$B$29</f>
-        <v>39499.28</v>
+        <v>35764.08</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5189,7 +5187,7 @@
       </c>
       <c r="D36" s="11" t="n">
         <f aca="false">D34+D35</f>
-        <v>211235.28</v>
+        <v>191260.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Plebiscyt filmu: dziesięciu finalistów i siedem wyróżnień
- regulamin filmu: jury wybiera dziesięciu finalistów; akademia przekazuje
  jury nie więcej niż dwadzieścia filmów; siedem wyróżnień bez nagrody
  pieniężnej (dyplom i miejsce w zestawie do pokazów); minutowy fragment
  na gali dla pięciu najwyżej ocenionych; dyplomy dla całej dziesiątki
- strona plebiscytu filmu w ślad za regulaminem
- budżet: dyplomy dla dziesiątki, kotwica honorarium jury 5 x 40 h x 290 zł
  (30 h oglądania dwudziestu filmów), noty przy nagrodach i dojazdach
- nota do MKiDN: rozdział o filmie, limit pracy jury, tabela kosztorysu
- wszędzie "medal" zamiast "medalion"

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -332,7 +332,7 @@
     <t xml:space="preserve">Nagrody filmu łącznie (brutto)</t>
   </si>
   <si>
-    <t xml:space="preserve">100 tys. + 50 tys. + 30 tys. dla czołowej trójki.</t>
+    <t xml:space="preserve">100 tys. + 50 tys. + 30 tys. dla czołowej trójki. Siedem wyróżnień nie jest pieniężnych.</t>
   </si>
   <si>
     <t xml:space="preserve">Nagroda publiczności filmu (brutto)</t>
@@ -344,13 +344,13 @@
     <t xml:space="preserve">Medal zwycięzcy i dyplomy filmu (netto)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ten sam mosiężny medal co w pozostałych plebiscytach; dyplomy dla pięciu finalistów.</t>
+    <t xml:space="preserve">Ten sam medal co w pozostałych plebiscytach; dyplomy dla dziesięciu finalistów.</t>
   </si>
   <si>
     <t xml:space="preserve">Liczba filmów finałowych</t>
   </si>
   <si>
-    <t xml:space="preserve">Pięciu finalistów, bo tyle minutowych emisji mieści się na gali.</t>
+    <t xml:space="preserve">Dziesięciu finalistów: trójka z nagrodami pieniężnymi i siedem wyróżnień. Minutowe skróty na gali dostaje pięć najwyżej ocenionych.</t>
   </si>
   <si>
     <t xml:space="preserve">Liczba jurorów filmu</t>
@@ -362,7 +362,7 @@
     <t xml:space="preserve">Godzin oceny na jurora filmu</t>
   </si>
   <si>
-    <t xml:space="preserve">Jury ogląda listę węższą po Akademii, ale filmy trwają do 90 minut - stąd więcej godzin niż przy plakacie.</t>
+    <t xml:space="preserve">Akademia przekazuje jury nie więcej niż dwadzieścia filmów (§ 8 ust. 5a); dwadzieścia filmów po najwyżej 90 minut to 30 godzin samego oglądania, reszta na karty oceny, obrady i werdykt.</t>
   </si>
   <si>
     <t xml:space="preserve">Stawka jury filmu za godzinę (netto)</t>
@@ -749,10 +749,10 @@
     <t xml:space="preserve">nagranie i premiera na początku 2027, otwiera nabór</t>
   </si>
   <si>
-    <t xml:space="preserve">Medalion zwycięzcy i dyplomy finalistów (netto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ten sam medalion, który otrzymuje laureat konkursu rozmów; dyplomy dla całej dziesiątki</t>
+    <t xml:space="preserve">Medal zwycięzcy i dyplomy finalistów (netto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ten sam medal, który otrzymuje laureat plebiscytu rozmów; dyplomy dla całej dziesiątki</t>
   </si>
   <si>
     <t xml:space="preserve">Honoraria jury plebiscytu za ocenę (netto)</t>
@@ -1040,7 +1040,7 @@
     <t xml:space="preserve">dwa przejścia oceny, pięciu finalistów, kolejność trójki</t>
   </si>
   <si>
-    <t xml:space="preserve">Zebranie fragmentów od finalistów i przygotowanie emisji galowych</t>
+    <t xml:space="preserve">Zebranie fragmentów od piątki i przygotowanie skrótów galowych</t>
   </si>
   <si>
     <t xml:space="preserve">autor wybiera fragment w terminie nie krótszym niż 14 dni; organizator zbiera, sprawdza format i układa kolejność</t>
@@ -1070,19 +1070,19 @@
     <t xml:space="preserve">Nagrody filmu (brutto dla laureatów)</t>
   </si>
   <si>
-    <t xml:space="preserve">czołowa trójka: 100, 50 i 30 tys.; podatek 10% jak przy Nagrodzie</t>
+    <t xml:space="preserve">czołowa trójka: 100, 50 i 30 tys.; siedem wyróżnień bez nagrody pieniężnej; podatek 10% jak przy Nagrodzie</t>
   </si>
   <si>
     <t xml:space="preserve">jedna nagroda, dla filmu z największą liczbą głosów</t>
   </si>
   <si>
-    <t xml:space="preserve">ten sam medalion, który otrzymują zwycięzcy pozostałych plebiscytów; dyplomy dla pięciu finalistów</t>
+    <t xml:space="preserve">ten sam medal, który otrzymują zwycięzcy pozostałych plebiscytów; dyplomy dla dziesięciu finalistów</t>
   </si>
   <si>
     <t xml:space="preserve">Honoraria jury filmu za ocenę (netto)</t>
   </si>
   <si>
-    <t xml:space="preserve">DO USTALENIA - stawka godzinowa jest przy nazwisku złym narzędziem; kotwica z Wyjaśnień (5 osób x 25 h x 290 zł) dałaby 36 250 zł</t>
+    <t xml:space="preserve">DO USTALENIA - kotwica z Wyjaśnień (5 osób x 40 h x 290 zł) dałaby 58 000 zł; 40 h to 30 h oglądania dwudziestu filmów przekazanych jury plus karty, obrady i werdykt</t>
   </si>
   <si>
     <t xml:space="preserve">Opracowanie techniczne minutowych emisji na galę (netto)</t>
@@ -1097,7 +1097,7 @@
     <t xml:space="preserve">DO WYCENY - sala, projekcja, obsługa; regulamin § 10 ust. 4 wymaga ogłoszenia terminu najpóźniej w dniu gali</t>
   </si>
   <si>
-    <t xml:space="preserve">DO WYCENY - jak przy plebiscycie piosenki; pięciu finalistów, często ze składem</t>
+    <t xml:space="preserve">DO WYCENY - jak przy plebiscycie piosenki; dziesięciu finalistów, często z ekipą</t>
   </si>
   <si>
     <t xml:space="preserve">Obsługa prawna regulaminu filmu (netto)</t>
@@ -2561,7 +2561,7 @@
         <v>106</v>
       </c>
       <c r="B70" s="14" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>107</v>
@@ -2583,7 +2583,7 @@
         <v>110</v>
       </c>
       <c r="B72" s="14" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>111</v>

</xml_diff>

<commit_message>
Budżet Gali: pozycja na tantiemy dla OZZ
Publiczne wykonanie muzyki na gali - hymn i trzy piosenki na żywo oraz
muzyka w zwiastunach piątki filmów - wymaga rozliczenia niezależnie od
uprawnień uczestników, a obowiązek ten regulamin filmu zostawia przy
Organizatorze. Pozycja stoi bez kwoty, do ustalenia repertuaru.

Suma Budżetu Gali bez zmian: 35 168 zł netto, 43 256,64 zł brutto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="380">
   <si>
     <t xml:space="preserve">Budżet pierwszej edycji Nagrody Konstela</t>
   </si>
@@ -1158,6 +1158,12 @@
   </si>
   <si>
     <t xml:space="preserve">do wyceny</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tantiemy dla organizacji zbiorowego zarządzania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO WYCENY - publiczne wykonanie muzyki na gali: hymn i trzy piosenki na żywo oraz muzyka w zwiastunach piątki filmów; obowiązek po stronie Organizatora, nieprzenoszony na uczestników (§ 12 ust. 2a regulaminu filmu)</t>
   </si>
   <si>
     <t xml:space="preserve">Rezerwa (od pracy i kosztów)</t>
@@ -1912,7 +1918,7 @@
         <v>19</v>
       </c>
       <c r="C12" s="9" t="n">
-        <f aca="false">'Budżet Gali'!$D$25</f>
+        <f aca="false">'Budżet Gali'!$D$26</f>
         <v>35168</v>
       </c>
     </row>
@@ -1921,7 +1927,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="11" t="n">
-        <f aca="false">'Budżet Nagrody'!$D$35+'Budżet Gali'!$D$25+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$32+'Budżet Plakatu'!$D$34+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$34</f>
+        <f aca="false">'Budżet Nagrody'!$D$35+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$32+'Budżet Plakatu'!$D$34+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$34</f>
         <v>1686506.8</v>
       </c>
       <c r="D13" s="3"/>
@@ -7056,72 +7062,75 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="21" t="s">
+        <v>377</v>
+      </c>
+      <c r="B19" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="24" t="n">
+        <f aca="false">B19*C19</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="9" t="n">
-        <f aca="false">SUM(D12:D18)</f>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="9" t="n">
+        <f aca="false">SUM(D12:D19)</f>
         <v>21500</v>
       </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
+      <c r="A21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D23" s="8" t="n">
         <f aca="false">E8</f>
         <v>9900</v>
       </c>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
-        <v>172</v>
-      </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="8" t="n">
-        <f aca="false">D19</f>
-        <v>21500</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>377</v>
+        <v>172</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="8" t="n">
-        <f aca="false">(D22+D23)*Wyjaśnienia!$B$30</f>
-        <v>3768</v>
+        <f aca="false">D20</f>
+        <v>21500</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -7129,14 +7138,14 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="s">
-        <v>174</v>
+      <c r="A25" s="21" t="s">
+        <v>379</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
-      <c r="D25" s="9" t="n">
-        <f aca="false">SUM(D22:D24)</f>
-        <v>35168</v>
+      <c r="D25" s="8" t="n">
+        <f aca="false">(D23+D24)*Wyjaśnienia!$B$30</f>
+        <v>3768</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -7144,14 +7153,14 @@
       <c r="H25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="s">
-        <v>175</v>
+      <c r="A26" s="6" t="s">
+        <v>174</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
-      <c r="D26" s="8" t="n">
-        <f aca="false">D25*Wyjaśnienia!$B$33</f>
-        <v>8088.64</v>
+      <c r="D26" s="9" t="n">
+        <f aca="false">SUM(D23:D25)</f>
+        <v>35168</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -7159,21 +7168,35 @@
       <c r="H26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="s">
-        <v>176</v>
+      <c r="A27" s="21" t="s">
+        <v>175</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
-      <c r="D27" s="27" t="n">
-        <f aca="false">D25+D26</f>
-        <v>43256.64</v>
+      <c r="D27" s="8" t="n">
+        <f aca="false">D26*Wyjaśnienia!$B$33</f>
+        <v>8088.64</v>
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="27" t="n">
+        <f aca="false">D26+D27</f>
+        <v>43256.64</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+    </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -7258,7 +7281,7 @@
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A22:F22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Dystrybucja kinowa: dystrybutor zamiast partnera z salą, wpływy przy autorze
- regulamin filmu § 9 ust. 1 lit. a2, § 10 ust. 4 i § 12 ust. 2 lit. d
  mówią o dystrybutorze i o pokazach kinowych
- nowy § 10 ust. 4a: zestaw składa Organizator, umowę z dystrybutorem
  zawiera Uczestnik, wpływy z biletów i dalszej eksploatacji są jego,
  Organizator nie bierze udziału ani prowizji, może natomiast uzgodnić
  z dystrybutorem pokrycie kosztów przygotowania zestawu - ta sama
  konstrukcja co przy płycie w plebiscycie piosenki
- strona plebiscytu: dwa akapity o pieniądzach z biletów
- pytania do kancelarii: nowy pkt 4b, pięć pytań
- budżet filmu i nota do MKiDN w ślad za tym

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -1046,7 +1046,7 @@
     <t xml:space="preserve">autor wybiera fragment w terminie nie krótszym niż 14 dni; organizator zbiera, sprawdza format i układa kolejność</t>
   </si>
   <si>
-    <t xml:space="preserve">Organizacja pełnych pokazów filmów finałowych poza galą</t>
+    <t xml:space="preserve">Złożenie zestawu dziesiątki i rozmowy z dystrybutorami</t>
   </si>
   <si>
     <t xml:space="preserve">regulamin § 10 ust. 4: termin i miejsce ogłaszane najpóźniej w dniu gali, udział za zgodą autora</t>
@@ -1091,10 +1091,10 @@
     <t xml:space="preserve">DO WYCENY - pobranie pięciu zwiastunów w jakości emisyjnej, zgodność formatów, normalizacja dźwięku, plansze z tytułami; zwiastun dostarcza autor, Organizator nie montuje fragmentów filmów</t>
   </si>
   <si>
-    <t xml:space="preserve">Pełne pokazy filmów finałowych (netto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO WYCENY - sala, projekcja, obsługa; regulamin § 10 ust. 4 wymaga ogłoszenia terminu najpóźniej w dniu gali</t>
+    <t xml:space="preserve">Pokazy kinowe filmów finałowych (netto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO WYCENY - opracowanie techniczne kopii, napisy i materiały informacyjne dla zestawu dziesiątki; zależy od pozyskania dystrybutora (§ 10 ust. 4), z którym Organizator może uzgodnić pokrycie tych kosztów</t>
   </si>
   <si>
     <t xml:space="preserve">DO WYCENY - jak przy plebiscycie piosenki; dziesięciu finalistów, często z ekipą</t>

</xml_diff>

<commit_message>
Nagroda za uzasadnienie wyboru we wszystkich czterech plebiscytach
- oddanie głosu w nagrodzie publiczności wymaga uzasadnienia od 700 do
  1500 znaków; bez niego głos nie zostaje oddany
- uzasadnienia ocenia trzyosobowy zespół powołany spoza jury, ogłaszany
  przed rozpoczęciem głosowania; bez losowania
- cztery regulaminy, osobna sekcja na czterech stronach, polityka
  prywatności
- kafel Nagrody Publiczności ujednolicony na czterech stronach
- piosenka: kafel drugiego i trzeciego miejsca bez zdania o dyplomach,
  dyplom przy kaflu nagrania studyjnego
- budżet: nagroda 1 000 zł dodana w rozmowie, filmie i plakacie, czyli
  +3 000 zł; Budżet Nagrody 535 996,80, Plakatu 154 480, Filmu 256 800,
  wszystkie budżety 1 689 626,80 zł; nota do MKiDN w ślad za tym

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="380">
   <si>
     <t xml:space="preserve">Budżet pierwszej edycji Nagrody Konstela</t>
   </si>
@@ -155,7 +155,7 @@
     <t xml:space="preserve">Nagrody publiczności łącznie (brutto)</t>
   </si>
   <si>
-    <t xml:space="preserve">3 tys. dla wykonawcy, 1 tys. za uzasadnienie. Do potwierdzenia.</t>
+    <t xml:space="preserve">3 000 zł dla wykonawcy oraz 1 000 zł za najlepsze uzasadnienie wyboru. Uzasadnienie jest obowiązkowe przy każdym głosie (§ 11 ust. 2 regulaminu).</t>
   </si>
   <si>
     <t xml:space="preserve">Nagranie studyjne - koszt za utwór (netto)</t>
@@ -272,10 +272,10 @@
     <t xml:space="preserve">50 tys. + 25 tys. + 15 tys. dla czołowej trójki.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nagroda publiczności plakatu (brutto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jedna nagroda, bez nagrody za uzasadnienie.</t>
+    <t xml:space="preserve">Nagrody publiczności plakatu łącznie (brutto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 000 zł dla pracy z największą liczbą głosów oraz 1 000 zł za najlepsze uzasadnienie wyboru (§ 12 ust. 6).</t>
   </si>
   <si>
     <t xml:space="preserve">Medal zwycięzcy i dyplomy plakatu (netto)</t>
@@ -335,10 +335,10 @@
     <t xml:space="preserve">100 tys. + 50 tys. + 30 tys. dla czołowej trójki. Siedem wyróżnień nie jest pieniężnych.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nagroda publiczności filmu (brutto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jedna nagroda, dla filmu z największą liczbą głosów.</t>
+    <t xml:space="preserve">Nagrody publiczności filmu łącznie (brutto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 000 zł dla filmu z największą liczbą głosów oraz 1 000 zł za najlepsze uzasadnienie wyboru (§ 11a ust. 5).</t>
   </si>
   <si>
     <t xml:space="preserve">Medal zwycięzcy i dyplomy filmu (netto)</t>
@@ -524,7 +524,10 @@
     <t xml:space="preserve">materiały, obsługa prasowa przy starcie i rozstrzygnięciu, płatne dotarcie</t>
   </si>
   <si>
-    <t xml:space="preserve">Nagroda publiczności</t>
+    <t xml:space="preserve">Nagrody publiczności (brutto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 000 zł dla zgłoszenia z największą liczbą głosów oraz 1 000 zł za najlepsze uzasadnienie wyboru (§ 11 ust. 8a)</t>
   </si>
   <si>
     <t xml:space="preserve">Ubezpieczenie OC organizatora</t>
@@ -732,9 +735,6 @@
   </si>
   <si>
     <t xml:space="preserve">czołowa trójka; podatek 10% jak przy Nagrodzie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nagrody publiczności (brutto)</t>
   </si>
   <si>
     <t xml:space="preserve">dla wykonawcy oraz za najlepsze uzasadnienie wyboru</t>
@@ -1827,7 +1827,7 @@
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">'Budżet Nagrody'!$D$35</f>
-        <v>534876.8</v>
+        <v>535996.8</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'Budżet Plakatu'!$D$34</f>
-        <v>153480</v>
+        <v>154480</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'Budżet Filmu'!$D$34</f>
-        <v>255800</v>
+        <v>256800</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="C13" s="11" t="n">
         <f aca="false">'Budżet Nagrody'!$D$35+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$32+'Budżet Plakatu'!$D$34+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$34</f>
-        <v>1686506.8</v>
+        <v>1689626.8</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -2418,7 +2418,7 @@
         <v>81</v>
       </c>
       <c r="B55" s="18" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>82</v>
@@ -2545,7 +2545,7 @@
         <v>102</v>
       </c>
       <c r="B68" s="14" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>103</v>
@@ -3201,21 +3201,23 @@
         <v>165</v>
       </c>
       <c r="B26" s="26" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="C26" s="22" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="24" t="n">
         <f aca="false">B26*C26</f>
-        <v>3000</v>
-      </c>
-      <c r="E26" s="15"/>
+        <v>4000</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>166</v>
+      </c>
       <c r="F26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B27" s="26" t="n">
         <v>0</v>
@@ -3228,7 +3230,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -3236,13 +3238,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="9" t="n">
         <f aca="false">SUM(D21:D27)</f>
-        <v>52950</v>
+        <v>53950</v>
       </c>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
@@ -3256,7 +3258,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
@@ -3268,7 +3270,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -3283,7 +3285,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -3298,13 +3300,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="8" t="n">
         <f aca="false">D28</f>
-        <v>52950</v>
+        <v>53950</v>
       </c>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
@@ -3313,24 +3315,24 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D34" s="3" t="n">
         <f aca="false">(D32+D33)*Wyjaśnienia!$B$30</f>
-        <v>14986.8</v>
+        <v>15106.8</v>
       </c>
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="9" t="n">
         <f aca="false">SUM(D31:D34)</f>
-        <v>534876.8</v>
+        <v>535996.8</v>
       </c>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
@@ -3339,13 +3341,13 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="8" t="n">
         <f aca="false">D35*Wyjaśnienia!$B$33</f>
-        <v>123021.664</v>
+        <v>123279.264</v>
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -3354,13 +3356,13 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="27" t="n">
         <f aca="false">D35+D36</f>
-        <v>657898.464</v>
+        <v>659276.064</v>
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -3484,7 +3486,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -3552,7 +3554,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>45</v>
@@ -3569,14 +3571,14 @@
         <v>9900</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B8" s="22" t="n">
         <v>40</v>
@@ -3593,14 +3595,14 @@
         <v>8800</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B9" s="22" t="n">
         <v>0</v>
@@ -3617,14 +3619,14 @@
         <v>2200</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B10" s="22" t="n">
         <v>50</v>
@@ -3641,14 +3643,14 @@
         <v>11000</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>25</v>
@@ -3665,14 +3667,14 @@
         <v>5500</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B12" s="22" t="n">
         <v>160</v>
@@ -3689,14 +3691,14 @@
         <v>35200</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B13" s="22" t="n">
         <v>50</v>
@@ -3713,14 +3715,14 @@
         <v>11000</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B14" s="22" t="n">
         <v>72</v>
@@ -3800,7 +3802,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B19" s="26" t="n">
         <v>3000</v>
@@ -3813,7 +3815,7 @@
         <v>3000</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -3821,7 +3823,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B20" s="26" t="n">
         <v>6000</v>
@@ -3834,17 +3836,17 @@
         <v>6000</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B21" s="26" t="n">
         <v>10000</v>
@@ -3857,7 +3859,7 @@
         <v>10000</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -3865,7 +3867,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="21" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B22" s="26" t="n">
         <v>40000</v>
@@ -3878,7 +3880,7 @@
         <v>40000</v>
       </c>
       <c r="E22" s="15" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -3886,7 +3888,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B23" s="26" t="n">
         <v>4000</v>
@@ -3899,7 +3901,7 @@
         <v>4000</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -3907,7 +3909,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B24" s="26" t="n">
         <v>3000</v>
@@ -3920,7 +3922,7 @@
         <v>3000</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -3928,7 +3930,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B25" s="26" t="n">
         <v>4000</v>
@@ -3941,7 +3943,7 @@
         <v>4000</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -3949,7 +3951,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B26" s="26" t="n">
         <v>0</v>
@@ -3962,7 +3964,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -3970,7 +3972,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B27" s="26" t="n">
         <v>15000</v>
@@ -3983,7 +3985,7 @@
         <v>15000</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -3991,7 +3993,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B28" s="26" t="n">
         <v>6000</v>
@@ -4004,7 +4006,7 @@
         <v>6000</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -4012,7 +4014,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B29" s="26" t="n">
         <v>30000</v>
@@ -4025,7 +4027,7 @@
         <v>30000</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -4033,7 +4035,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="28" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B30" s="18" t="n">
         <v>4500</v>
@@ -4046,12 +4048,12 @@
         <v>4500</v>
       </c>
       <c r="F30" s="28" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B31" s="18" t="n">
         <v>0</v>
@@ -4064,13 +4066,13 @@
         <v>0</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F31" s="28"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -4095,7 +4097,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -4107,7 +4109,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -4122,7 +4124,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -4137,7 +4139,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -4152,7 +4154,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -4167,7 +4169,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -4182,7 +4184,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -4310,7 +4312,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -4378,7 +4380,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>0</v>
@@ -4395,14 +4397,14 @@
         <v>5500</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B8" s="22" t="n">
         <v>40</v>
@@ -4417,14 +4419,14 @@
         <v>8800</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B9" s="22" t="n">
         <v>30</v>
@@ -4439,14 +4441,14 @@
         <v>6600</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B10" s="22" t="n">
         <v>20</v>
@@ -4461,14 +4463,14 @@
         <v>4400</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>50</v>
@@ -4483,7 +4485,7 @@
         <v>11000</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -4503,7 +4505,7 @@
         <v>36300</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
@@ -4552,7 +4554,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B16" s="24" t="n">
         <f aca="false">Wyjaśnienia!$B$24</f>
@@ -4566,7 +4568,7 @@
         <v>35000</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -4574,7 +4576,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>235</v>
+        <v>165</v>
       </c>
       <c r="B17" s="24" t="n">
         <f aca="false">Wyjaśnienia!$B$25</f>
@@ -4745,7 +4747,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -4770,7 +4772,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
@@ -4782,7 +4784,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -4797,7 +4799,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -4827,7 +4829,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -4842,7 +4844,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -4857,7 +4859,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -4872,7 +4874,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -5096,7 +5098,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>20</v>
@@ -5207,7 +5209,7 @@
         <v>41800</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5262,14 +5264,14 @@
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">Wyjaśnienia!$B$55</f>
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="C19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="8" t="n">
         <f aca="false">B19*C19</f>
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>269</v>
@@ -5407,16 +5409,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D27" s="11" t="n">
         <f aca="false">SUM(D18:D26)</f>
-        <v>105200</v>
+        <v>106200</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
@@ -5426,16 +5428,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">Wyjaśnienia!$B$54+Wyjaśnienia!$B$55</f>
-        <v>93000</v>
+        <v>94000</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D31" s="8" t="n">
         <f aca="false">E14</f>
@@ -5453,7 +5455,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D33" s="8" t="n">
         <f aca="false">(D31+D32)*Wyjaśnienia!$B$63</f>
@@ -5462,29 +5464,29 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D34" s="11" t="n">
         <f aca="false">SUM(D30:D33)</f>
-        <v>153480</v>
+        <v>154480</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D35" s="8" t="n">
         <f aca="false">D34*Wyjaśnienia!$B$33</f>
-        <v>35300.4</v>
+        <v>35530.4</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D36" s="11" t="n">
         <f aca="false">D34+D35</f>
-        <v>188780.4</v>
+        <v>190010.4</v>
       </c>
     </row>
   </sheetData>
@@ -5842,7 +5844,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="37" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D27" s="42" t="n">
         <f aca="false">SUM(D23:D26)</f>
@@ -5851,7 +5853,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B29" s="36"/>
       <c r="C29" s="36"/>
@@ -5870,7 +5872,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="28" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D31" s="41" t="n">
         <f aca="false">D27</f>
@@ -5888,7 +5890,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="37" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D33" s="42" t="n">
         <f aca="false">SUM(D30:D32)</f>
@@ -5897,7 +5899,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="28" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D34" s="41" t="n">
         <f aca="false">D33*Wyjaśnienia!$B$33</f>
@@ -5906,7 +5908,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="37" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D35" s="42" t="n">
         <f aca="false">D33+D34</f>
@@ -6350,7 +6352,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B10" s="20" t="n">
         <v>20</v>
@@ -6518,14 +6520,14 @@
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">Wyjaśnienia!$B$68</f>
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="C20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
         <f aca="false">B20*C20</f>
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>348</v>
@@ -6642,18 +6644,18 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="32"/>
       <c r="D27" s="11" t="n">
         <f aca="false">SUM(D19:D26)</f>
-        <v>184200</v>
+        <v>185200</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
@@ -6663,16 +6665,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">Wyjaśnienia!$B$67+Wyjaśnienia!$B$68</f>
-        <v>183000</v>
+        <v>184000</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D31" s="8" t="n">
         <f aca="false">E15</f>
@@ -6690,7 +6692,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D33" s="8" t="n">
         <f aca="false">(D31+D32)*Wyjaśnienia!$B$74</f>
@@ -6699,29 +6701,29 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D34" s="11" t="n">
         <f aca="false">SUM(D30:D33)</f>
-        <v>255800</v>
+        <v>256800</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D35" s="8" t="n">
         <f aca="false">D34*Wyjaśnienia!$B$33</f>
-        <v>58834</v>
+        <v>59064</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D36" s="11" t="n">
         <f aca="false">D34+D35</f>
-        <v>314634</v>
+        <v>315864</v>
       </c>
     </row>
   </sheetData>
@@ -7081,7 +7083,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -7101,7 +7103,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -7113,7 +7115,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D23" s="8" t="n">
         <f aca="false">E8</f>
@@ -7124,7 +7126,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -7154,7 +7156,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -7169,7 +7171,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -7184,7 +7186,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>

</xml_diff>

<commit_message>
Jedna nazwa nagrody za uzasadnienia w regulaminach, budżecie i nocie
"Nagroda dla publicznych ocen zgłoszonych rozmów, filmów, piosenek,
plakatów" zamiast "nagroda za najlepsze uzasadnienie wyboru".
Zdanie o progu na stronach bez porównania o piwnicy, z zakresem
opisanym słownie: od dwóch zdań do krótkiego akapitu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -155,7 +155,7 @@
     <t xml:space="preserve">Nagrody publiczności łącznie (brutto)</t>
   </si>
   <si>
-    <t xml:space="preserve">3 000 zł dla wykonawcy oraz 1 000 zł za najlepsze uzasadnienie wyboru. Uzasadnienie jest obowiązkowe przy każdym głosie (§ 11 ust. 2 regulaminu).</t>
+    <t xml:space="preserve">3 000 zł dla wykonawcy oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych piosenek. Uzasadnienie jest obowiązkowe przy każdym głosie, od 200 do 1500 znaków (§ 11 ust. 2 regulaminu).</t>
   </si>
   <si>
     <t xml:space="preserve">Nagranie studyjne - koszt za utwór (netto)</t>
@@ -275,7 +275,7 @@
     <t xml:space="preserve">Nagrody publiczności plakatu łącznie (brutto)</t>
   </si>
   <si>
-    <t xml:space="preserve">3 000 zł dla pracy z największą liczbą głosów oraz 1 000 zł za najlepsze uzasadnienie wyboru (§ 12 ust. 6).</t>
+    <t xml:space="preserve">3 000 zł dla pracy z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych plakatów (§ 12 ust. 6).</t>
   </si>
   <si>
     <t xml:space="preserve">Medal zwycięzcy i dyplomy plakatu (netto)</t>
@@ -338,7 +338,7 @@
     <t xml:space="preserve">Nagrody publiczności filmu łącznie (brutto)</t>
   </si>
   <si>
-    <t xml:space="preserve">3 000 zł dla filmu z największą liczbą głosów oraz 1 000 zł za najlepsze uzasadnienie wyboru (§ 11a ust. 5).</t>
+    <t xml:space="preserve">3 000 zł dla filmu z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych filmów (§ 11a ust. 5).</t>
   </si>
   <si>
     <t xml:space="preserve">Medal zwycięzcy i dyplomy filmu (netto)</t>
@@ -527,7 +527,7 @@
     <t xml:space="preserve">Nagrody publiczności (brutto)</t>
   </si>
   <si>
-    <t xml:space="preserve">3 000 zł dla zgłoszenia z największą liczbą głosów oraz 1 000 zł za najlepsze uzasadnienie wyboru (§ 11 ust. 8a)</t>
+    <t xml:space="preserve">3 000 zł dla zgłoszenia z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych rozmów (§ 11 ust. 8a)</t>
   </si>
   <si>
     <t xml:space="preserve">Ubezpieczenie OC organizatora</t>

</xml_diff>

<commit_message>
Potwierdzenia wspoluprawnionych, pole na tekst piosenki, polisa w budzecie plakatu
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="382">
   <si>
     <t xml:space="preserve">Budżet pierwszej edycji Nagrody Konstela</t>
   </si>
@@ -215,7 +215,7 @@
     <t xml:space="preserve">Realizacja części artystycznej gali</t>
   </si>
   <si>
-    <t xml:space="preserve">Po wpisaniu tych kwot rosną Budżet Plebiscytu, Budżet Plakatu i Budżet Filmu. W Budżecie Plakatu czekają na wycenę trzy pozycje, w Budżecie Filmu pięć - wszystkie opisane w kolumnie Uwagi.</t>
+    <t xml:space="preserve">Po wpisaniu tych kwot rosną Budżet Plebiscytu, Budżet Plakatu i Budżet Filmu. W Budżecie Plakatu czekają na wycenę cztery pozycje, w Budżecie Filmu pięć - wszystkie opisane w kolumnie Uwagi.</t>
   </si>
   <si>
     <t xml:space="preserve">JAK CZYTAĆ BUDŻETY</t>
@@ -870,6 +870,12 @@
   </si>
   <si>
     <t xml:space="preserve">DO WYCENY - jak przy plebiscycie piosenki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polisa: wycena prac, rozszerzenie na przechowywanie i okres po sprzedaży (netto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO WYCENY - polisa ma objąć cały uzgodniony okres: transport w obie strony, przechowywanie u organizatora, obie wystawy oraz czas po sprzedaży do wydania pracy nabywcy; do ustalenia suma ubezpieczenia na pracę, udział własny i procedura zgłoszenia szkody</t>
   </si>
   <si>
     <t xml:space="preserve">Finansuje: Sponsor Akademii. Kwoty netto. Vouchery są świadczeniem rzeczowym i rosną wprost z liczbą ocenionych rozmów.</t>
@@ -1889,7 +1895,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="9" t="n">
-        <f aca="false">'Budżet Plakatu'!$D$34</f>
+        <f aca="false">'Budżet Plakatu'!$D$35</f>
         <v>154480</v>
       </c>
       <c r="D10" s="3"/>
@@ -1927,7 +1933,7 @@
         <v>20</v>
       </c>
       <c r="C13" s="11" t="n">
-        <f aca="false">'Budżet Nagrody'!$D$35+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$32+'Budżet Plakatu'!$D$34+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$34</f>
+        <f aca="false">'Budżet Nagrody'!$D$35+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$32+'Budżet Plakatu'!$D$35+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$34</f>
         <v>1689626.8</v>
       </c>
       <c r="D13" s="3"/>
@@ -4983,7 +4989,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="54"/>
@@ -5408,84 +5414,105 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="8" t="n">
+        <f aca="false">B27*C27</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="D27" s="11" t="n">
-        <f aca="false">SUM(D18:D26)</f>
+      <c r="D28" s="11" t="n">
+        <f aca="false">SUM(D18:D27)</f>
         <v>106200</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="31" t="s">
+      <c r="A29" s="30"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
-      <c r="D29" s="31"/>
-      <c r="E29" s="31"/>
-      <c r="F29" s="31"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D30" s="8" t="n">
+      <c r="D31" s="8" t="n">
         <f aca="false">Wyjaśnienia!$B$54+Wyjaśnienia!$B$55</f>
         <v>94000</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="D31" s="8" t="n">
+      <c r="D32" s="8" t="n">
         <f aca="false">E14</f>
         <v>41800</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <f aca="false">D27-D30</f>
-        <v>12200</v>
-      </c>
-    </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="D33" s="8" t="n">
+        <f aca="false">D28-D31</f>
+        <v>12200</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="D33" s="8" t="n">
-        <f aca="false">(D31+D32)*Wyjaśnienia!$B$63</f>
+      <c r="D34" s="8" t="n">
+        <f aca="false">(D32+D33)*Wyjaśnienia!$B$63</f>
         <v>6480</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="s">
         <v>175</v>
       </c>
-      <c r="D34" s="11" t="n">
-        <f aca="false">SUM(D30:D33)</f>
+      <c r="D35" s="11" t="n">
+        <f aca="false">SUM(D31:D34)</f>
         <v>154480</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D35" s="8" t="n">
-        <f aca="false">D34*Wyjaśnienia!$B$33</f>
+      <c r="D36" s="8" t="n">
+        <f aca="false">D35*Wyjaśnienia!$B$33</f>
         <v>35530.4</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="D36" s="11" t="n">
-        <f aca="false">D34+D35</f>
+      <c r="D37" s="11" t="n">
+        <f aca="false">D35+D36</f>
         <v>190010.4</v>
       </c>
     </row>
@@ -5536,7 +5563,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="35" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B2" s="35"/>
       <c r="C2" s="35"/>
@@ -5546,7 +5573,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="35" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -5556,7 +5583,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="36" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B5" s="36"/>
       <c r="C5" s="36"/>
@@ -5569,7 +5596,7 @@
         <v>124</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F6" s="37" t="s">
         <v>129</v>
@@ -5577,79 +5604,79 @@
     </row>
     <row r="7" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B7" s="39" t="n">
         <f aca="false">Wyjaśnienia!$B$17</f>
         <v>150</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B8" s="39" t="n">
         <f aca="false">Wyjaśnienia!$B$46</f>
         <v>2</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="37" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B9" s="40" t="n">
         <f aca="false">B7*B8</f>
         <v>300</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B10" s="39" t="n">
         <f aca="false">Wyjaśnienia!$B$66</f>
         <v>150</v>
       </c>
       <c r="F10" s="28" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B11" s="39" t="n">
         <f aca="false">Wyjaśnienia!$B$75</f>
         <v>2</v>
       </c>
       <c r="F11" s="28" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="37" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B12" s="40" t="n">
         <f aca="false">B10*B11</f>
         <v>300</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B14" s="36"/>
       <c r="C14" s="36"/>
@@ -5662,7 +5689,7 @@
         <v>124</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C15" s="38" t="s">
         <v>153</v>
@@ -5676,7 +5703,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B16" s="41" t="n">
         <f aca="false">Wyjaśnienia!$B$48</f>
@@ -5691,12 +5718,12 @@
         <v>37500</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B17" s="41" t="n">
         <f aca="false">Wyjaśnienia!$B$47</f>
@@ -5711,12 +5738,12 @@
         <v>1500</v>
       </c>
       <c r="F17" s="28" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="28" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B18" s="41" t="n">
         <f aca="false">Wyjaśnienia!$B$76</f>
@@ -5731,12 +5758,12 @@
         <v>90000</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="37" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D19" s="42" t="n">
         <f aca="false">SUM(D16:D18)</f>
@@ -5772,7 +5799,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B23" s="41" t="n">
         <v>2000</v>
@@ -5785,12 +5812,12 @@
         <v>2000</v>
       </c>
       <c r="F23" s="28" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="28" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B24" s="41" t="n">
         <v>3000</v>
@@ -5803,12 +5830,12 @@
         <v>3000</v>
       </c>
       <c r="F24" s="28" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="28" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B25" s="41" t="n">
         <v>5000</v>
@@ -5821,12 +5848,12 @@
         <v>5000</v>
       </c>
       <c r="F25" s="28" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="28" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B26" s="41" t="n">
         <v>4000</v>
@@ -5839,7 +5866,7 @@
         <v>4000</v>
       </c>
       <c r="F26" s="28" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5863,7 +5890,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="28" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D30" s="41" t="n">
         <f aca="false">D19</f>
@@ -5881,7 +5908,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="28" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D32" s="41" t="n">
         <f aca="false">(D30+D31)*Wyjaśnienia!$B$30</f>
@@ -5917,7 +5944,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="36" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B37" s="36"/>
       <c r="C37" s="36"/>
@@ -5927,7 +5954,7 @@
     </row>
     <row r="38" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="35" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B38" s="35"/>
       <c r="C38" s="35"/>
@@ -5937,19 +5964,19 @@
     </row>
     <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B39" s="38" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C39" s="38" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E39" s="38" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6059,19 +6086,19 @@
     </row>
     <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="38" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B46" s="38" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C46" s="38" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D46" s="38" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E46" s="38" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6181,7 +6208,7 @@
     </row>
     <row r="53" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="35" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B53" s="35"/>
       <c r="C53" s="35"/>
@@ -6240,7 +6267,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B2" s="30"/>
       <c r="C2" s="30"/>
@@ -6250,7 +6277,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B3" s="30"/>
       <c r="C3" s="30"/>
@@ -6290,7 +6317,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B7" s="20" t="n">
         <v>0</v>
@@ -6307,12 +6334,12 @@
         <v>6600</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>25</v>
@@ -6327,12 +6354,12 @@
         <v>5500</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>60</v>
@@ -6347,7 +6374,7 @@
         <v>13200</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6372,7 +6399,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B11" s="20" t="n">
         <v>40</v>
@@ -6387,12 +6414,12 @@
         <v>8800</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B12" s="20" t="n">
         <v>40</v>
@@ -6407,12 +6434,12 @@
         <v>8800</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B13" s="20" t="n">
         <v>25</v>
@@ -6427,12 +6454,12 @@
         <v>5500</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B14" s="20" t="n">
         <v>50</v>
@@ -6447,7 +6474,7 @@
         <v>11000</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6465,7 +6492,7 @@
         <v>63800</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6497,7 +6524,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">Wyjaśnienia!$B$67</f>
@@ -6511,7 +6538,7 @@
         <v>180000</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6530,7 +6557,7 @@
         <v>4000</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6549,12 +6576,12 @@
         <v>1200</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B22" s="8" t="n">
         <v>0</v>
@@ -6567,12 +6594,12 @@
         <v>0</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B23" s="8" t="n">
         <v>0</v>
@@ -6585,12 +6612,12 @@
         <v>0</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B24" s="8" t="n">
         <v>0</v>
@@ -6603,7 +6630,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6621,12 +6648,12 @@
         <v>0</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B26" s="8" t="n">
         <v>0</v>
@@ -6639,7 +6666,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6763,7 +6790,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6775,7 +6802,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -6843,7 +6870,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>45</v>
@@ -6860,7 +6887,7 @@
         <v>9900</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
@@ -6927,7 +6954,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B12" s="26" t="n">
         <v>8000</v>
@@ -6940,7 +6967,7 @@
         <v>8000</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -6948,7 +6975,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="21" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B13" s="26" t="n">
         <v>1500</v>
@@ -6961,7 +6988,7 @@
         <v>1500</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -6969,7 +6996,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B14" s="26" t="n">
         <v>4000</v>
@@ -6982,7 +7009,7 @@
         <v>4000</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -6990,7 +7017,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="21" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B15" s="26" t="n">
         <v>8000</v>
@@ -7003,7 +7030,7 @@
         <v>8000</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -7011,7 +7038,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B16" s="26" t="n">
         <v>0</v>
@@ -7024,12 +7051,12 @@
         <v>0</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B17" s="26" t="n">
         <v>0</v>
@@ -7042,12 +7069,12 @@
         <v>0</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B18" s="26" t="n">
         <v>0</v>
@@ -7060,12 +7087,12 @@
         <v>0</v>
       </c>
       <c r="E18" s="15" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B19" s="26" t="n">
         <v>0</v>
@@ -7078,7 +7105,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7141,7 +7168,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>

</xml_diff>

<commit_message>
Redakcja wstepu do hymnu i lista otwartych wycen w Wyjasnieniach
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -1279,7 +1279,7 @@
     <row r="37" ht="15" customHeight="1" s="44">
       <c r="A37" s="49" t="inlineStr">
         <is>
-          <t>Honoraria jury plebiscytu</t>
+          <t>Honoraria jury plebiscytu piosenki - osobno za ocenę zgłoszeń i za etap przygotowania karty oceny</t>
         </is>
       </c>
       <c r="D37" s="46" t="n"/>
@@ -4167,7 +4167,7 @@
           <t>Razem koszty twarde</t>
         </is>
       </c>
-      <c r="D26">
+      <c r="D26" s="46">
         <f>SUM(D16:D25)</f>
         <v/>
       </c>
@@ -4382,10 +4382,10 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Honoraria jury za etap przygotowawczy we wszystkich czterech budżetach
Obietnica płatnego opracowania karty oceny jest na wszystkich stronach
naboru do jury, a w arkuszu miała ją tylko piosenka. Kwoty do ustalenia,
formuły podsumowań przepisane po wstawieniu wierszy, scalenia naprawione.
Sumy edycji bez zmian: 1 689 626,80 zł netto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="C6" s="51">
-        <f>'Budżet Nagrody'!$D$35</f>
+        <f>'Budżet Nagrody'!$D$36</f>
         <v/>
       </c>
       <c r="D6" s="46" t="n"/>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="C10" s="52">
-        <f>'Budżet Plakatu'!$D$35</f>
+        <f>'Budżet Plakatu'!$D$36</f>
         <v/>
       </c>
       <c r="D10" s="46" t="n"/>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="C11" s="52">
-        <f>'Budżet Filmu'!$D$34</f>
+        <f>'Budżet Filmu'!$D$35</f>
         <v/>
       </c>
     </row>
@@ -861,7 +861,7 @@
         </is>
       </c>
       <c r="C13" s="54">
-        <f>'Budżet Nagrody'!$D$35+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$33+'Budżet Plakatu'!$D$35+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$34</f>
+        <f>'Budżet Nagrody'!$D$36+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$38+'Budżet Plebiscytu'!$D$33+'Budżet Plakatu'!$D$36+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$35</f>
         <v/>
       </c>
       <c r="D13" s="46" t="n"/>
@@ -1279,7 +1279,7 @@
     <row r="37" ht="15" customHeight="1" s="44">
       <c r="A37" s="49" t="inlineStr">
         <is>
-          <t>Honoraria jury plebiscytu piosenki - osobno za ocenę zgłoszeń i za etap przygotowania karty oceny</t>
+          <t>Honoraria jury we wszystkich plebiscytach - osobno za ocenę zgłoszeń i za etap przygotowania karty oceny</t>
         </is>
       </c>
       <c r="D37" s="46" t="n"/>
@@ -1838,7 +1838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="54" customWidth="1" style="43" min="1" max="1"/>
@@ -2384,11 +2384,11 @@
     <row r="25" ht="15" customHeight="1" s="44">
       <c r="A25" s="62" t="inlineStr">
         <is>
-          <t>Promocja naboru</t>
+          <t>Honoraria jury za etap przygotowawczy: karta oceny i wagi kryteriów (netto)</t>
         </is>
       </c>
       <c r="B25" s="67" t="n">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="C25" s="63" t="n">
         <v>1</v>
@@ -2399,21 +2399,19 @@
       </c>
       <c r="E25" s="56" t="inlineStr">
         <is>
-          <t>materiały, obsługa prasowa przy starcie i rozstrzygnięciu, płatne dotarcie</t>
+          <t>DO USTALENIA - etap przed naborem, osobny od oceny zgłoszeń; obejmuje opisy przedziałów punktowych i przykłady ich zastosowania</t>
         </is>
       </c>
       <c r="F25" s="46" t="n"/>
-      <c r="G25" s="46" t="n"/>
-      <c r="H25" s="46" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="44">
       <c r="A26" s="62" t="inlineStr">
         <is>
-          <t>Nagrody publiczności (brutto)</t>
+          <t>Promocja naboru</t>
         </is>
       </c>
       <c r="B26" s="67" t="n">
-        <v>4000</v>
+        <v>15000</v>
       </c>
       <c r="C26" s="63" t="n">
         <v>1</v>
@@ -2424,19 +2422,21 @@
       </c>
       <c r="E26" s="56" t="inlineStr">
         <is>
-          <t>3 000 zł dla zgłoszenia z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych rozmów (§ 11 ust. 8a)</t>
+          <t>materiały, obsługa prasowa przy starcie i rozstrzygnięciu, płatne dotarcie</t>
         </is>
       </c>
       <c r="F26" s="46" t="n"/>
+      <c r="G26" s="46" t="n"/>
+      <c r="H26" s="46" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="44">
       <c r="A27" s="62" t="inlineStr">
         <is>
-          <t>Ubezpieczenie OC organizatora</t>
+          <t>Nagrody publiczności (brutto)</t>
         </is>
       </c>
       <c r="B27" s="67" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="C27" s="63" t="n">
         <v>1</v>
@@ -2447,71 +2447,77 @@
       </c>
       <c r="E27" s="56" t="inlineStr">
         <is>
+          <t>3 000 zł dla zgłoszenia z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych rozmów (§ 11 ust. 8a)</t>
+        </is>
+      </c>
+      <c r="F27" s="46" t="n"/>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="44">
+      <c r="A28" s="62" t="inlineStr">
+        <is>
+          <t>Ubezpieczenie OC organizatora</t>
+        </is>
+      </c>
+      <c r="B28" s="67" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="65">
+        <f>B28*C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="56" t="inlineStr">
+        <is>
           <t>do ustalenia po konsultacji prawnej; na razie pokryte rezerwą</t>
         </is>
       </c>
-      <c r="F27" s="46" t="n"/>
-      <c r="G27" s="46" t="n"/>
-      <c r="H27" s="46" t="n"/>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="44">
-      <c r="A28" s="49" t="inlineStr">
-        <is>
-          <t>Razem koszty twarde</t>
-        </is>
-      </c>
-      <c r="B28" s="46" t="n"/>
-      <c r="C28" s="46" t="n"/>
-      <c r="D28" s="52">
-        <f>SUM(D21:D27)</f>
-        <v/>
-      </c>
-      <c r="E28" s="46" t="n"/>
       <c r="F28" s="46" t="n"/>
       <c r="G28" s="46" t="n"/>
       <c r="H28" s="46" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="44">
-      <c r="A29" s="46" t="n"/>
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>Razem koszty twarde</t>
+        </is>
+      </c>
+      <c r="B29" s="46" t="n"/>
+      <c r="C29" s="46" t="n"/>
+      <c r="D29" s="52">
+        <f>SUM(D21:D28)</f>
+        <v/>
+      </c>
+      <c r="E29" s="46" t="n"/>
+      <c r="F29" s="46" t="n"/>
       <c r="G29" s="46" t="n"/>
       <c r="H29" s="46" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="44">
-      <c r="A30" s="48" t="inlineStr">
-        <is>
-          <t>PODSUMOWANIE</t>
-        </is>
-      </c>
+      <c r="A30" s="46" t="n"/>
       <c r="G30" s="46" t="n"/>
       <c r="H30" s="46" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="44">
-      <c r="A31" s="62" t="inlineStr">
-        <is>
-          <t>Nagrody (brutto dla laureatów, bez VAT)</t>
-        </is>
-      </c>
-      <c r="B31" s="46" t="n"/>
-      <c r="C31" s="46" t="n"/>
-      <c r="D31" s="65">
-        <f>Wyjaśnienia!$B$18+Wyjaśnienia!$B$21+Wyjaśnienia!$B$22+Wyjaśnienia!$B$19*Wyjaśnienia!$B$20</f>
-        <v/>
-      </c>
-      <c r="E31" s="46" t="n"/>
-      <c r="F31" s="46" t="n"/>
+      <c r="A31" s="48" t="inlineStr">
+        <is>
+          <t>PODSUMOWANIE</t>
+        </is>
+      </c>
       <c r="G31" s="46" t="n"/>
       <c r="H31" s="46" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="44">
       <c r="A32" s="62" t="inlineStr">
         <is>
-          <t>Praca organizatora</t>
+          <t>Nagrody (brutto dla laureatów, bez VAT)</t>
         </is>
       </c>
       <c r="B32" s="46" t="n"/>
       <c r="C32" s="46" t="n"/>
-      <c r="D32" s="51">
-        <f>E17</f>
+      <c r="D32" s="65">
+        <f>Wyjaśnienia!$B$18+Wyjaśnienia!$B$21+Wyjaśnienia!$B$22+Wyjaśnienia!$B$19*Wyjaśnienia!$B$20</f>
         <v/>
       </c>
       <c r="E32" s="46" t="n"/>
@@ -2522,13 +2528,13 @@
     <row r="33" ht="15" customHeight="1" s="44">
       <c r="A33" s="62" t="inlineStr">
         <is>
-          <t>Koszty twarde</t>
+          <t>Praca organizatora</t>
         </is>
       </c>
       <c r="B33" s="46" t="n"/>
       <c r="C33" s="46" t="n"/>
       <c r="D33" s="51">
-        <f>D28</f>
+        <f>E17</f>
         <v/>
       </c>
       <c r="E33" s="46" t="n"/>
@@ -2539,43 +2545,43 @@
     <row r="34" ht="15" customHeight="1" s="44">
       <c r="A34" s="62" t="inlineStr">
         <is>
-          <t>Rezerwa (od pracy i kosztów, bez nagród)</t>
-        </is>
-      </c>
-      <c r="D34" s="46">
-        <f>(D32+D33)*Wyjaśnienia!$B$30</f>
-        <v/>
-      </c>
+          <t>Koszty twarde</t>
+        </is>
+      </c>
+      <c r="B34" s="46" t="n"/>
+      <c r="C34" s="46" t="n"/>
+      <c r="D34" s="51">
+        <f>D29</f>
+        <v/>
+      </c>
+      <c r="E34" s="46" t="n"/>
+      <c r="F34" s="46" t="n"/>
       <c r="G34" s="46" t="n"/>
       <c r="H34" s="46" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="44">
-      <c r="A35" s="49" t="inlineStr">
-        <is>
-          <t>RAZEM NETTO</t>
-        </is>
-      </c>
-      <c r="B35" s="46" t="n"/>
-      <c r="C35" s="46" t="n"/>
-      <c r="D35" s="52">
-        <f>SUM(D31:D34)</f>
-        <v/>
-      </c>
-      <c r="E35" s="46" t="n"/>
-      <c r="F35" s="46" t="n"/>
+      <c r="A35" s="62" t="inlineStr">
+        <is>
+          <t>Rezerwa (od pracy i kosztów, bez nagród)</t>
+        </is>
+      </c>
+      <c r="D35" s="46">
+        <f>(D33+D34)*Wyjaśnienia!$B$30</f>
+        <v/>
+      </c>
       <c r="G35" s="46" t="n"/>
       <c r="H35" s="46" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="44">
-      <c r="A36" s="62" t="inlineStr">
-        <is>
-          <t>VAT</t>
+      <c r="A36" s="49" t="inlineStr">
+        <is>
+          <t>RAZEM NETTO</t>
         </is>
       </c>
       <c r="B36" s="46" t="n"/>
       <c r="C36" s="46" t="n"/>
-      <c r="D36" s="51">
-        <f>D35*Wyjaśnienia!$B$33</f>
+      <c r="D36" s="52">
+        <f>SUM(D32:D35)</f>
         <v/>
       </c>
       <c r="E36" s="46" t="n"/>
@@ -2584,15 +2590,15 @@
       <c r="H36" s="46" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="44">
-      <c r="A37" s="49" t="inlineStr">
-        <is>
-          <t>DO ZAPŁATY BRUTTO - ta liczba trafia na fakturę</t>
+      <c r="A37" s="62" t="inlineStr">
+        <is>
+          <t>VAT</t>
         </is>
       </c>
       <c r="B37" s="46" t="n"/>
       <c r="C37" s="46" t="n"/>
-      <c r="D37" s="68">
-        <f>D35+D36</f>
+      <c r="D37" s="51">
+        <f>D36*Wyjaśnienia!$B$33</f>
         <v/>
       </c>
       <c r="E37" s="46" t="n"/>
@@ -2600,7 +2606,23 @@
       <c r="G37" s="46" t="n"/>
       <c r="H37" s="46" t="n"/>
     </row>
-    <row r="38" ht="15" customHeight="1" s="44"/>
+    <row r="38" ht="15" customHeight="1" s="44">
+      <c r="A38" s="49" t="inlineStr">
+        <is>
+          <t>DO ZAPŁATY BRUTTO - ta liczba trafia na fakturę</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="n"/>
+      <c r="C38" s="46" t="n"/>
+      <c r="D38" s="68">
+        <f>D36+D37</f>
+        <v/>
+      </c>
+      <c r="E38" s="46" t="n"/>
+      <c r="F38" s="46" t="n"/>
+      <c r="G38" s="46" t="n"/>
+      <c r="H38" s="46" t="n"/>
+    </row>
     <row r="39" ht="15" customHeight="1" s="44"/>
     <row r="40" ht="15" customHeight="1" s="44"/>
     <row r="41" ht="15" customHeight="1" s="44"/>
@@ -2674,8 +2696,8 @@
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A30:F30"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4399,7 +4421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="54" customWidth="1" style="46" min="1" max="1"/>
@@ -4788,16 +4810,14 @@
     <row r="22" ht="15" customHeight="1" s="44">
       <c r="A22" s="46" t="inlineStr">
         <is>
-          <t>Transport oryginałów w obie strony (netto)</t>
-        </is>
-      </c>
-      <c r="B22" s="51">
-        <f>Wyjaśnienia!$B$61*2</f>
-        <v/>
-      </c>
-      <c r="C22" s="71">
-        <f>Wyjaśnienia!$B$60</f>
-        <v/>
+          <t>Honoraria jury za etap przygotowawczy: karta oceny i wagi kryteriów (netto)</t>
+        </is>
+      </c>
+      <c r="B22" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="71" t="n">
+        <v>1</v>
       </c>
       <c r="D22" s="51">
         <f>B22*C22</f>
@@ -4805,22 +4825,23 @@
       </c>
       <c r="E22" s="46" t="inlineStr">
         <is>
-          <t>szacunek, nie oferta; organizator pokrywa obie strony</t>
+          <t>DO USTALENIA - etap przed naborem, osobny od oceny zgłoszeń; obejmuje opisy przedziałów punktowych i przykłady ich zastosowania</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="44">
       <c r="A23" s="46" t="inlineStr">
         <is>
-          <t>Ubezpieczenie prac na czas wystawy (netto)</t>
+          <t>Transport oryginałów w obie strony (netto)</t>
         </is>
       </c>
       <c r="B23" s="51">
-        <f>Wyjaśnienia!$B$62</f>
-        <v/>
-      </c>
-      <c r="C23" s="71" t="n">
-        <v>1</v>
+        <f>Wyjaśnienia!$B$61*2</f>
+        <v/>
+      </c>
+      <c r="C23" s="71">
+        <f>Wyjaśnienia!$B$60</f>
+        <v/>
       </c>
       <c r="D23" s="51">
         <f>B23*C23</f>
@@ -4828,18 +4849,19 @@
       </c>
       <c r="E23" s="46" t="inlineStr">
         <is>
-          <t>szacunek przy sumie deklarowanej rzędu 100 tys. zł</t>
+          <t>szacunek, nie oferta; organizator pokrywa obie strony</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="44">
       <c r="A24" s="46" t="inlineStr">
         <is>
-          <t>Realizacja wystawy przy gali i wernisażu w galerii (netto)</t>
-        </is>
-      </c>
-      <c r="B24" s="59" t="n">
-        <v>0</v>
+          <t>Ubezpieczenie prac na czas wystawy (netto)</t>
+        </is>
+      </c>
+      <c r="B24" s="51">
+        <f>Wyjaśnienia!$B$62</f>
+        <v/>
       </c>
       <c r="C24" s="71" t="n">
         <v>1</v>
@@ -4850,14 +4872,14 @@
       </c>
       <c r="E24" s="46" t="inlineStr">
         <is>
-          <t>DO WYCENY - zawieszenie, oświetlenie, opisy prac w dwóch miejscach, przewóz między nimi, obsługa wernisażu</t>
+          <t>szacunek przy sumie deklarowanej rzędu 100 tys. zł</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="44">
       <c r="A25" s="46" t="inlineStr">
         <is>
-          <t>Obsługa prawna regulaminu plakatu (netto)</t>
+          <t>Realizacja wystawy przy gali i wernisażu w galerii (netto)</t>
         </is>
       </c>
       <c r="B25" s="59" t="n">
@@ -4872,14 +4894,14 @@
       </c>
       <c r="E25" s="46" t="inlineStr">
         <is>
-          <t>DO WYCENY - odrębne zlecenie kancelarii, nie złożone</t>
+          <t>DO WYCENY - zawieszenie, oświetlenie, opisy prac w dwóch miejscach, przewóz między nimi, obsługa wernisażu</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="44">
       <c r="A26" s="46" t="inlineStr">
         <is>
-          <t>Dojazd i nocleg finalistów na galę (netto)</t>
+          <t>Obsługa prawna regulaminu plakatu (netto)</t>
         </is>
       </c>
       <c r="B26" s="59" t="n">
@@ -4894,14 +4916,14 @@
       </c>
       <c r="E26" s="46" t="inlineStr">
         <is>
-          <t>DO WYCENY - jak przy plebiscycie piosenki</t>
+          <t>DO WYCENY - odrębne zlecenie kancelarii, nie złożone</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="44">
       <c r="A27" s="46" t="inlineStr">
         <is>
-          <t>Polisa: wycena prac, rozszerzenie na przechowywanie i okres po sprzedaży (netto)</t>
+          <t>Dojazd i nocleg finalistów na galę (netto)</t>
         </is>
       </c>
       <c r="B27" s="59" t="n">
@@ -4916,105 +4938,127 @@
       </c>
       <c r="E27" s="46" t="inlineStr">
         <is>
+          <t>DO WYCENY - jak przy plebiscycie piosenki</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1" s="44">
+      <c r="A28" s="46" t="inlineStr">
+        <is>
+          <t>Polisa: wycena prac, rozszerzenie na przechowywanie i okres po sprzedaży (netto)</t>
+        </is>
+      </c>
+      <c r="B28" s="59" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="51">
+        <f>B28*C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="46" t="inlineStr">
+        <is>
           <t>DO WYCENY - polisa ma objąć cały uzgodniony okres: transport w obie strony, przechowywanie u organizatora, obie wystawy oraz czas po sprzedaży do wydania pracy nabywcy; do ustalenia suma ubezpieczenia na pracę, udział własny i procedura zgłoszenia szkody</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="44">
-      <c r="A28" s="53" t="inlineStr">
+    <row r="29" ht="15" customHeight="1" s="44">
+      <c r="A29" s="53" t="inlineStr">
         <is>
           <t>Razem koszty twarde</t>
         </is>
       </c>
-      <c r="D28" s="54">
-        <f>SUM(D18:D27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="44">
-      <c r="A29" s="46" t="n"/>
+      <c r="D29">
+        <f>SUM(D18:D28)</f>
+        <v/>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="44">
-      <c r="A30" s="53" t="inlineStr">
+      <c r="A30" s="46" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="44">
+      <c r="A31" s="53" t="inlineStr">
         <is>
           <t>PODSUMOWANIE</t>
         </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="44">
-      <c r="A31" s="46" t="inlineStr">
-        <is>
-          <t>Nagrody (brutto dla laureatów, bez VAT)</t>
-        </is>
-      </c>
-      <c r="D31" s="51">
-        <f>Wyjaśnienia!$B$54+Wyjaśnienia!$B$55</f>
-        <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="44">
       <c r="A32" s="46" t="inlineStr">
         <is>
-          <t>Praca organizatora</t>
+          <t>Nagrody (brutto dla laureatów, bez VAT)</t>
         </is>
       </c>
       <c r="D32" s="51">
-        <f>E14</f>
+        <f>Wyjaśnienia!$B$54+Wyjaśnienia!$B$55</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="44">
       <c r="A33" s="46" t="inlineStr">
         <is>
-          <t>Koszty twarde bez nagród</t>
+          <t>Praca organizatora</t>
         </is>
       </c>
       <c r="D33" s="51">
-        <f>D28-D31</f>
+        <f>E14</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="44">
       <c r="A34" s="46" t="inlineStr">
         <is>
+          <t>Koszty twarde bez nagród</t>
+        </is>
+      </c>
+      <c r="D34" s="51">
+        <f>D29-D32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="44">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
           <t>Rezerwa (od pracy i kosztów, bez nagród)</t>
         </is>
       </c>
-      <c r="D34" s="51">
-        <f>(D32+D33)*Wyjaśnienia!$B$63</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="44">
-      <c r="A35" s="53" t="inlineStr">
+      <c r="D35" s="51">
+        <f>(D33+D34)*Wyjaśnienia!$B$63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="44">
+      <c r="A36" s="53" t="inlineStr">
         <is>
           <t>RAZEM NETTO</t>
         </is>
       </c>
-      <c r="D35" s="54">
-        <f>SUM(D31:D34)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="44">
-      <c r="A36" s="46" t="inlineStr">
+      <c r="D36" s="54">
+        <f>SUM(D32:D35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="44">
+      <c r="A37" s="46" t="inlineStr">
         <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="D36" s="51">
-        <f>D35*Wyjaśnienia!$B$33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="15" customHeight="1" s="44">
-      <c r="A37" s="53" t="inlineStr">
+      <c r="D37" s="51">
+        <f>D36*Wyjaśnienia!$B$33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="53" t="inlineStr">
         <is>
           <t>DO ZAPŁATY BRUTTO - ta liczba trafia na fakturę</t>
         </is>
       </c>
-      <c r="D37" s="54">
-        <f>D35+D36</f>
+      <c r="D38" s="54">
+        <f>D36+D37</f>
         <v/>
       </c>
     </row>
@@ -5025,7 +5069,7 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5824,7 +5868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.5703125" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="54" customWidth="1" style="46" min="1" max="1"/>
@@ -6239,7 +6283,7 @@
     <row r="23" ht="15" customHeight="1" s="44">
       <c r="A23" s="46" t="inlineStr">
         <is>
-          <t>Przygotowanie techniczne zwiastunów do emisji galowej (netto)</t>
+          <t>Honoraria jury za etap przygotowawczy: karta oceny i wagi kryteriów (netto)</t>
         </is>
       </c>
       <c r="B23" s="51" t="n">
@@ -6254,14 +6298,14 @@
       </c>
       <c r="E23" s="46" t="inlineStr">
         <is>
-          <t>DO WYCENY - pobranie pięciu zwiastunów w jakości emisyjnej, zgodność formatów, normalizacja dźwięku, plansze z tytułami; zwiastun dostarcza autor, Organizator nie montuje fragmentów filmów</t>
+          <t>DO USTALENIA - etap przed naborem, osobny od oceny zgłoszeń; obejmuje opisy przedziałów punktowych i przykłady ich zastosowania</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="44">
       <c r="A24" s="46" t="inlineStr">
         <is>
-          <t>Pokazy kinowe filmów finałowych (netto)</t>
+          <t>Przygotowanie techniczne zwiastunów do emisji galowej (netto)</t>
         </is>
       </c>
       <c r="B24" s="51" t="n">
@@ -6276,14 +6320,14 @@
       </c>
       <c r="E24" s="46" t="inlineStr">
         <is>
-          <t>DO WYCENY - opracowanie techniczne kopii, napisy i materiały informacyjne dla zestawu dziesiątki; zależy od pozyskania dystrybutora (§ 10 ust. 4), z którym Organizator może uzgodnić pokrycie tych kosztów</t>
+          <t>DO WYCENY - pobranie pięciu zwiastunów w jakości emisyjnej, zgodność formatów, normalizacja dźwięku, plansze z tytułami; zwiastun dostarcza autor, Organizator nie montuje fragmentów filmów</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="44">
       <c r="A25" s="46" t="inlineStr">
         <is>
-          <t>Dojazd i nocleg finalistów na galę (netto)</t>
+          <t>Pokazy kinowe filmów finałowych (netto)</t>
         </is>
       </c>
       <c r="B25" s="51" t="n">
@@ -6298,14 +6342,14 @@
       </c>
       <c r="E25" s="46" t="inlineStr">
         <is>
-          <t>DO WYCENY - jak przy plebiscycie piosenki; dziesięciu finalistów, często z ekipą</t>
+          <t>DO WYCENY - opracowanie techniczne kopii, napisy i materiały informacyjne dla zestawu dziesiątki; zależy od pozyskania dystrybutora (§ 10 ust. 4), z którym Organizator może uzgodnić pokrycie tych kosztów</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="44">
       <c r="A26" s="46" t="inlineStr">
         <is>
-          <t>Obsługa prawna regulaminu filmu (netto)</t>
+          <t>Dojazd i nocleg finalistów na galę (netto)</t>
         </is>
       </c>
       <c r="B26" s="51" t="n">
@@ -6320,104 +6364,127 @@
       </c>
       <c r="E26" s="46" t="inlineStr">
         <is>
+          <t>DO WYCENY - jak przy plebiscycie piosenki; dziesięciu finalistów, często z ekipą</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="44">
+      <c r="A27" s="46" t="inlineStr">
+        <is>
+          <t>Obsługa prawna regulaminu filmu (netto)</t>
+        </is>
+      </c>
+      <c r="B27" s="51" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="51">
+        <f>B27*C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="46" t="inlineStr">
+        <is>
           <t>DO WYCENY - odrębne zlecenie kancelarii, nie złożone; siedem miejsc wypisanych na końcu regulaminu, w tym status filmu wygenerowanego w całości</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="44">
-      <c r="A27" s="53" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="53" t="inlineStr">
         <is>
           <t>Razem koszty twarde</t>
         </is>
       </c>
-      <c r="B27" s="51" t="n"/>
-      <c r="C27" s="71" t="n"/>
-      <c r="D27" s="54">
-        <f>SUM(D19:D26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="44">
-      <c r="A29" s="53" t="inlineStr">
+      <c r="B28" s="51" t="n"/>
+      <c r="C28" s="71" t="n"/>
+      <c r="D28" s="54">
+        <f>SUM(D19:D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1" s="44"/>
+    <row r="30" ht="15" customHeight="1" s="44">
+      <c r="A30" s="53" t="inlineStr">
         <is>
           <t>PODSUMOWANIE</t>
         </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="44">
-      <c r="A30" s="46" t="inlineStr">
-        <is>
-          <t>Nagrody (brutto dla laureatów, bez VAT)</t>
-        </is>
-      </c>
-      <c r="D30" s="51">
-        <f>Wyjaśnienia!$B$67+Wyjaśnienia!$B$68</f>
-        <v/>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="44">
       <c r="A31" s="46" t="inlineStr">
         <is>
-          <t>Praca organizatora</t>
+          <t>Nagrody (brutto dla laureatów, bez VAT)</t>
         </is>
       </c>
       <c r="D31" s="51">
-        <f>E15</f>
+        <f>Wyjaśnienia!$B$67+Wyjaśnienia!$B$68</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="44">
       <c r="A32" s="46" t="inlineStr">
         <is>
-          <t>Koszty twarde bez nagród</t>
+          <t>Praca organizatora</t>
         </is>
       </c>
       <c r="D32" s="51">
-        <f>D27-D30</f>
+        <f>E15</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="44">
       <c r="A33" s="46" t="inlineStr">
         <is>
+          <t>Koszty twarde bez nagród</t>
+        </is>
+      </c>
+      <c r="D33" s="51">
+        <f>D28-D31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="44">
+      <c r="A34" s="46" t="inlineStr">
+        <is>
           <t>Rezerwa (od pracy i kosztów, bez nagród)</t>
         </is>
       </c>
-      <c r="D33" s="51">
-        <f>(D31+D32)*Wyjaśnienia!$B$74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="44">
-      <c r="A34" s="53" t="inlineStr">
+      <c r="D34" s="51">
+        <f>(D32+D33)*Wyjaśnienia!$B$74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="44">
+      <c r="A35" s="53" t="inlineStr">
         <is>
           <t>RAZEM NETTO</t>
         </is>
       </c>
-      <c r="D34" s="54">
-        <f>SUM(D30:D33)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="44">
-      <c r="A35" s="46" t="inlineStr">
+      <c r="D35" s="54">
+        <f>SUM(D31:D34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="44">
+      <c r="A36" s="46" t="inlineStr">
         <is>
           <t>VAT</t>
         </is>
       </c>
-      <c r="D35" s="51">
-        <f>D34*Wyjaśnienia!$B$33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="44">
-      <c r="A36" s="53" t="inlineStr">
+      <c r="D36" s="51">
+        <f>D35*Wyjaśnienia!$B$33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="53" t="inlineStr">
         <is>
           <t>DO ZAPŁATY BRUTTO - ta liczba trafia na fakturę</t>
         </is>
       </c>
-      <c r="D36" s="54">
-        <f>D34+D35</f>
+      <c r="D37" s="54">
+        <f>D35+D36</f>
         <v/>
       </c>
     </row>
@@ -6428,7 +6495,7 @@
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A30:F30"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Rozpoczęcie edycji nie jest uzależnione od hymnu
Premiera hymnu przestaje być warunkiem otwarcia naboru we wszystkich
materiałach: piśmie i nocie dla MKiDN, liście pytań dla kancelarii,
koncepcji i w uwadze przy pozycji budżetowej. Termin nagrania zależy
od zabezpieczenia środków i od skompletowania jury, które hymn wykonuje.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -4027,7 +4027,7 @@
       </c>
       <c r="E19" s="56" t="inlineStr">
         <is>
-          <t>nagranie i premiera na początku 2027, otwiera nabór</t>
+          <t>premiera w czasie trwania naboru w 2027; otwarcie edycji nie jest od niej uzależnione</t>
         </is>
       </c>
       <c r="F19" s="46" t="n"/>
@@ -4970,7 +4970,7 @@
           <t>Razem koszty twarde</t>
         </is>
       </c>
-      <c r="D29">
+      <c r="D29" s="46">
         <f>SUM(D18:D28)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Nowa drabinka nagród w plebiscycie na rozmowę
300 tys. zł, 40 tys. zł, 10 tys. zł i siedem wyróżnień po 3 tys. zł,
czyli pula 371 tys. zł zamiast 395 tys. Porządek nagród przestaje być
odwrócony: dotąd wyróżnienie było dwukrotnie wyższe od trzeciego
miejsca. Kwoty przeliczone w arkuszu i poprawione w notach dla obu
ministerstw; suma edycji wynosi teraz 1 665 626,80 zł netto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="B19" s="55" t="n">
-        <v>10000</v>
+        <v>3000</v>
       </c>
       <c r="C19" s="56" t="inlineStr">
         <is>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="B21" s="55" t="n">
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="C21" s="56" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
         </is>
       </c>
       <c r="B22" s="55" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="C22" s="56" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Arkusz budżetowy mówi "plebiscyt" o naszych plebiscytach
Sześć komórek zostało przy starej nazwie, bo czyszczenie słowa
"konkurs" przeszło po stronach, a nie po treści komórek: mecenas
plebiscytu na plakat w zakładce Wyjaśnienia i w nagłówku Budżetu
Plakatu, dwie notki o medalu i dwie o przejęciu pierwszej oceny przez
Akademię. Dwa odwołania do konkursów obcych - konkursy plakatowe jako
kanał dotarcia i wyniki konkursów przy weryfikacji daty filmu -
zostają, bo dotyczą cudzych przedsięwzięć. Sumy bez zmian.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -809,7 +809,7 @@
       </c>
       <c r="B10" s="46" t="inlineStr">
         <is>
-          <t>Mecenas konkursu plakatu</t>
+          <t>Mecenas plebiscytu na plakat</t>
         </is>
       </c>
       <c r="C10" s="52">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="C29" s="56" t="inlineStr">
         <is>
-          <t>Ten sam mosiężny medal co w konkursie rozmów, cena jak w Budżecie Nagrody.</t>
+          <t>Ten sam mosiężny medal co w plebiscycie na rozmowę, cena jak w Budżecie Nagrody.</t>
         </is>
       </c>
       <c r="D29" s="46" t="n"/>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="C56" s="43" t="inlineStr">
         <is>
-          <t>Ten sam mosiężny medal co w konkursie rozmów, cena jak w Budżecie Nagrody.</t>
+          <t>Ten sam mosiężny medal co w plebiscycie na rozmowę, cena jak w Budżecie Nagrody.</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="F12" s="46" t="inlineStr">
         <is>
-          <t>Powyżej progu zgłoszeń pierwsze przejście oceny przechodzi na Akademię, tak jak w konkursie rozmów - dlatego te godziny nie rosną z naborem. Minuty na zgłoszenie dotyczą wyłącznie kontroli formalnej.</t>
+          <t>Powyżej progu zgłoszeń pierwsze przejście oceny przechodzi na Akademię, tak jak w plebiscycie na rozmowę - dlatego te godziny nie rosną z naborem. Minuty na zgłoszenie dotyczą wyłącznie kontroli formalnej.</t>
         </is>
       </c>
       <c r="G12" s="46" t="n"/>
@@ -4442,7 +4442,7 @@
     <row r="2" ht="15" customHeight="1" s="44">
       <c r="A2" s="46" t="inlineStr">
         <is>
-          <t>Finansuje: Mecenas konkursu plakatu. Kwoty netto, chyba że napisano inaczej.</t>
+          <t>Finansuje: Mecenas plebiscytu na plakat. Kwoty netto, chyba że napisano inaczej.</t>
         </is>
       </c>
     </row>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="F14" s="46" t="inlineStr">
         <is>
-          <t>Powyżej progu zgłoszeń pierwsze przejście oceny przechodzi na Akademię, tak jak w konkursie rozmów - dlatego te godziny nie rosną z naborem. Minuty na zgłoszenie dotyczą wyłącznie kontroli formalnej.</t>
+          <t>Powyżej progu zgłoszeń pierwsze przejście oceny przechodzi na Akademię, tak jak w plebiscycie na rozmowę - dlatego te godziny nie rosną z naborem. Minuty na zgłoszenie dotyczą wyłącznie kontroli formalnej.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tabela skalowania akademii liczy godziny pracy, nie osoby
Kolumna "Potrzebnych czytelników" dzieliła liczbę odczytów przez puste
pole "Maksimum zgłoszeń na czytelnika", przez co pięć wierszy tabeli
pokazywało błąd dzielenia. Sama wielkość była przy tym krucha: ile
zgłoszeń przeczyta jedna osoba, zależy od tego, czy robi to etatowo,
czy wieczorami, więc nie jest parametrem konstrukcji.

Tabela podaje teraz godziny pracy akademii, liczone od liczby odczytów
i od przyjętego czasu jednego odczytu wraz z kartą oceny, który wynosi
30 minut i jest polem do edycji. Przy 150 zgłoszeniach daje to 150
godzin, przy 1000 - tysiąc. Sumy budżetu bez zmian.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -254,7 +254,7 @@
     <t xml:space="preserve">Maksymalnie 20 zgłoszeń na czytelnika (regulamin § 8).</t>
   </si>
   <si>
-    <t xml:space="preserve">Maksimum zgłoszeń na czytelnika</t>
+    <t xml:space="preserve">Czas na jeden odczyt rozmowy wraz z kartą oceny (minut)</t>
   </si>
   <si>
     <t xml:space="preserve">PLAKAT - PARAMETRY</t>
@@ -995,7 +995,7 @@
     <t xml:space="preserve">JAK TO SIĘ SKALUJE</t>
   </si>
   <si>
-    <t xml:space="preserve">Vouchery i honoraria za obejrzenia rosną wprost z liczbą zgłoszeń, więc sponsor płaci za wykonaną pracę, a nie za prognozę. Ludzi trzeba jednak znaleźć osobno: kolumny Potrzebnych liczą osoby od liczby ODCZYTÓW i OBEJRZEŃ, nie od liczby zgłoszeń. Tabela przy większych wolumenach nie modeluje odrębnie trybu jednoosobowego, drugich odczytów poniżej progu ani audytu losowego - te trzy rzeczy trzeba policzyć osobno przed ogłoszeniem progu.</t>
+    <t xml:space="preserve">Vouchery i honoraria za obejrzenia rosną wprost z liczbą zgłoszeń, więc sponsor płaci za wykonaną pracę, a nie za prognozę. Kolumna godzin liczy pracę akademii od liczby ODCZYTÓW, po przyjętym czasie jednego odczytu z zakładki Wyjaśnienia; ilu osób to wymaga, zależy od tego, ile godzin daje pojedynczy czytelnik, i tego tabela nie przesądza. Przy większych wolumenach nie modeluje też odrębnie trybu jednoosobowego, drugich odczytów poniżej progu ani audytu losowego - te trzy rzeczy trzeba policzyć osobno przed ogłoszeniem progu.</t>
   </si>
   <si>
     <t xml:space="preserve">Zgłoszeń w edycji</t>
@@ -1010,7 +1010,7 @@
     <t xml:space="preserve">Koszt voucherów</t>
   </si>
   <si>
-    <t xml:space="preserve">Potrzebnych czytelników</t>
+    <t xml:space="preserve">Godzin pracy akademii</t>
   </si>
   <si>
     <t xml:space="preserve">Filmów w edycji</t>
@@ -1338,7 +1338,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1412,6 +1412,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2399,10 +2403,13 @@
       <c r="A50" s="3" t="s">
         <v>75</v>
       </c>
+      <c r="B50" s="19" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="19" t="s">
+      <c r="A52" s="20" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2410,7 +2417,7 @@
       <c r="A53" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B53" s="20" t="n">
+      <c r="B53" s="21" t="n">
         <v>150</v>
       </c>
       <c r="C53" s="1" t="s">
@@ -2454,7 +2461,7 @@
       <c r="A57" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B57" s="20" t="n">
+      <c r="B57" s="21" t="n">
         <v>5</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -2465,7 +2472,7 @@
       <c r="A58" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B58" s="20" t="n">
+      <c r="B58" s="21" t="n">
         <v>10</v>
       </c>
       <c r="C58" s="1" t="s">
@@ -2487,7 +2494,7 @@
       <c r="A60" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B60" s="20" t="n">
+      <c r="B60" s="21" t="n">
         <v>10</v>
       </c>
       <c r="C60" s="1" t="s">
@@ -2529,7 +2536,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="19" t="s">
+      <c r="A65" s="20" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2806,20 +2813,20 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>60</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="24" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$17/60</f>
         <v>60</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="25" t="n">
         <f aca="false">D7*Wyjaśnienia!$B$16</f>
         <v>13200</v>
       </c>
@@ -2830,20 +2837,20 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <v>24</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="24" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$17/60</f>
         <v>24</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="25" t="n">
         <f aca="false">D8*Wyjaśnienia!$B$16</f>
         <v>5280</v>
       </c>
@@ -2854,20 +2861,20 @@
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="24" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$17/60</f>
         <v>50</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="25" t="n">
         <f aca="false">D9*Wyjaśnienia!$B$16</f>
         <v>11000</v>
       </c>
@@ -2878,20 +2885,20 @@
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>6</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="24" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$17/60</f>
         <v>23</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="E10" s="25" t="n">
         <f aca="false">D10*Wyjaśnienia!$B$16</f>
         <v>5060</v>
       </c>
@@ -2902,20 +2909,20 @@
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="22" t="s">
         <v>138</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="24" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$17/60</f>
         <v>20</v>
       </c>
-      <c r="E11" s="24" t="n">
+      <c r="E11" s="25" t="n">
         <f aca="false">D11*Wyjaśnienia!$B$16</f>
         <v>4400</v>
       </c>
@@ -2926,20 +2933,20 @@
       <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="B12" s="22" t="n">
+      <c r="B12" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="24" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$17/60</f>
         <v>20</v>
       </c>
-      <c r="E12" s="24" t="n">
+      <c r="E12" s="25" t="n">
         <f aca="false">D12*Wyjaśnienia!$B$16</f>
         <v>4400</v>
       </c>
@@ -2950,20 +2957,20 @@
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="B13" s="22" t="n">
+      <c r="B13" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="24" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$17/60</f>
         <v>40</v>
       </c>
-      <c r="E13" s="24" t="n">
+      <c r="E13" s="25" t="n">
         <f aca="false">D13*Wyjaśnienia!$B$16</f>
         <v>8800</v>
       </c>
@@ -2974,20 +2981,20 @@
       <c r="H13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B14" s="22" t="n">
+      <c r="B14" s="23" t="n">
         <v>25</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="24" t="n">
         <f aca="false">B14+C14*Wyjaśnienia!$B$17/60</f>
         <v>25</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="25" t="n">
         <f aca="false">D14*Wyjaśnienia!$B$16</f>
         <v>5500</v>
       </c>
@@ -2998,20 +3005,20 @@
       <c r="H14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="23" t="n">
         <v>25</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="24" t="n">
         <f aca="false">B15+C15*Wyjaśnienia!$B$17/60</f>
         <v>25</v>
       </c>
-      <c r="E15" s="24" t="n">
+      <c r="E15" s="25" t="n">
         <f aca="false">D15*Wyjaśnienia!$B$16</f>
         <v>5500</v>
       </c>
@@ -3022,20 +3029,20 @@
       <c r="H15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="24" t="n">
         <f aca="false">B16+C16*Wyjaśnienia!$B$17/60</f>
         <v>40</v>
       </c>
-      <c r="E16" s="24" t="n">
+      <c r="E16" s="25" t="n">
         <f aca="false">D16*Wyjaśnienia!$B$16</f>
         <v>8800</v>
       </c>
@@ -3051,7 +3058,7 @@
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
-      <c r="D17" s="25" t="n">
+      <c r="D17" s="26" t="n">
         <f aca="false">SUM(D7:D16)</f>
         <v>327</v>
       </c>
@@ -3105,16 +3112,16 @@
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="22" t="s">
         <v>154</v>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="27" t="n">
         <v>1200</v>
       </c>
-      <c r="C21" s="22" t="n">
+      <c r="C21" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="25" t="n">
         <f aca="false">B21*C21</f>
         <v>1200</v>
       </c>
@@ -3126,16 +3133,16 @@
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="27" t="n">
         <v>1500</v>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="25" t="n">
         <f aca="false">B22*C22</f>
         <v>1500</v>
       </c>
@@ -3147,16 +3154,16 @@
       <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="27" t="n">
         <v>250</v>
       </c>
-      <c r="C23" s="22" t="n">
+      <c r="C23" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="25" t="n">
         <f aca="false">B23*C23</f>
         <v>250</v>
       </c>
@@ -3168,16 +3175,16 @@
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="B24" s="26" t="n">
+      <c r="B24" s="27" t="n">
         <v>32000</v>
       </c>
-      <c r="C24" s="22" t="n">
+      <c r="C24" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="24" t="n">
+      <c r="D24" s="25" t="n">
         <f aca="false">B24*C24</f>
         <v>32000</v>
       </c>
@@ -3191,16 +3198,16 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B25" s="26" t="n">
+      <c r="B25" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C25" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="24" t="n">
+      <c r="D25" s="25" t="n">
         <f aca="false">B25*C25</f>
         <v>0</v>
       </c>
@@ -3210,16 +3217,16 @@
       <c r="F25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="B26" s="26" t="n">
+      <c r="B26" s="27" t="n">
         <v>15000</v>
       </c>
-      <c r="C26" s="22" t="n">
+      <c r="C26" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="24" t="n">
+      <c r="D26" s="25" t="n">
         <f aca="false">B26*C26</f>
         <v>15000</v>
       </c>
@@ -3231,16 +3238,16 @@
       <c r="H26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="B27" s="26" t="n">
+      <c r="B27" s="27" t="n">
         <v>4000</v>
       </c>
-      <c r="C27" s="22" t="n">
+      <c r="C27" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D27" s="25" t="n">
         <f aca="false">B27*C27</f>
         <v>4000</v>
       </c>
@@ -3250,16 +3257,16 @@
       <c r="F27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="22" t="s">
         <v>169</v>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C28" s="22" t="n">
+      <c r="C28" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="24" t="n">
+      <c r="D28" s="25" t="n">
         <f aca="false">B28*C28</f>
         <v>0</v>
       </c>
@@ -3303,12 +3310,12 @@
       <c r="H31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="22" t="s">
         <v>173</v>
       </c>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
-      <c r="D32" s="24" t="n">
+      <c r="D32" s="25" t="n">
         <f aca="false">Wyjaśnienia!$B$18+Wyjaśnienia!$B$21+Wyjaśnienia!$B$22+Wyjaśnienia!$B$19*Wyjaśnienia!$B$20</f>
         <v>371000</v>
       </c>
@@ -3318,7 +3325,7 @@
       <c r="H32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="21" t="s">
+      <c r="A33" s="22" t="s">
         <v>174</v>
       </c>
       <c r="B33" s="3"/>
@@ -3333,7 +3340,7 @@
       <c r="H33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="22" t="s">
         <v>175</v>
       </c>
       <c r="B34" s="3"/>
@@ -3348,7 +3355,7 @@
       <c r="H34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="22" t="s">
         <v>176</v>
       </c>
       <c r="D35" s="3" t="n">
@@ -3374,7 +3381,7 @@
       <c r="H36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21" t="s">
+      <c r="A37" s="22" t="s">
         <v>178</v>
       </c>
       <c r="B37" s="3"/>
@@ -3394,7 +3401,7 @@
       </c>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
-      <c r="D38" s="27" t="n">
+      <c r="D38" s="28" t="n">
         <f aca="false">D36+D37</f>
         <v>629756.064</v>
       </c>
@@ -3586,20 +3593,20 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>45</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="24" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$17/60</f>
         <v>45</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="25" t="n">
         <f aca="false">D7*Wyjaśnienia!$B$16</f>
         <v>9900</v>
       </c>
@@ -3610,20 +3617,20 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="24" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$17/60</f>
         <v>40</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="25" t="n">
         <f aca="false">D8*Wyjaśnienia!$B$16</f>
         <v>8800</v>
       </c>
@@ -3634,20 +3641,20 @@
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="24" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$17/60</f>
         <v>10</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="25" t="n">
         <f aca="false">D9*Wyjaśnienia!$B$16</f>
         <v>2200</v>
       </c>
@@ -3658,20 +3665,20 @@
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="24" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$17/60</f>
         <v>50</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="E10" s="25" t="n">
         <f aca="false">D10*Wyjaśnienia!$B$16</f>
         <v>11000</v>
       </c>
@@ -3682,20 +3689,20 @@
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="23" t="n">
         <v>25</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C11" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="24" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$17/60</f>
         <v>25</v>
       </c>
-      <c r="E11" s="24" t="n">
+      <c r="E11" s="25" t="n">
         <f aca="false">D11*Wyjaśnienia!$B$16</f>
         <v>5500</v>
       </c>
@@ -3706,20 +3713,20 @@
       <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>191</v>
       </c>
-      <c r="B12" s="22" t="n">
+      <c r="B12" s="23" t="n">
         <v>160</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="23" t="n">
+      <c r="D12" s="24" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$17/60</f>
         <v>160</v>
       </c>
-      <c r="E12" s="24" t="n">
+      <c r="E12" s="25" t="n">
         <f aca="false">D12*Wyjaśnienia!$B$16</f>
         <v>35200</v>
       </c>
@@ -3730,20 +3737,20 @@
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="B13" s="22" t="n">
+      <c r="B13" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="24" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$17/60</f>
         <v>50</v>
       </c>
-      <c r="E13" s="24" t="n">
+      <c r="E13" s="25" t="n">
         <f aca="false">D13*Wyjaśnienia!$B$16</f>
         <v>11000</v>
       </c>
@@ -3754,20 +3761,20 @@
       <c r="H13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>195</v>
       </c>
-      <c r="B14" s="22" t="n">
+      <c r="B14" s="23" t="n">
         <v>72</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="24" t="n">
         <f aca="false">B14+C14*Wyjaśnienia!$B$17/60</f>
         <v>72</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="25" t="n">
         <f aca="false">D14*Wyjaśnienia!$B$16</f>
         <v>15840</v>
       </c>
@@ -3779,7 +3786,7 @@
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
-      <c r="D15" s="25" t="n">
+      <c r="D15" s="26" t="n">
         <f aca="false">SUM(D7:D14)</f>
         <v>452</v>
       </c>
@@ -3834,16 +3841,16 @@
       <c r="H18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="B19" s="26" t="n">
+      <c r="B19" s="27" t="n">
         <v>3000</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="25" t="n">
         <f aca="false">B19*C19</f>
         <v>3000</v>
       </c>
@@ -3855,16 +3862,16 @@
       <c r="H19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="B20" s="26" t="n">
+      <c r="B20" s="27" t="n">
         <v>6000</v>
       </c>
-      <c r="C20" s="22" t="n">
+      <c r="C20" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="25" t="n">
         <f aca="false">B20*C20</f>
         <v>6000</v>
       </c>
@@ -3878,16 +3885,16 @@
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="22" t="s">
         <v>201</v>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="27" t="n">
         <v>10000</v>
       </c>
-      <c r="C21" s="22" t="n">
+      <c r="C21" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="25" t="n">
         <f aca="false">B21*C21</f>
         <v>10000</v>
       </c>
@@ -3899,16 +3906,16 @@
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>203</v>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="27" t="n">
         <v>40000</v>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="25" t="n">
         <f aca="false">B22*C22</f>
         <v>40000</v>
       </c>
@@ -3920,16 +3927,16 @@
       <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="22" t="s">
         <v>205</v>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="27" t="n">
         <v>4000</v>
       </c>
-      <c r="C23" s="22" t="n">
+      <c r="C23" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="25" t="n">
         <f aca="false">B23*C23</f>
         <v>4000</v>
       </c>
@@ -3941,16 +3948,16 @@
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>207</v>
       </c>
-      <c r="B24" s="26" t="n">
+      <c r="B24" s="27" t="n">
         <v>3000</v>
       </c>
-      <c r="C24" s="22" t="n">
+      <c r="C24" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="24" t="n">
+      <c r="D24" s="25" t="n">
         <f aca="false">B24*C24</f>
         <v>3000</v>
       </c>
@@ -3962,16 +3969,16 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="22" t="s">
         <v>209</v>
       </c>
-      <c r="B25" s="26" t="n">
+      <c r="B25" s="27" t="n">
         <v>4000</v>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C25" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="24" t="n">
+      <c r="D25" s="25" t="n">
         <f aca="false">B25*C25</f>
         <v>4000</v>
       </c>
@@ -3983,16 +3990,16 @@
       <c r="H25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="21" t="s">
+      <c r="A26" s="22" t="s">
         <v>211</v>
       </c>
-      <c r="B26" s="26" t="n">
+      <c r="B26" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="22" t="n">
+      <c r="C26" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="24" t="n">
+      <c r="D26" s="25" t="n">
         <f aca="false">B26*C26</f>
         <v>0</v>
       </c>
@@ -4004,16 +4011,16 @@
       <c r="H26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="22" t="s">
         <v>213</v>
       </c>
-      <c r="B27" s="26" t="n">
+      <c r="B27" s="27" t="n">
         <v>15000</v>
       </c>
-      <c r="C27" s="22" t="n">
+      <c r="C27" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D27" s="25" t="n">
         <f aca="false">B27*C27</f>
         <v>15000</v>
       </c>
@@ -4025,16 +4032,16 @@
       <c r="H27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="s">
+      <c r="A28" s="22" t="s">
         <v>215</v>
       </c>
-      <c r="B28" s="26" t="n">
+      <c r="B28" s="27" t="n">
         <v>6000</v>
       </c>
-      <c r="C28" s="22" t="n">
+      <c r="C28" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D28" s="24" t="n">
+      <c r="D28" s="25" t="n">
         <f aca="false">B28*C28</f>
         <v>6000</v>
       </c>
@@ -4046,16 +4053,16 @@
       <c r="H28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="B29" s="26" t="n">
+      <c r="B29" s="27" t="n">
         <v>30000</v>
       </c>
-      <c r="C29" s="22" t="n">
+      <c r="C29" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="24" t="n">
+      <c r="D29" s="25" t="n">
         <f aca="false">B29*C29</f>
         <v>30000</v>
       </c>
@@ -4067,31 +4074,31 @@
       <c r="H29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="29" t="s">
         <v>219</v>
       </c>
       <c r="B30" s="18" t="n">
         <v>4500</v>
       </c>
-      <c r="C30" s="29" t="n">
+      <c r="C30" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="8" t="n">
         <f aca="false">B30*C30</f>
         <v>4500</v>
       </c>
-      <c r="F30" s="28" t="s">
+      <c r="F30" s="29" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="29" t="s">
         <v>221</v>
       </c>
       <c r="B31" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="29" t="n">
+      <c r="C31" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="8" t="n">
@@ -4101,7 +4108,7 @@
       <c r="E31" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="F31" s="28"/>
+      <c r="F31" s="29"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
@@ -4119,12 +4126,12 @@
       <c r="H32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="30"/>
-      <c r="B33" s="30"/>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
+      <c r="A33" s="31"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="31"/>
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
     </row>
@@ -4141,7 +4148,7 @@
       <c r="H34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="21" t="s">
+      <c r="A35" s="22" t="s">
         <v>174</v>
       </c>
       <c r="B35" s="3"/>
@@ -4156,7 +4163,7 @@
       <c r="H35" s="3"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="21" t="s">
+      <c r="A36" s="22" t="s">
         <v>175</v>
       </c>
       <c r="B36" s="3"/>
@@ -4171,7 +4178,7 @@
       <c r="H36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="21" t="s">
+      <c r="A37" s="22" t="s">
         <v>223</v>
       </c>
       <c r="B37" s="3"/>
@@ -4201,7 +4208,7 @@
       <c r="H38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21" t="s">
+      <c r="A39" s="22" t="s">
         <v>178</v>
       </c>
       <c r="B39" s="3"/>
@@ -4221,7 +4228,7 @@
       </c>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
-      <c r="D40" s="27" t="n">
+      <c r="D40" s="28" t="n">
         <f aca="false">D38+D39</f>
         <v>359679.06</v>
       </c>
@@ -4412,20 +4419,20 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="24" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$23/60</f>
         <v>25</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="25" t="n">
         <f aca="false">D7*Wyjaśnienia!$B$16</f>
         <v>5500</v>
       </c>
@@ -4436,18 +4443,18 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23" t="n">
+      <c r="C8" s="24"/>
+      <c r="D8" s="24" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$23/60</f>
         <v>40</v>
       </c>
-      <c r="E8" s="24" t="n">
+      <c r="E8" s="25" t="n">
         <f aca="false">D8*Wyjaśnienia!$B$16</f>
         <v>8800</v>
       </c>
@@ -4458,18 +4465,18 @@
       <c r="H8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="22" t="s">
         <v>229</v>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23" t="n">
+      <c r="C9" s="24"/>
+      <c r="D9" s="24" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$23/60</f>
         <v>30</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="25" t="n">
         <f aca="false">D9*Wyjaśnienia!$B$16</f>
         <v>6600</v>
       </c>
@@ -4480,18 +4487,18 @@
       <c r="H9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>231</v>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23" t="n">
+      <c r="C10" s="24"/>
+      <c r="D10" s="24" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$23/60</f>
         <v>20</v>
       </c>
-      <c r="E10" s="24" t="n">
+      <c r="E10" s="25" t="n">
         <f aca="false">D10*Wyjaśnienia!$B$16</f>
         <v>4400</v>
       </c>
@@ -4502,18 +4509,18 @@
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="21" t="s">
+      <c r="A11" s="22" t="s">
         <v>233</v>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23" t="n">
+      <c r="C11" s="24"/>
+      <c r="D11" s="24" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$23/60</f>
         <v>50</v>
       </c>
-      <c r="E11" s="24" t="n">
+      <c r="E11" s="25" t="n">
         <f aca="false">D11*Wyjaśnienia!$B$16</f>
         <v>11000</v>
       </c>
@@ -4529,7 +4536,7 @@
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
-      <c r="D12" s="25" t="n">
+      <c r="D12" s="26" t="n">
         <f aca="false">SUM(D7:D11)</f>
         <v>165</v>
       </c>
@@ -4586,17 +4593,17 @@
       <c r="H15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>236</v>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="25" t="n">
         <f aca="false">Wyjaśnienia!$B$24</f>
         <v>35000</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="25" t="n">
         <f aca="false">B16*C16</f>
         <v>35000</v>
       </c>
@@ -4608,17 +4615,17 @@
       <c r="H16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="B17" s="24" t="n">
+      <c r="B17" s="25" t="n">
         <f aca="false">Wyjaśnienia!$B$25</f>
         <v>4000</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="25" t="n">
         <f aca="false">B17*C17</f>
         <v>4000</v>
       </c>
@@ -4630,18 +4637,18 @@
       <c r="H17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>239</v>
       </c>
-      <c r="B18" s="24" t="n">
+      <c r="B18" s="25" t="n">
         <f aca="false">Wyjaśnienia!$B$26</f>
         <v>7500</v>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="24" t="n">
         <f aca="false">Wyjaśnienia!$B$27</f>
         <v>10</v>
       </c>
-      <c r="D18" s="24" t="n">
+      <c r="D18" s="25" t="n">
         <f aca="false">B18*C18</f>
         <v>75000</v>
       </c>
@@ -4653,17 +4660,17 @@
       <c r="H18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="B19" s="24" t="n">
+      <c r="B19" s="25" t="n">
         <f aca="false">Wyjaśnienia!$B$28</f>
         <v>80000</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="25" t="n">
         <f aca="false">B19*C19</f>
         <v>80000</v>
       </c>
@@ -4675,17 +4682,17 @@
       <c r="H19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>242</v>
       </c>
-      <c r="B20" s="24" t="n">
+      <c r="B20" s="25" t="n">
         <f aca="false">Wyjaśnienia!$B$29</f>
         <v>1200</v>
       </c>
-      <c r="C20" s="22" t="n">
+      <c r="C20" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="25" t="n">
         <f aca="false">B20*C20</f>
         <v>1200</v>
       </c>
@@ -4697,16 +4704,16 @@
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="22" t="s">
         <v>244</v>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="22" t="n">
+      <c r="C21" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="25" t="n">
         <f aca="false">B21*C21</f>
         <v>0</v>
       </c>
@@ -4718,16 +4725,16 @@
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C22" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="25" t="n">
         <f aca="false">B22*C22</f>
         <v>0</v>
       </c>
@@ -4737,16 +4744,16 @@
       <c r="F22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="22" t="s">
         <v>247</v>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C23" s="22" t="n">
+      <c r="C23" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="25" t="n">
         <f aca="false">B23*C23</f>
         <v>0</v>
       </c>
@@ -4758,13 +4765,13 @@
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="29" t="s">
         <v>249</v>
       </c>
       <c r="B24" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="29" t="n">
+      <c r="C24" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8" t="n">
@@ -4774,18 +4781,18 @@
       <c r="E24" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F24" s="29" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="29" t="s">
         <v>252</v>
       </c>
       <c r="B25" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="29" t="n">
+      <c r="C25" s="30" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -4795,7 +4802,7 @@
       <c r="E25" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="F25" s="28"/>
+      <c r="F25" s="29"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
@@ -4809,12 +4816,12 @@
       <c r="H26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="30"/>
-      <c r="B27" s="30"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
-      <c r="F27" s="30"/>
+      <c r="A27" s="31"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
     </row>
@@ -4831,12 +4838,12 @@
       <c r="H28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="s">
+      <c r="A29" s="22" t="s">
         <v>173</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
-      <c r="D29" s="24" t="n">
+      <c r="D29" s="25" t="n">
         <f aca="false">Wyjaśnienia!$B$24+Wyjaśnienia!$B$25</f>
         <v>39000</v>
       </c>
@@ -4846,7 +4853,7 @@
       <c r="H29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="21" t="s">
+      <c r="A30" s="22" t="s">
         <v>174</v>
       </c>
       <c r="B30" s="3"/>
@@ -4861,7 +4868,7 @@
       <c r="H30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="21" t="s">
+      <c r="A31" s="22" t="s">
         <v>254</v>
       </c>
       <c r="B31" s="3"/>
@@ -4876,7 +4883,7 @@
       <c r="H31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="22" t="s">
         <v>176</v>
       </c>
       <c r="B32" s="3"/>
@@ -4906,7 +4913,7 @@
       <c r="H33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="s">
+      <c r="A34" s="22" t="s">
         <v>178</v>
       </c>
       <c r="B34" s="3"/>
@@ -4926,7 +4933,7 @@
       </c>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
-      <c r="D35" s="27" t="n">
+      <c r="D35" s="28" t="n">
         <f aca="false">D33+D34</f>
         <v>313158</v>
       </c>
@@ -5042,44 +5049,44 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>255</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="31" t="s">
         <v>122</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
@@ -5105,13 +5112,13 @@
       <c r="A7" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B7" s="20" t="n">
+      <c r="B7" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="33" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$53/60</f>
         <v>20</v>
       </c>
@@ -5127,11 +5134,11 @@
       <c r="A8" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32" t="n">
+      <c r="C8" s="33"/>
+      <c r="D8" s="33" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$53/60</f>
         <v>30</v>
       </c>
@@ -5147,11 +5154,11 @@
       <c r="A9" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="B9" s="20" t="n">
+      <c r="B9" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32" t="n">
+      <c r="C9" s="33"/>
+      <c r="D9" s="33" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$53/60</f>
         <v>20</v>
       </c>
@@ -5167,11 +5174,11 @@
       <c r="A10" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="21" t="n">
         <v>35</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32" t="n">
+      <c r="C10" s="33"/>
+      <c r="D10" s="33" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$53/60</f>
         <v>35</v>
       </c>
@@ -5187,11 +5194,11 @@
       <c r="A11" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="C11" s="32"/>
-      <c r="D11" s="32" t="n">
+      <c r="C11" s="33"/>
+      <c r="D11" s="33" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$53/60</f>
         <v>15</v>
       </c>
@@ -5207,11 +5214,11 @@
       <c r="A12" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32" t="n">
+      <c r="C12" s="33"/>
+      <c r="D12" s="33" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$53/60</f>
         <v>50</v>
       </c>
@@ -5227,11 +5234,11 @@
       <c r="A13" s="3" t="s">
         <v>267</v>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32" t="n">
+      <c r="C13" s="33"/>
+      <c r="D13" s="33" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$53/60</f>
         <v>20</v>
       </c>
@@ -5247,7 +5254,7 @@
       <c r="A14" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="D14" s="33" t="n">
+      <c r="D14" s="34" t="n">
         <f aca="false">SUM(D7:D13)</f>
         <v>190</v>
       </c>
@@ -5260,14 +5267,14 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="s">
+      <c r="A16" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
@@ -5294,7 +5301,7 @@
         <f aca="false">Wyjaśnienia!$B$54</f>
         <v>90000</v>
       </c>
-      <c r="C18" s="32" t="n">
+      <c r="C18" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="8" t="n">
@@ -5313,7 +5320,7 @@
         <f aca="false">Wyjaśnienia!$B$55</f>
         <v>4000</v>
       </c>
-      <c r="C19" s="32" t="n">
+      <c r="C19" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="8" t="n">
@@ -5332,7 +5339,7 @@
         <f aca="false">Wyjaśnienia!$B$56</f>
         <v>1200</v>
       </c>
-      <c r="C20" s="32" t="n">
+      <c r="C20" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
@@ -5350,7 +5357,7 @@
       <c r="B21" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="32" t="n">
+      <c r="C21" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="8" t="n">
@@ -5368,7 +5375,7 @@
       <c r="B22" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="32" t="n">
+      <c r="C22" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="8" t="n">
@@ -5387,7 +5394,7 @@
         <f aca="false">Wyjaśnienia!$B$61*2</f>
         <v>800</v>
       </c>
-      <c r="C23" s="32" t="n">
+      <c r="C23" s="33" t="n">
         <f aca="false">Wyjaśnienia!$B$60</f>
         <v>10</v>
       </c>
@@ -5407,7 +5414,7 @@
         <f aca="false">Wyjaśnienia!$B$62</f>
         <v>3000</v>
       </c>
-      <c r="C24" s="32" t="n">
+      <c r="C24" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8" t="n">
@@ -5425,7 +5432,7 @@
       <c r="B25" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="32" t="n">
+      <c r="C25" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -5443,7 +5450,7 @@
       <c r="B26" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="32" t="n">
+      <c r="C26" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="8" t="n">
@@ -5461,7 +5468,7 @@
       <c r="B27" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="32" t="n">
+      <c r="C27" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="8" t="n">
@@ -5479,7 +5486,7 @@
       <c r="B28" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C28" s="32" t="n">
+      <c r="C28" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="8" t="n">
@@ -5500,12 +5507,12 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="30"/>
-      <c r="B30" s="30"/>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
+      <c r="A30" s="31"/>
+      <c r="B30" s="31"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
@@ -5566,7 +5573,7 @@
         <v>35530.4</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
         <v>179</v>
       </c>
@@ -5611,669 +5618,669 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="36" t="s">
         <v>286</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="36" t="s">
         <v>287</v>
       </c>
-      <c r="B3" s="35"/>
-      <c r="C3" s="35"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="37" t="s">
         <v>288</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="39" t="s">
         <v>289</v>
       </c>
-      <c r="F6" s="37" t="s">
+      <c r="F6" s="38" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="29" t="s">
         <v>290</v>
       </c>
-      <c r="B7" s="39" t="n">
+      <c r="B7" s="40" t="n">
         <f aca="false">Wyjaśnienia!$B$17</f>
         <v>150</v>
       </c>
-      <c r="F7" s="28" t="s">
+      <c r="F7" s="29" t="s">
         <v>291</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="29" t="s">
         <v>292</v>
       </c>
-      <c r="B8" s="39" t="n">
+      <c r="B8" s="40" t="n">
         <f aca="false">Wyjaśnienia!$B$46</f>
         <v>2</v>
       </c>
-      <c r="F8" s="28" t="s">
+      <c r="F8" s="29" t="s">
         <v>293</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="38" t="s">
         <v>294</v>
       </c>
-      <c r="B9" s="40" t="n">
+      <c r="B9" s="41" t="n">
         <f aca="false">B7*B8</f>
         <v>300</v>
       </c>
-      <c r="F9" s="28" t="s">
+      <c r="F9" s="29" t="s">
         <v>295</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="29" t="s">
         <v>296</v>
       </c>
-      <c r="B10" s="39" t="n">
+      <c r="B10" s="40" t="n">
         <f aca="false">Wyjaśnienia!$B$66</f>
         <v>150</v>
       </c>
-      <c r="F10" s="28" t="s">
+      <c r="F10" s="29" t="s">
         <v>297</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="29" t="s">
         <v>298</v>
       </c>
-      <c r="B11" s="39" t="n">
+      <c r="B11" s="40" t="n">
         <f aca="false">Wyjaśnienia!$B$75</f>
         <v>2</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="29" t="s">
         <v>299</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="s">
+      <c r="A12" s="38" t="s">
         <v>300</v>
       </c>
-      <c r="B12" s="40" t="n">
+      <c r="B12" s="41" t="n">
         <f aca="false">B10*B11</f>
         <v>300</v>
       </c>
-      <c r="F12" s="28" t="s">
+      <c r="F12" s="29" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="37" t="s">
         <v>302</v>
       </c>
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="37"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37" t="s">
+      <c r="A15" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="39" t="s">
         <v>303</v>
       </c>
-      <c r="C15" s="38" t="s">
+      <c r="C15" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="F15" s="37" t="s">
+      <c r="F15" s="38" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="29" t="s">
         <v>304</v>
       </c>
-      <c r="B16" s="41" t="n">
+      <c r="B16" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$48</f>
         <v>2500</v>
       </c>
-      <c r="C16" s="39" t="n">
+      <c r="C16" s="40" t="n">
         <f aca="false">Wyjaśnienia!$B$49</f>
         <v>15</v>
       </c>
-      <c r="D16" s="41" t="n">
+      <c r="D16" s="42" t="n">
         <f aca="false">B16*C16</f>
         <v>37500</v>
       </c>
-      <c r="F16" s="28" t="s">
+      <c r="F16" s="29" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="29" t="s">
         <v>306</v>
       </c>
-      <c r="B17" s="41" t="n">
+      <c r="B17" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$47</f>
         <v>500</v>
       </c>
-      <c r="C17" s="39" t="n">
+      <c r="C17" s="40" t="n">
         <f aca="false">ROUNDUP(B9/100,0)</f>
         <v>3</v>
       </c>
-      <c r="D17" s="41" t="n">
+      <c r="D17" s="42" t="n">
         <f aca="false">B17*C17</f>
         <v>1500</v>
       </c>
-      <c r="F17" s="28" t="s">
+      <c r="F17" s="29" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="29" t="s">
         <v>308</v>
       </c>
-      <c r="B18" s="41" t="n">
+      <c r="B18" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$76</f>
         <v>300</v>
       </c>
-      <c r="C18" s="39" t="n">
+      <c r="C18" s="40" t="n">
         <f aca="false">B12</f>
         <v>300</v>
       </c>
-      <c r="D18" s="41" t="n">
+      <c r="D18" s="42" t="n">
         <f aca="false">B18*C18</f>
         <v>90000</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="29" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37" t="s">
+      <c r="A19" s="38" t="s">
         <v>310</v>
       </c>
-      <c r="D19" s="42" t="n">
+      <c r="D19" s="43" t="n">
         <f aca="false">SUM(D16:D18)</f>
         <v>129000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="37" t="s">
         <v>151</v>
       </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="37" t="s">
+      <c r="A22" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="B22" s="38" t="s">
+      <c r="B22" s="39" t="s">
         <v>152</v>
       </c>
-      <c r="C22" s="38" t="s">
+      <c r="C22" s="39" t="s">
         <v>153</v>
       </c>
-      <c r="D22" s="38" t="s">
+      <c r="D22" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="F22" s="37" t="s">
+      <c r="F22" s="38" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="29" t="s">
         <v>311</v>
       </c>
-      <c r="B23" s="41" t="n">
+      <c r="B23" s="42" t="n">
         <v>2000</v>
       </c>
-      <c r="C23" s="39" t="n">
+      <c r="C23" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="41" t="n">
+      <c r="D23" s="42" t="n">
         <f aca="false">B23*C23</f>
         <v>2000</v>
       </c>
-      <c r="F23" s="28" t="s">
+      <c r="F23" s="29" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="29" t="s">
         <v>313</v>
       </c>
-      <c r="B24" s="41" t="n">
+      <c r="B24" s="42" t="n">
         <v>3000</v>
       </c>
-      <c r="C24" s="39" t="n">
+      <c r="C24" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="41" t="n">
+      <c r="D24" s="42" t="n">
         <f aca="false">B24*C24</f>
         <v>3000</v>
       </c>
-      <c r="F24" s="28" t="s">
+      <c r="F24" s="29" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="29" t="s">
         <v>315</v>
       </c>
-      <c r="B25" s="41" t="n">
+      <c r="B25" s="42" t="n">
         <v>5000</v>
       </c>
-      <c r="C25" s="39" t="n">
+      <c r="C25" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="41" t="n">
+      <c r="D25" s="42" t="n">
         <f aca="false">B25*C25</f>
         <v>5000</v>
       </c>
-      <c r="F25" s="28" t="s">
+      <c r="F25" s="29" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="29" t="s">
         <v>317</v>
       </c>
-      <c r="B26" s="41" t="n">
+      <c r="B26" s="42" t="n">
         <v>4000</v>
       </c>
-      <c r="C26" s="39" t="n">
+      <c r="C26" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="41" t="n">
+      <c r="D26" s="42" t="n">
         <f aca="false">B26*C26</f>
         <v>4000</v>
       </c>
-      <c r="F26" s="28" t="s">
+      <c r="F26" s="29" t="s">
         <v>318</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="37" t="s">
+      <c r="A27" s="38" t="s">
         <v>171</v>
       </c>
-      <c r="D27" s="42" t="n">
+      <c r="D27" s="43" t="n">
         <f aca="false">SUM(D23:D26)</f>
         <v>14000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="36" t="s">
+      <c r="A29" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="B29" s="36"/>
-      <c r="C29" s="36"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="36"/>
-      <c r="F29" s="36"/>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="29" t="s">
         <v>319</v>
       </c>
-      <c r="D30" s="41" t="n">
+      <c r="D30" s="42" t="n">
         <f aca="false">D19</f>
         <v>129000</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="D31" s="41" t="n">
+      <c r="D31" s="42" t="n">
         <f aca="false">D27</f>
         <v>14000</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="29" t="s">
         <v>320</v>
       </c>
-      <c r="D32" s="41" t="n">
+      <c r="D32" s="42" t="n">
         <f aca="false">(D30+D31)*Wyjaśnienia!$B$30</f>
         <v>17160</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="37" t="s">
+      <c r="A33" s="38" t="s">
         <v>177</v>
       </c>
-      <c r="D33" s="42" t="n">
+      <c r="D33" s="43" t="n">
         <f aca="false">SUM(D30:D32)</f>
         <v>160160</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="28" t="s">
+      <c r="A34" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="D34" s="41" t="n">
+      <c r="D34" s="42" t="n">
         <f aca="false">D33*Wyjaśnienia!$B$33</f>
         <v>36836.8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="37" t="s">
+      <c r="A35" s="38" t="s">
         <v>179</v>
       </c>
-      <c r="D35" s="42" t="n">
+      <c r="D35" s="43" t="n">
         <f aca="false">D33+D34</f>
         <v>196996.8</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="36" t="s">
+      <c r="A37" s="37" t="s">
         <v>321</v>
       </c>
-      <c r="B37" s="36"/>
-      <c r="C37" s="36"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="36"/>
+      <c r="B37" s="37"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="37"/>
+      <c r="E37" s="37"/>
+      <c r="F37" s="37"/>
     </row>
     <row r="38" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="35" t="s">
+      <c r="A38" s="36" t="s">
         <v>322</v>
       </c>
-      <c r="B38" s="35"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="35"/>
-      <c r="F38" s="35"/>
+      <c r="B38" s="36"/>
+      <c r="C38" s="36"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="36"/>
+      <c r="F38" s="36"/>
     </row>
     <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="38" t="s">
+      <c r="A39" s="39" t="s">
         <v>323</v>
       </c>
-      <c r="B39" s="38" t="s">
+      <c r="B39" s="39" t="s">
         <v>324</v>
       </c>
-      <c r="C39" s="38" t="s">
+      <c r="C39" s="39" t="s">
         <v>325</v>
       </c>
-      <c r="D39" s="38" t="s">
+      <c r="D39" s="39" t="s">
         <v>326</v>
       </c>
-      <c r="E39" s="38" t="s">
+      <c r="E39" s="39" t="s">
         <v>327</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="39" t="n">
+      <c r="A40" s="40" t="n">
         <v>150</v>
       </c>
-      <c r="B40" s="39" t="n">
+      <c r="B40" s="40" t="n">
         <f aca="false">A40*Wyjaśnienia!$B$46</f>
         <v>300</v>
       </c>
-      <c r="C40" s="39" t="n">
+      <c r="C40" s="40" t="n">
         <f aca="false">ROUNDUP(B40/100,0)</f>
         <v>3</v>
       </c>
-      <c r="D40" s="41" t="n">
+      <c r="D40" s="42" t="n">
         <f aca="false">C40*Wyjaśnienia!$B$47</f>
         <v>1500</v>
       </c>
-      <c r="E40" s="39" t="e">
-        <f aca="false">ROUNDUP(B40/Wyjaśnienia!$B$50,0)</f>
-        <v>#DIV/0!</v>
+      <c r="E40" s="40" t="n">
+        <f aca="false">ROUNDUP(B40*Wyjaśnienia!$B$50/60,0)</f>
+        <v>150</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="39" t="n">
+      <c r="A41" s="40" t="n">
         <v>1000</v>
       </c>
-      <c r="B41" s="39" t="n">
+      <c r="B41" s="40" t="n">
         <f aca="false">A41*Wyjaśnienia!$B$46</f>
         <v>2000</v>
       </c>
-      <c r="C41" s="39" t="n">
+      <c r="C41" s="40" t="n">
         <f aca="false">ROUNDUP(B41/100,0)</f>
         <v>20</v>
       </c>
-      <c r="D41" s="41" t="n">
+      <c r="D41" s="42" t="n">
         <f aca="false">C41*Wyjaśnienia!$B$47</f>
         <v>10000</v>
       </c>
-      <c r="E41" s="39" t="e">
-        <f aca="false">ROUNDUP(B41/Wyjaśnienia!$B$50,0)</f>
-        <v>#DIV/0!</v>
+      <c r="E41" s="40" t="n">
+        <f aca="false">ROUNDUP(B41*Wyjaśnienia!$B$50/60,0)</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="39" t="n">
+      <c r="A42" s="40" t="n">
         <v>10000</v>
       </c>
-      <c r="B42" s="39" t="n">
+      <c r="B42" s="40" t="n">
         <f aca="false">A42*Wyjaśnienia!$B$46</f>
         <v>20000</v>
       </c>
-      <c r="C42" s="39" t="n">
+      <c r="C42" s="40" t="n">
         <f aca="false">ROUNDUP(B42/100,0)</f>
         <v>200</v>
       </c>
-      <c r="D42" s="41" t="n">
+      <c r="D42" s="42" t="n">
         <f aca="false">C42*Wyjaśnienia!$B$47</f>
         <v>100000</v>
       </c>
-      <c r="E42" s="39" t="e">
-        <f aca="false">ROUNDUP(B42/Wyjaśnienia!$B$50,0)</f>
-        <v>#DIV/0!</v>
+      <c r="E42" s="40" t="n">
+        <f aca="false">ROUNDUP(B42*Wyjaśnienia!$B$50/60,0)</f>
+        <v>10000</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="39" t="n">
+      <c r="A43" s="40" t="n">
         <v>100000</v>
       </c>
-      <c r="B43" s="39" t="n">
+      <c r="B43" s="40" t="n">
         <f aca="false">A43*Wyjaśnienia!$B$46</f>
         <v>200000</v>
       </c>
-      <c r="C43" s="39" t="n">
+      <c r="C43" s="40" t="n">
         <f aca="false">ROUNDUP(B43/100,0)</f>
         <v>2000</v>
       </c>
-      <c r="D43" s="41" t="n">
+      <c r="D43" s="42" t="n">
         <f aca="false">C43*Wyjaśnienia!$B$47</f>
         <v>1000000</v>
       </c>
-      <c r="E43" s="39" t="e">
-        <f aca="false">ROUNDUP(B43/Wyjaśnienia!$B$50,0)</f>
-        <v>#DIV/0!</v>
+      <c r="E43" s="40" t="n">
+        <f aca="false">ROUNDUP(B43*Wyjaśnienia!$B$50/60,0)</f>
+        <v>100000</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="39" t="n">
+      <c r="A44" s="40" t="n">
         <v>1000000</v>
       </c>
-      <c r="B44" s="39" t="n">
+      <c r="B44" s="40" t="n">
         <f aca="false">A44*Wyjaśnienia!$B$46</f>
         <v>2000000</v>
       </c>
-      <c r="C44" s="39" t="n">
+      <c r="C44" s="40" t="n">
         <f aca="false">ROUNDUP(B44/100,0)</f>
         <v>20000</v>
       </c>
-      <c r="D44" s="41" t="n">
+      <c r="D44" s="42" t="n">
         <f aca="false">C44*Wyjaśnienia!$B$47</f>
         <v>10000000</v>
       </c>
-      <c r="E44" s="39" t="e">
-        <f aca="false">ROUNDUP(B44/Wyjaśnienia!$B$50,0)</f>
-        <v>#DIV/0!</v>
+      <c r="E44" s="40" t="n">
+        <f aca="false">ROUNDUP(B44*Wyjaśnienia!$B$50/60,0)</f>
+        <v>1000000</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="38" t="s">
+      <c r="A46" s="39" t="s">
         <v>328</v>
       </c>
-      <c r="B46" s="38" t="s">
+      <c r="B46" s="39" t="s">
         <v>329</v>
       </c>
-      <c r="C46" s="38" t="s">
+      <c r="C46" s="39" t="s">
         <v>330</v>
       </c>
-      <c r="D46" s="38" t="s">
+      <c r="D46" s="39" t="s">
         <v>331</v>
       </c>
-      <c r="E46" s="38" t="s">
+      <c r="E46" s="39" t="s">
         <v>332</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="39" t="n">
+      <c r="A47" s="40" t="n">
         <v>30</v>
       </c>
-      <c r="B47" s="39" t="n">
+      <c r="B47" s="40" t="n">
         <f aca="false">A47*Wyjaśnienia!$B$75</f>
         <v>60</v>
       </c>
-      <c r="C47" s="41" t="n">
+      <c r="C47" s="42" t="n">
         <f aca="false">B47*Wyjaśnienia!$B$76</f>
         <v>18000</v>
       </c>
-      <c r="D47" s="39" t="n">
+      <c r="D47" s="40" t="n">
         <f aca="false">B47*2</f>
         <v>120</v>
       </c>
-      <c r="E47" s="39" t="n">
+      <c r="E47" s="40" t="n">
         <f aca="false">ROUNDUP(A47/Wyjaśnienia!$B$77,0)</f>
         <v>3</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="39" t="n">
+      <c r="A48" s="40" t="n">
         <v>150</v>
       </c>
-      <c r="B48" s="39" t="n">
+      <c r="B48" s="40" t="n">
         <f aca="false">A48*Wyjaśnienia!$B$75</f>
         <v>300</v>
       </c>
-      <c r="C48" s="41" t="n">
+      <c r="C48" s="42" t="n">
         <f aca="false">B48*Wyjaśnienia!$B$76</f>
         <v>90000</v>
       </c>
-      <c r="D48" s="39" t="n">
+      <c r="D48" s="40" t="n">
         <f aca="false">B48*2</f>
         <v>600</v>
       </c>
-      <c r="E48" s="39" t="n">
+      <c r="E48" s="40" t="n">
         <f aca="false">ROUNDUP(A48/Wyjaśnienia!$B$77,0)</f>
         <v>15</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="39" t="n">
+      <c r="A49" s="40" t="n">
         <v>500</v>
       </c>
-      <c r="B49" s="39" t="n">
+      <c r="B49" s="40" t="n">
         <f aca="false">A49*Wyjaśnienia!$B$75</f>
         <v>1000</v>
       </c>
-      <c r="C49" s="41" t="n">
+      <c r="C49" s="42" t="n">
         <f aca="false">B49*Wyjaśnienia!$B$76</f>
         <v>300000</v>
       </c>
-      <c r="D49" s="39" t="n">
+      <c r="D49" s="40" t="n">
         <f aca="false">B49*2</f>
         <v>2000</v>
       </c>
-      <c r="E49" s="39" t="n">
+      <c r="E49" s="40" t="n">
         <f aca="false">ROUNDUP(A49/Wyjaśnienia!$B$77,0)</f>
         <v>50</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="39" t="n">
+      <c r="A50" s="40" t="n">
         <v>2000</v>
       </c>
-      <c r="B50" s="39" t="n">
+      <c r="B50" s="40" t="n">
         <f aca="false">A50*Wyjaśnienia!$B$75</f>
         <v>4000</v>
       </c>
-      <c r="C50" s="41" t="n">
+      <c r="C50" s="42" t="n">
         <f aca="false">B50*Wyjaśnienia!$B$76</f>
         <v>1200000</v>
       </c>
-      <c r="D50" s="39" t="n">
+      <c r="D50" s="40" t="n">
         <f aca="false">B50*2</f>
         <v>8000</v>
       </c>
-      <c r="E50" s="39" t="n">
+      <c r="E50" s="40" t="n">
         <f aca="false">ROUNDUP(A50/Wyjaśnienia!$B$77,0)</f>
         <v>200</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="39" t="n">
+      <c r="A51" s="40" t="n">
         <v>10000</v>
       </c>
-      <c r="B51" s="39" t="n">
+      <c r="B51" s="40" t="n">
         <f aca="false">A51*Wyjaśnienia!$B$75</f>
         <v>20000</v>
       </c>
-      <c r="C51" s="41" t="n">
+      <c r="C51" s="42" t="n">
         <f aca="false">B51*Wyjaśnienia!$B$76</f>
         <v>6000000</v>
       </c>
-      <c r="D51" s="39" t="n">
+      <c r="D51" s="40" t="n">
         <f aca="false">B51*2</f>
         <v>40000</v>
       </c>
-      <c r="E51" s="39" t="n">
+      <c r="E51" s="40" t="n">
         <f aca="false">ROUNDUP(A51/Wyjaśnienia!$B$77,0)</f>
         <v>1000</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="35" t="s">
+      <c r="A53" s="36" t="s">
         <v>333</v>
       </c>
-      <c r="B53" s="35"/>
-      <c r="C53" s="35"/>
-      <c r="D53" s="35"/>
-      <c r="E53" s="35"/>
-      <c r="F53" s="35"/>
+      <c r="B53" s="36"/>
+      <c r="C53" s="36"/>
+      <c r="D53" s="36"/>
+      <c r="E53" s="36"/>
+      <c r="F53" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -6315,44 +6322,44 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>334</v>
       </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="31" t="s">
         <v>335</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="s">
+      <c r="A5" s="32" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
@@ -6378,13 +6385,13 @@
       <c r="A7" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="B7" s="20" t="n">
+      <c r="B7" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="33" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$66/60</f>
         <v>30</v>
       </c>
@@ -6400,11 +6407,11 @@
       <c r="A8" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="21" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="32" t="n">
+      <c r="C8" s="21"/>
+      <c r="D8" s="33" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$66/60</f>
         <v>25</v>
       </c>
@@ -6420,11 +6427,11 @@
       <c r="A9" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="B9" s="20" t="n">
+      <c r="B9" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="32" t="n">
+      <c r="C9" s="21"/>
+      <c r="D9" s="33" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$66/60</f>
         <v>60</v>
       </c>
@@ -6440,11 +6447,11 @@
       <c r="A10" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="20"/>
-      <c r="D10" s="32" t="n">
+      <c r="C10" s="21"/>
+      <c r="D10" s="33" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$66/60</f>
         <v>20</v>
       </c>
@@ -6460,11 +6467,11 @@
       <c r="A11" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="32" t="n">
+      <c r="C11" s="21"/>
+      <c r="D11" s="33" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$66/60</f>
         <v>40</v>
       </c>
@@ -6480,11 +6487,11 @@
       <c r="A12" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="C12" s="20"/>
-      <c r="D12" s="32" t="n">
+      <c r="C12" s="21"/>
+      <c r="D12" s="33" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$66/60</f>
         <v>40</v>
       </c>
@@ -6500,11 +6507,11 @@
       <c r="A13" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="21" t="n">
         <v>25</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="32" t="n">
+      <c r="C13" s="21"/>
+      <c r="D13" s="33" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$66/60</f>
         <v>25</v>
       </c>
@@ -6520,11 +6527,11 @@
       <c r="A14" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="B14" s="20" t="n">
+      <c r="B14" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="32" t="n">
+      <c r="C14" s="21"/>
+      <c r="D14" s="33" t="n">
         <f aca="false">B14+C14*Wyjaśnienia!$B$66/60</f>
         <v>50</v>
       </c>
@@ -6540,9 +6547,9 @@
       <c r="A15" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="33" t="n">
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="34" t="n">
         <f aca="false">SUM(D7:D14)</f>
         <v>290</v>
       </c>
@@ -6555,14 +6562,14 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
+      <c r="B17" s="32"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32"/>
+      <c r="F17" s="32"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
@@ -6589,7 +6596,7 @@
         <f aca="false">Wyjaśnienia!$B$67</f>
         <v>180000</v>
       </c>
-      <c r="C19" s="32" t="n">
+      <c r="C19" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="8" t="n">
@@ -6608,7 +6615,7 @@
         <f aca="false">Wyjaśnienia!$B$68</f>
         <v>4000</v>
       </c>
-      <c r="C20" s="32" t="n">
+      <c r="C20" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
@@ -6627,7 +6634,7 @@
         <f aca="false">Wyjaśnienia!$B$69</f>
         <v>1200</v>
       </c>
-      <c r="C21" s="32" t="n">
+      <c r="C21" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="8" t="n">
@@ -6645,7 +6652,7 @@
       <c r="B22" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="32" t="n">
+      <c r="C22" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="8" t="n">
@@ -6663,7 +6670,7 @@
       <c r="B23" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C23" s="32" t="n">
+      <c r="C23" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="8" t="n">
@@ -6681,7 +6688,7 @@
       <c r="B24" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="32" t="n">
+      <c r="C24" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8" t="n">
@@ -6699,7 +6706,7 @@
       <c r="B25" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="32" t="n">
+      <c r="C25" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -6717,7 +6724,7 @@
       <c r="B26" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="32" t="n">
+      <c r="C26" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="8" t="n">
@@ -6735,7 +6742,7 @@
       <c r="B27" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="32" t="n">
+      <c r="C27" s="33" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="8" t="n">
@@ -6746,12 +6753,12 @@
         <v>363</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
         <v>171</v>
       </c>
       <c r="B28" s="8"/>
-      <c r="C28" s="32"/>
+      <c r="C28" s="33"/>
       <c r="D28" s="11" t="n">
         <f aca="false">SUM(D19:D27)</f>
         <v>185200</v>
@@ -6759,14 +6766,14 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="31" t="s">
+      <c r="A30" s="32" t="s">
         <v>172</v>
       </c>
-      <c r="B30" s="31"/>
-      <c r="C30" s="31"/>
-      <c r="D30" s="31"/>
-      <c r="E30" s="31"/>
-      <c r="F30" s="31"/>
+      <c r="B30" s="32"/>
+      <c r="C30" s="32"/>
+      <c r="D30" s="32"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
@@ -6822,7 +6829,7 @@
         <v>59064</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
         <v>179</v>
       </c>
@@ -6947,20 +6954,20 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="22" t="s">
         <v>366</v>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>45</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="24" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$17/60</f>
         <v>45</v>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="25" t="n">
         <f aca="false">D7*Wyjaśnienia!$B$16</f>
         <v>9900</v>
       </c>
@@ -6976,7 +6983,7 @@
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="26" t="n">
         <f aca="false">SUM(D7:D7)</f>
         <v>45</v>
       </c>
@@ -7031,16 +7038,16 @@
       <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>368</v>
       </c>
-      <c r="B12" s="26" t="n">
+      <c r="B12" s="27" t="n">
         <v>8000</v>
       </c>
-      <c r="C12" s="22" t="n">
+      <c r="C12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="24" t="n">
+      <c r="D12" s="25" t="n">
         <f aca="false">B12*C12</f>
         <v>8000</v>
       </c>
@@ -7052,16 +7059,16 @@
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="22" t="s">
         <v>370</v>
       </c>
-      <c r="B13" s="26" t="n">
+      <c r="B13" s="27" t="n">
         <v>1500</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="24" t="n">
+      <c r="D13" s="25" t="n">
         <f aca="false">B13*C13</f>
         <v>1500</v>
       </c>
@@ -7073,16 +7080,16 @@
       <c r="H13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>372</v>
       </c>
-      <c r="B14" s="26" t="n">
+      <c r="B14" s="27" t="n">
         <v>4000</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="25" t="n">
         <f aca="false">B14*C14</f>
         <v>4000</v>
       </c>
@@ -7094,16 +7101,16 @@
       <c r="H14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="22" t="s">
         <v>374</v>
       </c>
-      <c r="B15" s="26" t="n">
+      <c r="B15" s="27" t="n">
         <v>8000</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D15" s="24" t="n">
+      <c r="D15" s="25" t="n">
         <f aca="false">B15*C15</f>
         <v>8000</v>
       </c>
@@ -7115,16 +7122,16 @@
       <c r="H15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>376</v>
       </c>
-      <c r="B16" s="26" t="n">
+      <c r="B16" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="25" t="n">
         <f aca="false">B16*C16</f>
         <v>0</v>
       </c>
@@ -7133,16 +7140,16 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="22" t="s">
         <v>378</v>
       </c>
-      <c r="B17" s="26" t="n">
+      <c r="B17" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C17" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="25" t="n">
         <f aca="false">B17*C17</f>
         <v>0</v>
       </c>
@@ -7151,16 +7158,16 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>380</v>
       </c>
-      <c r="B18" s="26" t="n">
+      <c r="B18" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="22" t="n">
+      <c r="C18" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="24" t="n">
+      <c r="D18" s="25" t="n">
         <f aca="false">B18*C18</f>
         <v>0</v>
       </c>
@@ -7169,16 +7176,16 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="22" t="s">
         <v>382</v>
       </c>
-      <c r="B19" s="26" t="n">
+      <c r="B19" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C19" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="25" t="n">
         <f aca="false">B19*C19</f>
         <v>0</v>
       </c>
@@ -7219,7 +7226,7 @@
       <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="22" t="s">
         <v>174</v>
       </c>
       <c r="D23" s="8" t="n">
@@ -7230,7 +7237,7 @@
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>175</v>
       </c>
       <c r="B24" s="3"/>
@@ -7245,7 +7252,7 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="22" t="s">
         <v>384</v>
       </c>
       <c r="B25" s="3"/>
@@ -7275,7 +7282,7 @@
       <c r="H26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="22" t="s">
         <v>178</v>
       </c>
       <c r="B27" s="3"/>
@@ -7295,7 +7302,7 @@
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="27" t="n">
+      <c r="D28" s="28" t="n">
         <f aca="false">D26+D27</f>
         <v>43256.64</v>
       </c>

</xml_diff>

<commit_message>
Pismo otwiera listą wszystkich spraw, rozdzielone terminy akademii, dwie kwoty przy plakacie wyjaśnione, poprawki językowe i podatkowe
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -1364,7 +1364,7 @@
       <c r="H43" s="47" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="45">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="47" t="inlineStr">
         <is>
           <t>Kolumna "Rok kosztu" w każdej zakładce mówi, na który rok edycji przypada dana pozycja: 2027 to rok naboru, 2028 to ocena jury, nagrody, produkcja antologii, gala i wystawy. Rezerwa i marża dzielą się proporcjonalnie do kosztów danego roku. Podział w tym układzie pokazuje załącznik "Zestawienie zadania".</t>
         </is>
@@ -2452,12 +2452,12 @@
       </c>
       <c r="E25" s="57" t="inlineStr">
         <is>
-          <t>DO USTALENIA - etap przed naborem, osobny od oceny zgłoszeń; obejmuje opisy przedziałów punktowych i przykłady ich zastosowania</t>
+          <t>DO USTALENIA - etap przed naborem, osobny od oceny zgłoszeń; obejmuje opisy przedziałów punktowych i przykłady ich zastosowania Rok kosztu: 2027 - karta oceny powstaje przed otwarciem naboru. Jeżeli zapłata nastąpi później, pozycję trzeba przypisać do roku wypłaty.</t>
         </is>
       </c>
       <c r="F25" s="47" t="n"/>
       <c r="G25" s="82" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="45">
@@ -5296,7 +5296,7 @@
     <row r="41">
       <c r="A41" s="47" t="inlineStr">
         <is>
-          <t>Wystawa w galerii sztuki jest celem, nie zobowiązaniem regulaminowym, i ma własne źródło finansowania. Pozycje poniżej nie wchodzą do sum powyżej i nie są objęte pytaniem do Ministerstwa.</t>
+          <t>Wystawa w galerii sztuki jest celem, nie zobowiązaniem regulaminowym, i ma własne źródło finansowania. Pierwsza pozycja poniżej nie wchodzi do sum powyżej, bo czeka na wycenę. Druga powtarza godziny już policzone w wierszu 13 i również nie jest do sum dodawana - pokazuje tylko, ile z pracy organizatora przypada na część poza pytaniem do MKiDN.</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5373,7 @@
       </c>
       <c r="E44" s="47" t="inlineStr">
         <is>
-          <t>Te same 20 godzin, które są wykazane w wierszu 13 powyżej. Tutaj dla pokazania, ile z pracy organizatora przypada na część poza pytaniem - nie dodawać drugi raz.</t>
+          <t>Te same 20 godzin, które są policzone w wierszu 13 i w sumie głównej. Tutaj wyłącznie dla pokazania, ile z pracy organizatora przypada na część poza pytaniem - nie dodawać drugi raz.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wszystkie cztery kwoty nagród publiczności w zakładce Wyjaśnienia
Kwota dla plebiscytu na rozmowę stała dotąd wprost w Budżecie Nagrody,
a pozostałe trzy w Wyjaśnieniach - szukający pokrętła musiał wiedzieć,
gdzie patrzeć. Nowy wiersz parametrów przesuwa wszystko poniżej, więc
82 odwołania zostały przepisane; sumy wszystkich siedmiu budżetów po
przeliczeniu bez zmian.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -652,7 +652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.68359375" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="45.4" customWidth="1" style="44" min="1" max="1"/>
@@ -1093,35 +1093,25 @@
     <row r="26" ht="15" customHeight="1" s="45">
       <c r="A26" s="47" t="inlineStr">
         <is>
-          <t>Nagranie studyjne - koszt za utwór (netto)</t>
+          <t>Nagrody publiczności rozmowy łącznie (brutto)</t>
         </is>
       </c>
       <c r="B26" s="56" t="n">
-        <v>7500</v>
-      </c>
-      <c r="C26" s="57" t="inlineStr">
-        <is>
-          <t>Środek widełek 5-10 tys. Do wyceny przez Michała Sołtana.</t>
-        </is>
-      </c>
-      <c r="D26" s="47" t="n"/>
-      <c r="E26" s="47" t="n"/>
-      <c r="F26" s="47" t="n"/>
-      <c r="G26" s="47" t="n"/>
-      <c r="H26" s="47" t="n"/>
+        <v>12000</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="45">
       <c r="A27" s="47" t="inlineStr">
         <is>
-          <t>Liczba nagrań studyjnych</t>
+          <t>Nagranie studyjne - koszt za utwór (netto)</t>
         </is>
       </c>
       <c r="B27" s="56" t="n">
-        <v>10</v>
+        <v>7500</v>
       </c>
       <c r="C27" s="57" t="inlineStr">
         <is>
-          <t>Dziesięciu finalistów; te nagrania trafiają na płytę.</t>
+          <t>Środek widełek 5-10 tys. Do wyceny przez Michała Sołtana.</t>
         </is>
       </c>
       <c r="D27" s="47" t="n"/>
@@ -1133,15 +1123,15 @@
     <row r="28" ht="15" customHeight="1" s="45">
       <c r="A28" s="47" t="inlineStr">
         <is>
-          <t>Hymn z teledyskiem (netto)</t>
+          <t>Liczba nagrań studyjnych</t>
         </is>
       </c>
       <c r="B28" s="56" t="n">
-        <v>80000</v>
+        <v>10</v>
       </c>
       <c r="C28" s="57" t="inlineStr">
         <is>
-          <t>Środek widełek 60-100 tys. Górny koniec przy szerszym składzie.</t>
+          <t>Dziesięciu finalistów; te nagrania trafiają na płytę.</t>
         </is>
       </c>
       <c r="D28" s="47" t="n"/>
@@ -1153,15 +1143,15 @@
     <row r="29" ht="15" customHeight="1" s="45">
       <c r="A29" s="47" t="inlineStr">
         <is>
-          <t>Medal zwycięzcy i dyplomy piosenki (netto)</t>
+          <t>Hymn z teledyskiem (netto)</t>
         </is>
       </c>
       <c r="B29" s="56" t="n">
-        <v>1200</v>
+        <v>80000</v>
       </c>
       <c r="C29" s="57" t="inlineStr">
         <is>
-          <t>Ten sam medal co w plebiscycie na rozmowę, cena jak w Budżecie Nagrody.</t>
+          <t>Środek widełek 60-100 tys. Górny koniec przy szerszym składzie.</t>
         </is>
       </c>
       <c r="D29" s="47" t="n"/>
@@ -1173,15 +1163,15 @@
     <row r="30" ht="15" customHeight="1" s="45">
       <c r="A30" s="47" t="inlineStr">
         <is>
-          <t>Rezerwa w Budżecie Nagrody</t>
-        </is>
-      </c>
-      <c r="B30" s="58" t="n">
-        <v>0.12</v>
+          <t>Medal zwycięzcy i dyplomy piosenki (netto)</t>
+        </is>
+      </c>
+      <c r="B30" s="56" t="n">
+        <v>1200</v>
       </c>
       <c r="C30" s="57" t="inlineStr">
         <is>
-          <t>Narzut na nieprzewidziane.</t>
+          <t>Ten sam medal co w plebiscycie na rozmowę, cena jak w Budżecie Nagrody.</t>
         </is>
       </c>
       <c r="D30" s="47" t="n"/>
@@ -1193,15 +1183,15 @@
     <row r="31" ht="15" customHeight="1" s="45">
       <c r="A31" s="47" t="inlineStr">
         <is>
-          <t>Marża w Budżecie Antologii</t>
+          <t>Rezerwa w Budżecie Nagrody</t>
         </is>
       </c>
       <c r="B31" s="58" t="n">
-        <v>0.3</v>
+        <v>0.12</v>
       </c>
       <c r="C31" s="57" t="inlineStr">
         <is>
-          <t>Narzut wynagrodzenia podmiotu, który wykona tę część, liczony od pracy i kosztów twardych. Nie są to środki pozostające u Organizatora ani rezerwa. W kosztorysie dotacyjnym pozycja ta nie wystąpi.</t>
+          <t>Narzut na nieprzewidziane.</t>
         </is>
       </c>
       <c r="D31" s="47" t="n"/>
@@ -1213,15 +1203,15 @@
     <row r="32" ht="15" customHeight="1" s="45">
       <c r="A32" s="47" t="inlineStr">
         <is>
-          <t>Rezerwa w Budżecie Plebiscytu</t>
+          <t>Marża w Budżecie Antologii</t>
         </is>
       </c>
       <c r="B32" s="58" t="n">
-        <v>0.12</v>
+        <v>0.3</v>
       </c>
       <c r="C32" s="57" t="inlineStr">
         <is>
-          <t>Narzut na nieprzewidziane.</t>
+          <t>Narzut wynagrodzenia podmiotu, który wykona tę część, liczony od pracy i kosztów twardych. Nie są to środki pozostające u Organizatora ani rezerwa. W kosztorysie dotacyjnym pozycja ta nie wystąpi.</t>
         </is>
       </c>
       <c r="D32" s="47" t="n"/>
@@ -1233,15 +1223,15 @@
     <row r="33" ht="15" customHeight="1" s="45">
       <c r="A33" s="47" t="inlineStr">
         <is>
-          <t>Stawka VAT</t>
+          <t>Rezerwa w Budżecie Plebiscytu</t>
         </is>
       </c>
       <c r="B33" s="58" t="n">
-        <v>0.23</v>
+        <v>0.12</v>
       </c>
       <c r="C33" s="57" t="inlineStr">
         <is>
-          <t>Dotyczy faktur wystawianych sponsorom.</t>
+          <t>Narzut na nieprzewidziane.</t>
         </is>
       </c>
       <c r="D33" s="47" t="n"/>
@@ -1253,7 +1243,15 @@
     <row r="34" ht="15" customHeight="1" s="45">
       <c r="A34" s="47" t="inlineStr">
         <is>
-          <t>Podatek od nagród (ryczałt)</t>
+          <t>Stawka VAT</t>
+        </is>
+      </c>
+      <c r="B34" s="58" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C34" s="57" t="inlineStr">
+        <is>
+          <t>Dotyczy faktur wystawianych sponsorom.</t>
         </is>
       </c>
       <c r="D34" s="47" t="n"/>
@@ -1263,7 +1261,11 @@
       <c r="H34" s="47" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="45">
-      <c r="A35" s="47" t="n"/>
+      <c r="A35" s="47" t="inlineStr">
+        <is>
+          <t>Podatek od nagród (ryczałt)</t>
+        </is>
+      </c>
       <c r="D35" s="47" t="n"/>
       <c r="E35" s="47" t="n"/>
       <c r="F35" s="47" t="n"/>
@@ -1271,11 +1273,7 @@
       <c r="H35" s="47" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="45">
-      <c r="A36" s="49" t="inlineStr">
-        <is>
-          <t>CZEGO JESZCZE NIE MA</t>
-        </is>
-      </c>
+      <c r="A36" s="47" t="n"/>
       <c r="D36" s="47" t="n"/>
       <c r="E36" s="47" t="n"/>
       <c r="F36" s="47" t="n"/>
@@ -1283,9 +1281,9 @@
       <c r="H36" s="47" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="45">
-      <c r="A37" s="50" t="inlineStr">
-        <is>
-          <t>Honoraria jury we wszystkich plebiscytach - osobno za ocenę zgłoszeń i za etap przygotowania karty oceny</t>
+      <c r="A37" s="49" t="inlineStr">
+        <is>
+          <t>CZEGO JESZCZE NIE MA</t>
         </is>
       </c>
       <c r="D37" s="47" t="n"/>
@@ -1297,7 +1295,7 @@
     <row r="38" ht="15" customHeight="1" s="45">
       <c r="A38" s="50" t="inlineStr">
         <is>
-          <t>Realizacja części artystycznej gali</t>
+          <t>Honoraria jury we wszystkich plebiscytach - osobno za ocenę zgłoszeń i za etap przygotowania karty oceny</t>
         </is>
       </c>
       <c r="D38" s="47" t="n"/>
@@ -1307,9 +1305,9 @@
       <c r="H38" s="47" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="45">
-      <c r="A39" s="48" t="inlineStr">
-        <is>
-          <t>Po wpisaniu tych kwot rosną Budżet Plebiscytu, Budżet Plakatu i Budżet Filmu. W Budżecie Plakatu czekają na wycenę cztery pozycje, w Budżecie Filmu pięć - wszystkie opisane w kolumnie Uwagi.</t>
+      <c r="A39" s="50" t="inlineStr">
+        <is>
+          <t>Realizacja części artystycznej gali</t>
         </is>
       </c>
       <c r="D39" s="47" t="n"/>
@@ -1319,7 +1317,11 @@
       <c r="H39" s="47" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="45">
-      <c r="A40" s="47" t="n"/>
+      <c r="A40" s="48" t="inlineStr">
+        <is>
+          <t>Po wpisaniu tych kwot rosną Budżet Plebiscytu, Budżet Plakatu i Budżet Filmu. W Budżecie Plakatu czekają na wycenę cztery pozycje, w Budżecie Filmu pięć - wszystkie opisane w kolumnie Uwagi.</t>
+        </is>
+      </c>
       <c r="D40" s="47" t="n"/>
       <c r="E40" s="47" t="n"/>
       <c r="F40" s="47" t="n"/>
@@ -1327,11 +1329,7 @@
       <c r="H40" s="47" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="45">
-      <c r="A41" s="49" t="inlineStr">
-        <is>
-          <t>JAK CZYTAĆ BUDŻETY</t>
-        </is>
-      </c>
+      <c r="A41" s="47" t="n"/>
       <c r="D41" s="47" t="n"/>
       <c r="E41" s="47" t="n"/>
       <c r="F41" s="47" t="n"/>
@@ -1339,9 +1337,9 @@
       <c r="H41" s="47" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="45">
-      <c r="A42" s="48" t="inlineStr">
-        <is>
-          <t>Każda z zakładek budżetowych ma ten sam układ: praca organizatora, koszty twarde, podsumowanie.</t>
+      <c r="A42" s="49" t="inlineStr">
+        <is>
+          <t>JAK CZYTAĆ BUDŻETY</t>
         </is>
       </c>
       <c r="D42" s="47" t="n"/>
@@ -1353,7 +1351,7 @@
     <row r="43" ht="15" customHeight="1" s="45">
       <c r="A43" s="48" t="inlineStr">
         <is>
-          <t>W podsumowaniu jest kwota netto, VAT i kwota brutto, którą sponsor widzi na fakturze.</t>
+          <t>Każda z zakładek budżetowych ma ten sam układ: praca organizatora, koszty twarde, podsumowanie.</t>
         </is>
       </c>
       <c r="D43" s="47" t="n"/>
@@ -1363,451 +1361,462 @@
       <c r="H43" s="47" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="45">
-      <c r="A44" s="47" t="inlineStr">
+      <c r="A44" s="48" t="inlineStr">
+        <is>
+          <t>W podsumowaniu jest kwota netto, VAT i kwota brutto, którą sponsor widzi na fakturze.</t>
+        </is>
+      </c>
+      <c r="D44" s="47" t="n"/>
+      <c r="E44" s="47" t="n"/>
+      <c r="F44" s="47" t="n"/>
+      <c r="G44" s="47" t="n"/>
+      <c r="H44" s="47" t="n"/>
+    </row>
+    <row r="45" ht="15" customHeight="1" s="45">
+      <c r="A45" s="47" t="inlineStr">
         <is>
           <t>Kolumna "Rok kosztu" w każdej zakładce mówi, na który rok edycji przypada dana pozycja: 2027 to rok naboru, 2028 to ocena jury, nagrody, produkcja antologii, gala i wystawy. Rezerwa i marża dzielą się proporcjonalnie do kosztów danego roku. Podział w tym układzie pokazuje załącznik "Zestawienie zadania".</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="15" customHeight="1" s="45">
-      <c r="A45" s="59" t="inlineStr">
+    <row r="46" ht="15" customHeight="1" s="45">
+      <c r="A46" s="59" t="inlineStr">
         <is>
           <t>AKADEMIA - PARAMETRY SKALOWANIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="15" customHeight="1" s="45">
-      <c r="A46" s="47" t="inlineStr">
-        <is>
-          <t>Odczytów na jedno zgłoszenie w rundzie pierwszej</t>
-        </is>
-      </c>
-      <c r="B46" s="56" t="n">
-        <v>2</v>
-      </c>
-      <c r="C46" s="47" t="inlineStr">
-        <is>
-          <t>Regulamin § 8: co najmniej dwóch czytelników przy 21-60 zgłoszeniach; powyżej 200 przesiew jednoosobowy z drugim odczytem poniżej progu.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="45">
       <c r="A47" s="47" t="inlineStr">
         <is>
-          <t>Voucher za każde 100 ocenionych rozmów (netto)</t>
-        </is>
-      </c>
-      <c r="B47" s="60" t="n">
-        <v>500</v>
+          <t>Odczytów na jedno zgłoszenie w rundzie pierwszej</t>
+        </is>
+      </c>
+      <c r="B47" s="56" t="n">
+        <v>2</v>
       </c>
       <c r="C47" s="47" t="inlineStr">
         <is>
-          <t>Świadczenie rzeczowe sponsora Akademii. Do ustalenia ze sponsorem.</t>
+          <t>Regulamin § 8: co najmniej dwóch czytelników przy 21-60 zgłoszeniach; powyżej 200 przesiew jednoosobowy z drugim odczytem poniżej progu.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="45">
       <c r="A48" s="47" t="inlineStr">
         <is>
-          <t>Honorarium podstawowe czytelnika (netto)</t>
+          <t>Voucher za każde 100 ocenionych rozmów (netto)</t>
         </is>
       </c>
       <c r="B48" s="60" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="C48" s="47" t="inlineStr">
         <is>
-          <t>Przeniesione z Budżetu Nagrody. Voucher jest dodatkiem, nie zamiennikiem.</t>
+          <t>Świadczenie rzeczowe sponsora Akademii. Do ustalenia ze sponsorem.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="45">
       <c r="A49" s="47" t="inlineStr">
         <is>
-          <t>Liczba czytelników w pierwszej edycji</t>
-        </is>
-      </c>
-      <c r="B49" s="56" t="n">
-        <v>15</v>
+          <t>Honorarium podstawowe czytelnika (netto)</t>
+        </is>
+      </c>
+      <c r="B49" s="60" t="n">
+        <v>2500</v>
       </c>
       <c r="C49" s="47" t="inlineStr">
         <is>
-          <t>Maksymalnie 20 zgłoszeń na czytelnika (regulamin § 8).</t>
+          <t>Przeniesione z Budżetu Nagrody. Voucher jest dodatkiem, nie zamiennikiem.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="45">
       <c r="A50" s="47" t="inlineStr">
         <is>
+          <t>Liczba czytelników w pierwszej edycji</t>
+        </is>
+      </c>
+      <c r="B50" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="C50" s="47" t="inlineStr">
+        <is>
+          <t>Maksymalnie 20 zgłoszeń na czytelnika (regulamin § 8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15" customHeight="1" s="45">
+      <c r="A51" s="47" t="inlineStr">
+        <is>
           <t>Czas na jeden odczyt rozmowy wraz z kartą oceny (minut)</t>
         </is>
       </c>
-      <c r="B50" s="61" t="n">
+      <c r="B51" s="61" t="n">
         <v>30</v>
       </c>
     </row>
-    <row r="51" ht="15" customHeight="1" s="45"/>
-    <row r="52" ht="15" customHeight="1" s="45">
-      <c r="A52" s="62" t="inlineStr">
+    <row r="52" ht="15" customHeight="1" s="45"/>
+    <row r="53" ht="15" customHeight="1" s="45">
+      <c r="A53" s="62" t="inlineStr">
         <is>
           <t>PLAKAT - PARAMETRY</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="15" customHeight="1" s="45">
-      <c r="A53" s="44" t="inlineStr">
-        <is>
-          <t>Liczba zgłoszeń plakatów</t>
-        </is>
-      </c>
-      <c r="B53" s="63" t="n">
-        <v>150</v>
-      </c>
-      <c r="C53" s="44" t="inlineStr">
-        <is>
-          <t>Wpływa na koszt kontroli formalnej.</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="45">
       <c r="A54" s="44" t="inlineStr">
         <is>
-          <t>Nagrody plakatu łącznie (brutto)</t>
-        </is>
-      </c>
-      <c r="B54" s="60" t="n">
-        <v>90000</v>
+          <t>Liczba zgłoszeń plakatów</t>
+        </is>
+      </c>
+      <c r="B54" s="63" t="n">
+        <v>150</v>
       </c>
       <c r="C54" s="44" t="inlineStr">
         <is>
-          <t>50 tys. + 25 tys. + 15 tys. dla czołowej trójki.</t>
+          <t>Wpływa na koszt kontroli formalnej.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="45">
       <c r="A55" s="44" t="inlineStr">
         <is>
-          <t>Nagrody publiczności plakatu łącznie (brutto)</t>
+          <t>Nagrody plakatu łącznie (brutto)</t>
         </is>
       </c>
       <c r="B55" s="60" t="n">
-        <v>12000</v>
+        <v>90000</v>
       </c>
       <c r="C55" s="44" t="inlineStr">
         <is>
-          <t>3 000 zł dla pracy z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych plakatów (§ 12 ust. 6).</t>
+          <t>50 tys. + 25 tys. + 15 tys. dla czołowej trójki.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="45">
       <c r="A56" s="44" t="inlineStr">
         <is>
-          <t>Medal zwycięzcy i dyplomy plakatu (netto)</t>
+          <t>Nagrody publiczności plakatu łącznie (brutto)</t>
         </is>
       </c>
       <c r="B56" s="60" t="n">
-        <v>1200</v>
+        <v>12000</v>
       </c>
       <c r="C56" s="44" t="inlineStr">
         <is>
-          <t>Ten sam medal co w plebiscycie na rozmowę, cena jak w Budżecie Nagrody.</t>
+          <t>3 000 zł dla pracy z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych plakatów (§ 12 ust. 6).</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="45">
       <c r="A57" s="44" t="inlineStr">
         <is>
-          <t>Liczba jurorów plakatu</t>
-        </is>
-      </c>
-      <c r="B57" s="63" t="n">
-        <v>5</v>
+          <t>Medal zwycięzcy i dyplomy plakatu (netto)</t>
+        </is>
+      </c>
+      <c r="B57" s="60" t="n">
+        <v>1200</v>
       </c>
       <c r="C57" s="44" t="inlineStr">
         <is>
-          <t>Kotwica, nie decyzja: pozycja honorariów w Budżecie Plakatu stoi na zerze jako DO USTALENIA, do rozmowy z przewodniczącym jury.</t>
+          <t>Ten sam medal co w plebiscycie na rozmowę, cena jak w Budżecie Nagrody.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="45">
       <c r="A58" s="44" t="inlineStr">
         <is>
-          <t>Godzin oceny na jurora</t>
+          <t>Liczba jurorów plakatu</t>
         </is>
       </c>
       <c r="B58" s="63" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C58" s="44" t="inlineStr">
         <is>
-          <t>Oglądanie reprodukcji jest szybsze niż odsłuch utworów; przy jury przyjęto 15 h.</t>
+          <t>Kotwica, nie decyzja: pozycja honorariów w Budżecie Plakatu stoi na zerze jako DO USTALENIA, do rozmowy z przewodniczącym jury.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="45">
       <c r="A59" s="44" t="inlineStr">
         <is>
-          <t>Stawka jury plakatu za godzinę (netto)</t>
-        </is>
-      </c>
-      <c r="B59" s="60" t="n">
-        <v>290</v>
+          <t>Godzin oceny na jurora</t>
+        </is>
+      </c>
+      <c r="B59" s="63" t="n">
+        <v>10</v>
       </c>
       <c r="C59" s="44" t="inlineStr">
         <is>
-          <t>Stawka przyjęta dla jury oceniającej rozmowy.</t>
+          <t>Oglądanie reprodukcji jest szybsze niż odsłuch utworów; przy jury przyjęto 15 h.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="45">
       <c r="A60" s="44" t="inlineStr">
         <is>
-          <t>Liczba prac finałowych</t>
-        </is>
-      </c>
-      <c r="B60" s="63" t="n">
-        <v>10</v>
+          <t>Stawka jury plakatu za godzinę (netto)</t>
+        </is>
+      </c>
+      <c r="B60" s="60" t="n">
+        <v>290</v>
       </c>
       <c r="C60" s="44" t="inlineStr">
         <is>
-          <t>Dziesiątka, której oryginały jadą na wystawę.</t>
+          <t>Stawka przyjęta dla jury oceniającej rozmowy.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="45">
       <c r="A61" s="44" t="inlineStr">
         <is>
-          <t>Transport jednej pracy w jedną stronę (netto)</t>
-        </is>
-      </c>
-      <c r="B61" s="60" t="n">
-        <v>400</v>
+          <t>Liczba prac finałowych</t>
+        </is>
+      </c>
+      <c r="B61" s="63" t="n">
+        <v>10</v>
       </c>
       <c r="C61" s="44" t="inlineStr">
         <is>
-          <t>Szacunek, nie oferta. Format do 150 cm przekracza limity standardowych przesyłek.</t>
+          <t>Dziesiątka, której oryginały jadą na wystawę.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="45">
       <c r="A62" s="44" t="inlineStr">
         <is>
-          <t>Ubezpieczenie prac na czas wystawy (netto)</t>
+          <t>Transport jednej pracy w jedną stronę (netto)</t>
         </is>
       </c>
       <c r="B62" s="60" t="n">
-        <v>3000</v>
+        <v>400</v>
       </c>
       <c r="C62" s="44" t="inlineStr">
         <is>
-          <t>Szacunek przy sumie deklarowanej rzędu 100 tys. zł dla całej dziesiątki.</t>
+          <t>Szacunek, nie oferta. Format do 150 cm przekracza limity standardowych przesyłek.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="45">
       <c r="A63" s="44" t="inlineStr">
         <is>
+          <t>Ubezpieczenie prac na czas wystawy (netto)</t>
+        </is>
+      </c>
+      <c r="B63" s="60" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C63" s="44" t="inlineStr">
+        <is>
+          <t>Szacunek przy sumie deklarowanej rzędu 100 tys. zł dla całej dziesiątki.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15" customHeight="1" s="45">
+      <c r="A64" s="44" t="inlineStr">
+        <is>
           <t>Rezerwa w Budżecie Plakatu</t>
         </is>
       </c>
-      <c r="B63" s="60" t="n">
+      <c r="B64" s="60" t="n">
         <v>0.12</v>
       </c>
-      <c r="C63" s="44" t="inlineStr">
+      <c r="C64" s="44" t="inlineStr">
         <is>
           <t>Narzut na nieprzewidziane.</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="15" customHeight="1" s="45"/>
-    <row r="65" ht="15" customHeight="1" s="45">
-      <c r="A65" s="62" t="inlineStr">
+    <row r="65" ht="15" customHeight="1" s="45"/>
+    <row r="66" ht="15" customHeight="1" s="45">
+      <c r="A66" s="62" t="inlineStr">
         <is>
           <t>FILM - PARAMETRY</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15" customHeight="1" s="45">
-      <c r="A66" s="44" t="inlineStr">
-        <is>
-          <t>Liczba zgłoszeń filmów</t>
-        </is>
-      </c>
-      <c r="B66" s="56" t="n">
-        <v>150</v>
-      </c>
-      <c r="C66" s="44" t="inlineStr">
-        <is>
-          <t>Wpływa na koszt kontroli formalnej i na wielkość Akademii filmu.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="45">
       <c r="A67" s="44" t="inlineStr">
         <is>
-          <t>Nagrody filmu łącznie (brutto)</t>
+          <t>Liczba zgłoszeń filmów</t>
         </is>
       </c>
       <c r="B67" s="56" t="n">
-        <v>180000</v>
+        <v>150</v>
       </c>
       <c r="C67" s="44" t="inlineStr">
         <is>
-          <t>100 tys. + 50 tys. + 30 tys. dla czołowej trójki. Siedem wyróżnień nie jest pieniężnych.</t>
+          <t>Wpływa na koszt kontroli formalnej i na wielkość Akademii filmu.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="45">
       <c r="A68" s="44" t="inlineStr">
         <is>
-          <t>Nagrody publiczności filmu łącznie (brutto)</t>
+          <t>Nagrody filmu łącznie (brutto)</t>
         </is>
       </c>
       <c r="B68" s="56" t="n">
-        <v>12000</v>
+        <v>180000</v>
       </c>
       <c r="C68" s="44" t="inlineStr">
         <is>
-          <t>3 000 zł dla filmu z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych filmów (§ 11a ust. 5).</t>
+          <t>100 tys. + 50 tys. + 30 tys. dla czołowej trójki. Siedem wyróżnień nie jest pieniężnych.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="45">
       <c r="A69" s="44" t="inlineStr">
         <is>
-          <t>Medal zwycięzcy i dyplomy filmu (netto)</t>
+          <t>Nagrody publiczności filmu łącznie (brutto)</t>
         </is>
       </c>
       <c r="B69" s="56" t="n">
-        <v>1200</v>
+        <v>12000</v>
       </c>
       <c r="C69" s="44" t="inlineStr">
         <is>
-          <t>Ten sam medal co w pozostałych plebiscytach; dyplomy dla dziesięciu finalistów.</t>
+          <t>3 000 zł dla filmu z największą liczbą głosów oraz 1 000 zł jako Nagroda dla publicznych ocen zgłoszonych filmów (§ 11a ust. 5).</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="45">
       <c r="A70" s="44" t="inlineStr">
         <is>
-          <t>Liczba filmów finałowych</t>
+          <t>Medal zwycięzcy i dyplomy filmu (netto)</t>
         </is>
       </c>
       <c r="B70" s="56" t="n">
-        <v>10</v>
+        <v>1200</v>
       </c>
       <c r="C70" s="44" t="inlineStr">
         <is>
-          <t>Dziesięciu finalistów: trójka z nagrodami pieniężnymi i siedem wyróżnień. Minutowe skróty na gali dostaje pięć najwyżej ocenionych.</t>
+          <t>Ten sam medal co w pozostałych plebiscytach; dyplomy dla dziesięciu finalistów.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="45">
       <c r="A71" s="44" t="inlineStr">
         <is>
-          <t>Liczba jurorów filmu</t>
+          <t>Liczba filmów finałowych</t>
         </is>
       </c>
       <c r="B71" s="56" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C71" s="44" t="inlineStr">
         <is>
-          <t>Kotwica, nie decyzja: pozycja honorariów w Budżecie Filmu stoi na zerze jako DO USTALENIA.</t>
+          <t>Dziesięciu finalistów: trójka z nagrodami pieniężnymi i siedem wyróżnień. Minutowe skróty na gali dostaje pięć najwyżej ocenionych.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="45">
       <c r="A72" s="44" t="inlineStr">
         <is>
-          <t>Godzin oceny na jurora filmu</t>
+          <t>Liczba jurorów filmu</t>
         </is>
       </c>
       <c r="B72" s="56" t="n">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="C72" s="44" t="inlineStr">
         <is>
-          <t>Akademia przekazuje jury nie więcej niż dwadzieścia filmów (§ 8 ust. 5a); dwadzieścia filmów po najwyżej 90 minut to 30 godzin samego oglądania, reszta na karty oceny, obrady i werdykt.</t>
+          <t>Kotwica, nie decyzja: pozycja honorariów w Budżecie Filmu stoi na zerze jako DO USTALENIA.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="45">
       <c r="A73" s="44" t="inlineStr">
         <is>
-          <t>Stawka jury filmu za godzinę (netto)</t>
+          <t>Godzin oceny na jurora filmu</t>
         </is>
       </c>
       <c r="B73" s="56" t="n">
-        <v>290</v>
+        <v>40</v>
       </c>
       <c r="C73" s="44" t="inlineStr">
         <is>
-          <t>Stawka przyjęta dla jury oceniającej rozmowy.</t>
+          <t>Akademia przekazuje jury nie więcej niż dwadzieścia filmów (§ 8 ust. 5a); dwadzieścia filmów po najwyżej 90 minut to 30 godzin samego oglądania, reszta na karty oceny, obrady i werdykt.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="45">
       <c r="A74" s="44" t="inlineStr">
         <is>
-          <t>Rezerwa w Budżecie Filmu</t>
+          <t>Stawka jury filmu za godzinę (netto)</t>
         </is>
       </c>
       <c r="B74" s="56" t="n">
-        <v>0.12</v>
+        <v>290</v>
       </c>
       <c r="C74" s="44" t="inlineStr">
         <is>
-          <t>Narzut na nieprzewidziane, jak w pozostałych budżetach.</t>
+          <t>Stawka przyjęta dla jury oceniającej rozmowy.</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="45">
       <c r="A75" s="44" t="inlineStr">
         <is>
-          <t>Obejrzeń jednego filmu w Akademii</t>
+          <t>Rezerwa w Budżecie Filmu</t>
         </is>
       </c>
       <c r="B75" s="56" t="n">
-        <v>2</v>
+        <v>0.12</v>
       </c>
       <c r="C75" s="44" t="inlineStr">
         <is>
-          <t>Dwa niezależne obejrzenia, analogicznie do dwóch odczytów rozmowy.</t>
+          <t>Narzut na nieprzewidziane, jak w pozostałych budżetach.</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="45">
       <c r="A76" s="44" t="inlineStr">
         <is>
-          <t>Honorarium za obejrzenie jednego filmu (netto)</t>
+          <t>Obejrzeń jednego filmu w Akademii</t>
         </is>
       </c>
       <c r="B76" s="56" t="n">
-        <v>300</v>
+        <v>2</v>
       </c>
       <c r="C76" s="44" t="inlineStr">
         <is>
-          <t>Film do 90 minut plus karta oceny to około 2 godzin pracy. Ustalenie z 26.10.2026.</t>
+          <t>Dwa niezależne obejrzenia, analogicznie do dwóch odczytów rozmowy.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="45">
       <c r="A77" s="44" t="inlineStr">
         <is>
+          <t>Honorarium za obejrzenie jednego filmu (netto)</t>
+        </is>
+      </c>
+      <c r="B77" s="56" t="n">
+        <v>300</v>
+      </c>
+      <c r="C77" s="44" t="inlineStr">
+        <is>
+          <t>Film do 90 minut plus karta oceny to około 2 godzin pracy. Ustalenie z 26.10.2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="15" customHeight="1" s="45">
+      <c r="A78" s="44" t="inlineStr">
+        <is>
           <t>Maksimum filmów na jednego oceniającego</t>
         </is>
       </c>
-      <c r="B77" s="56" t="n">
+      <c r="B78" s="56" t="n">
         <v>10</v>
       </c>
-      <c r="C77" s="44" t="inlineStr">
+      <c r="C78" s="44" t="inlineStr">
         <is>
           <t>Dziesięć filmów to około 20 godzin oglądania. Wyznacza, ilu ludzi trzeba przy danym wolumenie.</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" s="45"/>
     <row r="79" ht="15" customHeight="1" s="45"/>
     <row r="80" ht="15" customHeight="1" s="45"/>
     <row r="81" ht="15" customHeight="1" s="45"/>
@@ -2484,8 +2493,9 @@
           <t>Nagrody publiczności (brutto)</t>
         </is>
       </c>
-      <c r="B27" s="70" t="n">
-        <v>12000</v>
+      <c r="B27" s="70">
+        <f>Wyjaśnienia!$B$26</f>
+        <v/>
       </c>
       <c r="C27" s="65" t="n">
         <v>1</v>
@@ -2496,7 +2506,7 @@
       </c>
       <c r="E27" s="57" t="inlineStr">
         <is>
-          <t>10 000 zł dla zgłoszenia z największą liczbą głosów oraz 2 000 zł za najlepsze uzasadnienie oddanego głosu; kwotę ustawia się tutaj, w pozostałych plebiscytach w zakładce Wyjaśnienia</t>
+          <t>10 000 zł dla zgłoszenia z największą liczbą głosów oraz 2 000 zł za najlepsze uzasadnienie oddanego głosu</t>
         </is>
       </c>
       <c r="F27" s="47" t="n"/>
@@ -2640,7 +2650,7 @@
         </is>
       </c>
       <c r="D36" s="47">
-        <f>(D34+D35-D27-D29)*Wyjaśnienia!$B$30</f>
+        <f>(D34+D35-D27-D29)*Wyjaśnienia!$B$31</f>
         <v/>
       </c>
       <c r="E36" s="44" t="inlineStr">
@@ -2675,7 +2685,7 @@
       <c r="B38" s="47" t="n"/>
       <c r="C38" s="47" t="n"/>
       <c r="D38" s="52">
-        <f>D37*Wyjaśnienia!$B$33</f>
+        <f>D37*Wyjaśnienia!$B$34</f>
         <v/>
       </c>
       <c r="E38" s="47" t="n"/>
@@ -3602,7 +3612,7 @@
       <c r="B37" s="47" t="n"/>
       <c r="C37" s="47" t="n"/>
       <c r="D37" s="52">
-        <f>(D35+D36)*Wyjaśnienia!$B$31</f>
+        <f>(D35+D36)*Wyjaśnienia!$B$32</f>
         <v/>
       </c>
       <c r="E37" s="47" t="n"/>
@@ -3634,7 +3644,7 @@
       <c r="B39" s="47" t="n"/>
       <c r="C39" s="47" t="n"/>
       <c r="D39" s="52">
-        <f>D38*Wyjaśnienia!$B$33</f>
+        <f>D38*Wyjaśnienia!$B$34</f>
         <v/>
       </c>
       <c r="E39" s="47" t="n"/>
@@ -4114,11 +4124,11 @@
         </is>
       </c>
       <c r="B18" s="67">
-        <f>Wyjaśnienia!$B$26</f>
+        <f>Wyjaśnienia!$B$27</f>
         <v/>
       </c>
       <c r="C18" s="66">
-        <f>Wyjaśnienia!$B$27</f>
+        <f>Wyjaśnienia!$B$28</f>
         <v/>
       </c>
       <c r="D18" s="67">
@@ -4143,7 +4153,7 @@
         </is>
       </c>
       <c r="B19" s="67">
-        <f>Wyjaśnienia!$B$28</f>
+        <f>Wyjaśnienia!$B$29</f>
         <v/>
       </c>
       <c r="C19" s="65" t="n">
@@ -4171,7 +4181,7 @@
         </is>
       </c>
       <c r="B20" s="67">
-        <f>Wyjaśnienia!$B$29</f>
+        <f>Wyjaśnienia!$B$30</f>
         <v/>
       </c>
       <c r="C20" s="65" t="n">
@@ -4409,7 +4419,7 @@
       <c r="B32" s="47" t="n"/>
       <c r="C32" s="47" t="n"/>
       <c r="D32" s="52">
-        <f>(D30+D31)*Wyjaśnienia!$B$32</f>
+        <f>(D30+D31)*Wyjaśnienia!$B$33</f>
         <v/>
       </c>
       <c r="E32" s="47" t="n"/>
@@ -4441,7 +4451,7 @@
       <c r="B34" s="47" t="n"/>
       <c r="C34" s="47" t="n"/>
       <c r="D34" s="52">
-        <f>D33*Wyjaśnienia!$B$33</f>
+        <f>D33*Wyjaśnienia!$B$34</f>
         <v/>
       </c>
       <c r="E34" s="47" t="n"/>
@@ -4646,7 +4656,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="68">
-        <f>B7+C7*Wyjaśnienia!$B$53/60</f>
+        <f>B7+C7*Wyjaśnienia!$B$54/60</f>
         <v/>
       </c>
       <c r="E7" s="52">
@@ -4673,7 +4683,7 @@
       </c>
       <c r="C8" s="68" t="n"/>
       <c r="D8" s="68">
-        <f>B8+C8*Wyjaśnienia!$B$53/60</f>
+        <f>B8+C8*Wyjaśnienia!$B$54/60</f>
         <v/>
       </c>
       <c r="E8" s="52">
@@ -4700,7 +4710,7 @@
       </c>
       <c r="C9" s="68" t="n"/>
       <c r="D9" s="68">
-        <f>B9+C9*Wyjaśnienia!$B$53/60</f>
+        <f>B9+C9*Wyjaśnienia!$B$54/60</f>
         <v/>
       </c>
       <c r="E9" s="52">
@@ -4727,7 +4737,7 @@
       </c>
       <c r="C10" s="68" t="n"/>
       <c r="D10" s="68">
-        <f>B10+C10*Wyjaśnienia!$B$53/60</f>
+        <f>B10+C10*Wyjaśnienia!$B$54/60</f>
         <v/>
       </c>
       <c r="E10" s="52">
@@ -4754,7 +4764,7 @@
       </c>
       <c r="C11" s="68" t="n"/>
       <c r="D11" s="68">
-        <f>B11+C11*Wyjaśnienia!$B$53/60</f>
+        <f>B11+C11*Wyjaśnienia!$B$54/60</f>
         <v/>
       </c>
       <c r="E11" s="52">
@@ -4781,7 +4791,7 @@
       </c>
       <c r="C12" s="68" t="n"/>
       <c r="D12" s="68">
-        <f>B12+C12*Wyjaśnienia!$B$53/60</f>
+        <f>B12+C12*Wyjaśnienia!$B$54/60</f>
         <v/>
       </c>
       <c r="E12" s="52">
@@ -4808,7 +4818,7 @@
       </c>
       <c r="C13" s="68" t="n"/>
       <c r="D13" s="68">
-        <f>B13+C13*Wyjaśnienia!$B$53/60</f>
+        <f>B13+C13*Wyjaśnienia!$B$54/60</f>
         <v/>
       </c>
       <c r="E13" s="52">
@@ -4890,7 +4900,7 @@
         </is>
       </c>
       <c r="B18" s="52">
-        <f>Wyjaśnienia!$B$54</f>
+        <f>Wyjaśnienia!$B$55</f>
         <v/>
       </c>
       <c r="C18" s="68" t="n">
@@ -4916,7 +4926,7 @@
         </is>
       </c>
       <c r="B19" s="52">
-        <f>Wyjaśnienia!$B$55</f>
+        <f>Wyjaśnienia!$B$56</f>
         <v/>
       </c>
       <c r="C19" s="68" t="n">
@@ -4942,7 +4952,7 @@
         </is>
       </c>
       <c r="B20" s="52">
-        <f>Wyjaśnienia!$B$56</f>
+        <f>Wyjaśnienia!$B$57</f>
         <v/>
       </c>
       <c r="C20" s="68" t="n">
@@ -5018,11 +5028,11 @@
         </is>
       </c>
       <c r="B23" s="52">
-        <f>Wyjaśnienia!$B$61*2</f>
+        <f>Wyjaśnienia!$B$62*2</f>
         <v/>
       </c>
       <c r="C23" s="68">
-        <f>Wyjaśnienia!$B$60</f>
+        <f>Wyjaśnienia!$B$61</f>
         <v/>
       </c>
       <c r="D23" s="52">
@@ -5045,7 +5055,7 @@
         </is>
       </c>
       <c r="B24" s="52">
-        <f>Wyjaśnienia!$B$62</f>
+        <f>Wyjaśnienia!$B$63</f>
         <v/>
       </c>
       <c r="C24" s="68" t="n">
@@ -5192,7 +5202,7 @@
         </is>
       </c>
       <c r="D32" s="52">
-        <f>Wyjaśnienia!$B$54+Wyjaśnienia!$B$55</f>
+        <f>Wyjaśnienia!$B$55+Wyjaśnienia!$B$56</f>
         <v/>
       </c>
     </row>
@@ -5225,7 +5235,7 @@
         </is>
       </c>
       <c r="D35" s="52">
-        <f>(D33+D34)*Wyjaśnienia!$B$63</f>
+        <f>(D33+D34)*Wyjaśnienia!$B$64</f>
         <v/>
       </c>
     </row>
@@ -5247,7 +5257,7 @@
         </is>
       </c>
       <c r="D37" s="52">
-        <f>D36*Wyjaśnienia!$B$33</f>
+        <f>D36*Wyjaśnienia!$B$34</f>
         <v/>
       </c>
     </row>
@@ -5454,7 +5464,7 @@
         </is>
       </c>
       <c r="B8" s="78">
-        <f>Wyjaśnienia!$B$46</f>
+        <f>Wyjaśnienia!$B$47</f>
         <v/>
       </c>
       <c r="F8" s="72" t="inlineStr">
@@ -5486,7 +5496,7 @@
         </is>
       </c>
       <c r="B10" s="78">
-        <f>Wyjaśnienia!$B$66</f>
+        <f>Wyjaśnienia!$B$67</f>
         <v/>
       </c>
       <c r="F10" s="72" t="inlineStr">
@@ -5502,7 +5512,7 @@
         </is>
       </c>
       <c r="B11" s="78">
-        <f>Wyjaśnienia!$B$75</f>
+        <f>Wyjaśnienia!$B$76</f>
         <v/>
       </c>
       <c r="F11" s="72" t="inlineStr">
@@ -5573,11 +5583,11 @@
         </is>
       </c>
       <c r="B16" s="80">
-        <f>Wyjaśnienia!$B$48</f>
+        <f>Wyjaśnienia!$B$49</f>
         <v/>
       </c>
       <c r="C16" s="78">
-        <f>Wyjaśnienia!$B$49</f>
+        <f>Wyjaśnienia!$B$50</f>
         <v/>
       </c>
       <c r="D16" s="80">
@@ -5600,7 +5610,7 @@
         </is>
       </c>
       <c r="B17" s="80">
-        <f>Wyjaśnienia!$B$47</f>
+        <f>Wyjaśnienia!$B$48</f>
         <v/>
       </c>
       <c r="C17" s="78">
@@ -5627,7 +5637,7 @@
         </is>
       </c>
       <c r="B18" s="80">
-        <f>Wyjaśnienia!$B$76</f>
+        <f>Wyjaśnienia!$B$77</f>
         <v/>
       </c>
       <c r="C18" s="78">
@@ -5844,7 +5854,7 @@
         </is>
       </c>
       <c r="D32" s="80">
-        <f>(D30+D31)*Wyjaśnienia!$B$30</f>
+        <f>(D30+D31)*Wyjaśnienia!$B$31</f>
         <v/>
       </c>
     </row>
@@ -5866,7 +5876,7 @@
         </is>
       </c>
       <c r="D34" s="80">
-        <f>D33*Wyjaśnienia!$B$33</f>
+        <f>D33*Wyjaśnienia!$B$34</f>
         <v/>
       </c>
     </row>
@@ -5927,7 +5937,7 @@
         <v>150</v>
       </c>
       <c r="B40" s="78">
-        <f>A40*Wyjaśnienia!$B$46</f>
+        <f>A40*Wyjaśnienia!$B$47</f>
         <v/>
       </c>
       <c r="C40" s="78">
@@ -5935,11 +5945,11 @@
         <v/>
       </c>
       <c r="D40" s="80">
-        <f>C40*Wyjaśnienia!$B$47</f>
+        <f>C40*Wyjaśnienia!$B$48</f>
         <v/>
       </c>
       <c r="E40" s="78">
-        <f>ROUNDUP(B40*Wyjaśnienia!$B$50/60,0)</f>
+        <f>ROUNDUP(B40*Wyjaśnienia!$B$51/60,0)</f>
         <v/>
       </c>
     </row>
@@ -5948,7 +5958,7 @@
         <v>1000</v>
       </c>
       <c r="B41" s="78">
-        <f>A41*Wyjaśnienia!$B$46</f>
+        <f>A41*Wyjaśnienia!$B$47</f>
         <v/>
       </c>
       <c r="C41" s="78">
@@ -5956,11 +5966,11 @@
         <v/>
       </c>
       <c r="D41" s="80">
-        <f>C41*Wyjaśnienia!$B$47</f>
+        <f>C41*Wyjaśnienia!$B$48</f>
         <v/>
       </c>
       <c r="E41" s="78">
-        <f>ROUNDUP(B41*Wyjaśnienia!$B$50/60,0)</f>
+        <f>ROUNDUP(B41*Wyjaśnienia!$B$51/60,0)</f>
         <v/>
       </c>
     </row>
@@ -5969,7 +5979,7 @@
         <v>10000</v>
       </c>
       <c r="B42" s="78">
-        <f>A42*Wyjaśnienia!$B$46</f>
+        <f>A42*Wyjaśnienia!$B$47</f>
         <v/>
       </c>
       <c r="C42" s="78">
@@ -5977,11 +5987,11 @@
         <v/>
       </c>
       <c r="D42" s="80">
-        <f>C42*Wyjaśnienia!$B$47</f>
+        <f>C42*Wyjaśnienia!$B$48</f>
         <v/>
       </c>
       <c r="E42" s="78">
-        <f>ROUNDUP(B42*Wyjaśnienia!$B$50/60,0)</f>
+        <f>ROUNDUP(B42*Wyjaśnienia!$B$51/60,0)</f>
         <v/>
       </c>
     </row>
@@ -5990,7 +6000,7 @@
         <v>100000</v>
       </c>
       <c r="B43" s="78">
-        <f>A43*Wyjaśnienia!$B$46</f>
+        <f>A43*Wyjaśnienia!$B$47</f>
         <v/>
       </c>
       <c r="C43" s="78">
@@ -5998,11 +6008,11 @@
         <v/>
       </c>
       <c r="D43" s="80">
-        <f>C43*Wyjaśnienia!$B$47</f>
+        <f>C43*Wyjaśnienia!$B$48</f>
         <v/>
       </c>
       <c r="E43" s="78">
-        <f>ROUNDUP(B43*Wyjaśnienia!$B$50/60,0)</f>
+        <f>ROUNDUP(B43*Wyjaśnienia!$B$51/60,0)</f>
         <v/>
       </c>
     </row>
@@ -6011,7 +6021,7 @@
         <v>1000000</v>
       </c>
       <c r="B44" s="78">
-        <f>A44*Wyjaśnienia!$B$46</f>
+        <f>A44*Wyjaśnienia!$B$47</f>
         <v/>
       </c>
       <c r="C44" s="78">
@@ -6019,11 +6029,11 @@
         <v/>
       </c>
       <c r="D44" s="80">
-        <f>C44*Wyjaśnienia!$B$47</f>
+        <f>C44*Wyjaśnienia!$B$48</f>
         <v/>
       </c>
       <c r="E44" s="78">
-        <f>ROUNDUP(B44*Wyjaśnienia!$B$50/60,0)</f>
+        <f>ROUNDUP(B44*Wyjaśnienia!$B$51/60,0)</f>
         <v/>
       </c>
     </row>
@@ -6059,11 +6069,11 @@
         <v>30</v>
       </c>
       <c r="B47" s="78">
-        <f>A47*Wyjaśnienia!$B$75</f>
+        <f>A47*Wyjaśnienia!$B$76</f>
         <v/>
       </c>
       <c r="C47" s="80">
-        <f>B47*Wyjaśnienia!$B$76</f>
+        <f>B47*Wyjaśnienia!$B$77</f>
         <v/>
       </c>
       <c r="D47" s="78">
@@ -6071,7 +6081,7 @@
         <v/>
       </c>
       <c r="E47" s="78">
-        <f>ROUNDUP(B47/Wyjaśnienia!$B$77,0)</f>
+        <f>ROUNDUP(B47/Wyjaśnienia!$B$78,0)</f>
         <v/>
       </c>
     </row>
@@ -6080,11 +6090,11 @@
         <v>150</v>
       </c>
       <c r="B48" s="78">
-        <f>A48*Wyjaśnienia!$B$75</f>
+        <f>A48*Wyjaśnienia!$B$76</f>
         <v/>
       </c>
       <c r="C48" s="80">
-        <f>B48*Wyjaśnienia!$B$76</f>
+        <f>B48*Wyjaśnienia!$B$77</f>
         <v/>
       </c>
       <c r="D48" s="78">
@@ -6092,7 +6102,7 @@
         <v/>
       </c>
       <c r="E48" s="78">
-        <f>ROUNDUP(B48/Wyjaśnienia!$B$77,0)</f>
+        <f>ROUNDUP(B48/Wyjaśnienia!$B$78,0)</f>
         <v/>
       </c>
     </row>
@@ -6101,11 +6111,11 @@
         <v>500</v>
       </c>
       <c r="B49" s="78">
-        <f>A49*Wyjaśnienia!$B$75</f>
+        <f>A49*Wyjaśnienia!$B$76</f>
         <v/>
       </c>
       <c r="C49" s="80">
-        <f>B49*Wyjaśnienia!$B$76</f>
+        <f>B49*Wyjaśnienia!$B$77</f>
         <v/>
       </c>
       <c r="D49" s="78">
@@ -6113,7 +6123,7 @@
         <v/>
       </c>
       <c r="E49" s="78">
-        <f>ROUNDUP(B49/Wyjaśnienia!$B$77,0)</f>
+        <f>ROUNDUP(B49/Wyjaśnienia!$B$78,0)</f>
         <v/>
       </c>
     </row>
@@ -6122,11 +6132,11 @@
         <v>2000</v>
       </c>
       <c r="B50" s="78">
-        <f>A50*Wyjaśnienia!$B$75</f>
+        <f>A50*Wyjaśnienia!$B$76</f>
         <v/>
       </c>
       <c r="C50" s="80">
-        <f>B50*Wyjaśnienia!$B$76</f>
+        <f>B50*Wyjaśnienia!$B$77</f>
         <v/>
       </c>
       <c r="D50" s="78">
@@ -6134,7 +6144,7 @@
         <v/>
       </c>
       <c r="E50" s="78">
-        <f>ROUNDUP(B50/Wyjaśnienia!$B$77,0)</f>
+        <f>ROUNDUP(B50/Wyjaśnienia!$B$78,0)</f>
         <v/>
       </c>
     </row>
@@ -6143,11 +6153,11 @@
         <v>10000</v>
       </c>
       <c r="B51" s="78">
-        <f>A51*Wyjaśnienia!$B$75</f>
+        <f>A51*Wyjaśnienia!$B$76</f>
         <v/>
       </c>
       <c r="C51" s="80">
-        <f>B51*Wyjaśnienia!$B$76</f>
+        <f>B51*Wyjaśnienia!$B$77</f>
         <v/>
       </c>
       <c r="D51" s="78">
@@ -6155,7 +6165,7 @@
         <v/>
       </c>
       <c r="E51" s="78">
-        <f>ROUNDUP(B51/Wyjaśnienia!$B$77,0)</f>
+        <f>ROUNDUP(B51/Wyjaśnienia!$B$78,0)</f>
         <v/>
       </c>
     </row>
@@ -6248,7 +6258,7 @@
         <v>0</v>
       </c>
       <c r="C59" s="78">
-        <f>Wyjaśnienia!$B$53*2</f>
+        <f>Wyjaśnienia!$B$54*2</f>
         <v/>
       </c>
       <c r="D59" s="80">
@@ -6444,7 +6454,7 @@
         <v>12</v>
       </c>
       <c r="D7" s="68">
-        <f>B7+C7*Wyjaśnienia!$B$66/60</f>
+        <f>B7+C7*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E7" s="52">
@@ -6471,7 +6481,7 @@
       </c>
       <c r="C8" s="63" t="n"/>
       <c r="D8" s="68">
-        <f>B8+C8*Wyjaśnienia!$B$66/60</f>
+        <f>B8+C8*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E8" s="52">
@@ -6498,7 +6508,7 @@
       </c>
       <c r="C9" s="63" t="n"/>
       <c r="D9" s="68">
-        <f>B9+C9*Wyjaśnienia!$B$66/60</f>
+        <f>B9+C9*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E9" s="52">
@@ -6525,7 +6535,7 @@
       </c>
       <c r="C10" s="63" t="n"/>
       <c r="D10" s="68">
-        <f>B10+C10*Wyjaśnienia!$B$66/60</f>
+        <f>B10+C10*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E10" s="52">
@@ -6552,7 +6562,7 @@
       </c>
       <c r="C11" s="63" t="n"/>
       <c r="D11" s="68">
-        <f>B11+C11*Wyjaśnienia!$B$66/60</f>
+        <f>B11+C11*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E11" s="52">
@@ -6579,7 +6589,7 @@
       </c>
       <c r="C12" s="63" t="n"/>
       <c r="D12" s="68">
-        <f>B12+C12*Wyjaśnienia!$B$66/60</f>
+        <f>B12+C12*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E12" s="52">
@@ -6606,7 +6616,7 @@
       </c>
       <c r="C13" s="63" t="n"/>
       <c r="D13" s="68">
-        <f>B13+C13*Wyjaśnienia!$B$66/60</f>
+        <f>B13+C13*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E13" s="52">
@@ -6633,7 +6643,7 @@
       </c>
       <c r="C14" s="63" t="n"/>
       <c r="D14" s="68">
-        <f>B14+C14*Wyjaśnienia!$B$66/60</f>
+        <f>B14+C14*Wyjaśnienia!$B$67/60</f>
         <v/>
       </c>
       <c r="E14" s="52">
@@ -6717,7 +6727,7 @@
         </is>
       </c>
       <c r="B19" s="52">
-        <f>Wyjaśnienia!$B$67</f>
+        <f>Wyjaśnienia!$B$68</f>
         <v/>
       </c>
       <c r="C19" s="68" t="n">
@@ -6743,7 +6753,7 @@
         </is>
       </c>
       <c r="B20" s="52">
-        <f>Wyjaśnienia!$B$68</f>
+        <f>Wyjaśnienia!$B$69</f>
         <v/>
       </c>
       <c r="C20" s="68" t="n">
@@ -6769,7 +6779,7 @@
         </is>
       </c>
       <c r="B21" s="52">
-        <f>Wyjaśnienia!$B$69</f>
+        <f>Wyjaśnienia!$B$70</f>
         <v/>
       </c>
       <c r="C21" s="68" t="n">
@@ -6966,7 +6976,7 @@
         </is>
       </c>
       <c r="D31" s="52">
-        <f>Wyjaśnienia!$B$67+Wyjaśnienia!$B$68</f>
+        <f>Wyjaśnienia!$B$68+Wyjaśnienia!$B$69</f>
         <v/>
       </c>
     </row>
@@ -6999,7 +7009,7 @@
         </is>
       </c>
       <c r="D34" s="52">
-        <f>(D32+D33)*Wyjaśnienia!$B$74</f>
+        <f>(D32+D33)*Wyjaśnienia!$B$75</f>
         <v/>
       </c>
     </row>
@@ -7021,7 +7031,7 @@
         </is>
       </c>
       <c r="D36" s="52">
-        <f>D35*Wyjaśnienia!$B$33</f>
+        <f>D35*Wyjaśnienia!$B$34</f>
         <v/>
       </c>
     </row>
@@ -7521,7 +7531,7 @@
       <c r="B25" s="47" t="n"/>
       <c r="C25" s="47" t="n"/>
       <c r="D25" s="52">
-        <f>(D23+D24)*Wyjaśnienia!$B$30</f>
+        <f>(D23+D24)*Wyjaśnienia!$B$31</f>
         <v/>
       </c>
       <c r="E25" s="47" t="n"/>
@@ -7553,7 +7563,7 @@
       <c r="B27" s="47" t="n"/>
       <c r="C27" s="47" t="n"/>
       <c r="D27" s="52">
-        <f>D26*Wyjaśnienia!$B$33</f>
+        <f>D26*Wyjaśnienia!$B$34</f>
         <v/>
       </c>
       <c r="E27" s="47" t="n"/>

</xml_diff>

<commit_message>
Dziesięć minut na kontrolę zgłoszenia plakatu i plik arkusza do pobrania
Osiem minut na kontrolę formalną zgłoszenia plakatu obejmowało obejrzenie
nagrania z pracy trwającego co najmniej trzy minuty, więc na sprawdzenie
pozostałych wymogów, zapis wyniku i korespondencję przy brakach zostawało
pięć. Podniesione do dziesięciu minut: 25 godzin zamiast 20, praca
organizatora 42 900 zł, oferta 167 072 zł netto.

Przeglądarka arkusza działa na JavaScripcie, więc narzędzie, które go nie
wykonuje, widzi sam ekran wczytywania i jawność kosztorysu przestaje
istnieć. Każda z ośmiu ofert ma teraz obok odnośnika do przeglądarki
odnośnik do pliku XLSX do pobrania.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -5055,7 +5055,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="63" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D7" s="68">
         <f>B7+C7*Wyjaśnienia!$B$55/60</f>
@@ -5067,7 +5067,7 @@
       </c>
       <c r="F7" s="47" t="inlineStr">
         <is>
-          <t>format, proporcje, rozdzielczość, oświadczenia; 8 minut na zgłoszenie</t>
+          <t>format, proporcje, rozdzielczość, oświadczenia; 10 minut na zgłoszenie, w tym obejrzenie nagrania z pracy trwającego co najmniej 3 minuty</t>
         </is>
       </c>
       <c r="G7" s="68" t="n">

</xml_diff>

<commit_message>
Jedna nazwa roli finansującej pulę nagród we wszystkich dokumentach
Rola nazywała się raz Fundatorem, raz Sponsorem: nagłówki trzech ofert i
kafle mówiły "Sponsor nagród", treść ofert i arkusz "Fundator". Wszędzie
zostaje Fundator nagród w plebiscycie na dany temat - w nagłówkach, w
treści, w siatce odnośników między ofertami, w kaflach na stronie dla
partnerów, w nocie koncepcyjnej i w opisach zakładek arkusza.

Mecenas plebiscytu plakatu, Mecenas Antologii i Mecenas Założycielski
zostają mecenasami, bo finansują nie samą pulę; sponsor gali i sponsor
Akademii zostają sponsorami. Rozróżnienie jest w ofertach wyjaśnione.

Adresy stron bez zmian.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -1901,7 +1901,7 @@
     <row r="2" ht="15" customHeight="1" s="45">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>Finansuje: Fundator puli nagród. Kwoty netto, chyba że napisano inaczej.</t>
+          <t>Finansuje: Fundator nagród w plebiscycie na najlepszą rozmowę ze sztuczną inteligencją. Kwoty netto, chyba że napisano inaczej.</t>
         </is>
       </c>
       <c r="H2" s="47" t="n"/>
@@ -4157,7 +4157,7 @@
     <row r="2" ht="15" customHeight="1" s="45">
       <c r="A2" s="48" t="inlineStr">
         <is>
-          <t>Finansuje: Sponsor plebiscytu. Kwoty netto, chyba że napisano inaczej.</t>
+          <t>Finansuje: Fundator nagród w plebiscycie na piosenkę o sztucznej inteligencji. Kwoty netto, chyba że napisano inaczej.</t>
         </is>
       </c>
       <c r="H2" s="47" t="n"/>
@@ -6811,7 +6811,7 @@
     <row r="2" ht="15" customHeight="1" s="45">
       <c r="A2" s="47" t="inlineStr">
         <is>
-          <t>Finansuje: Sponsor plebiscytu filmu. Kwoty netto, chyba że napisano inaczej.</t>
+          <t>Finansuje: Fundator nagród w plebiscycie na film o sztucznej inteligencji. Kwoty netto, chyba że napisano inaczej.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Arkusz: wiersze opisowe scalone na pełną szerokość w Wyjaśnieniach i w zakładkach budżetowych
W zakładce Wyjaśnienia nagłówki sekcji i akapity - między innymi "CZEGO JESZCZE
NIE MA" i "JAK CZYTAĆ BUDŻETY" - stały w kolumnie A bez scalenia, więc tekst
urywał się na szerokości pierwszej kolumny zamiast biec przez całą tabelę.
Scalone wiersze 15, 16, 38-41, 43-47, 54 i 67.

W ośmiu zakładkach budżetowych pasy i wiersze opisowe były scalone do kolumny F,
a tabele mają siedem kolumn od czasu dodania "Roku kosztu". Scalenia rozszerzone
do kolumny G, żeby kończyły się na krawędzi tabeli.

Sumy bez zmian: RAZEM 1 839 251,76 zł.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -1478,14 +1478,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1498,7 +1490,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1510,7 +1510,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1550,6 +1550,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1563,10 +1567,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1587,10 +1587,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1615,6 +1611,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2071,9 +2071,11 @@
       <c r="H14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="5" t="s">
         <v>23</v>
       </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
       <c r="D15" s="3"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -2081,9 +2083,11 @@
       <c r="H15" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
       <c r="D16" s="3"/>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -2094,10 +2098,10 @@
       <c r="A17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="12" t="n">
         <v>220</v>
       </c>
-      <c r="C17" s="15" t="s">
+      <c r="C17" s="13" t="s">
         <v>26</v>
       </c>
       <c r="D17" s="3"/>
@@ -2110,10 +2114,10 @@
       <c r="A18" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B18" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="C18" s="13" t="s">
         <v>28</v>
       </c>
       <c r="D18" s="3"/>
@@ -2126,10 +2130,10 @@
       <c r="A19" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B19" s="12" t="n">
         <v>300000</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="13" t="s">
         <v>30</v>
       </c>
       <c r="D19" s="3"/>
@@ -2142,10 +2146,10 @@
       <c r="A20" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="14" t="n">
+      <c r="B20" s="12" t="n">
         <v>3000</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="13" t="s">
         <v>32</v>
       </c>
       <c r="D20" s="3"/>
@@ -2158,10 +2162,10 @@
       <c r="A21" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="14" t="n">
+      <c r="B21" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="13" t="s">
         <v>34</v>
       </c>
       <c r="D21" s="3"/>
@@ -2174,10 +2178,10 @@
       <c r="A22" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="14" t="n">
+      <c r="B22" s="12" t="n">
         <v>40000</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="13" t="s">
         <v>36</v>
       </c>
     </row>
@@ -2185,10 +2189,10 @@
       <c r="A23" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="14" t="n">
+      <c r="B23" s="12" t="n">
         <v>10000</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="13" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2196,10 +2200,10 @@
       <c r="A24" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="14" t="n">
+      <c r="B24" s="12" t="n">
         <v>150</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="13" t="s">
         <v>40</v>
       </c>
       <c r="D24" s="3"/>
@@ -2212,10 +2216,10 @@
       <c r="A25" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="14" t="n">
+      <c r="B25" s="12" t="n">
         <v>35000</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="C25" s="13" t="s">
         <v>42</v>
       </c>
       <c r="D25" s="3"/>
@@ -2228,10 +2232,10 @@
       <c r="A26" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B26" s="14" t="n">
+      <c r="B26" s="12" t="n">
         <v>12000</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="13" t="s">
         <v>44</v>
       </c>
       <c r="D26" s="3"/>
@@ -2244,7 +2248,7 @@
       <c r="A27" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B27" s="14" t="n">
+      <c r="B27" s="12" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -2252,10 +2256,10 @@
       <c r="A28" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B28" s="14" t="n">
+      <c r="B28" s="12" t="n">
         <v>7500</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="13" t="s">
         <v>47</v>
       </c>
       <c r="D28" s="3"/>
@@ -2268,10 +2272,10 @@
       <c r="A29" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B29" s="14" t="n">
+      <c r="B29" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="13" t="s">
         <v>49</v>
       </c>
       <c r="D29" s="3"/>
@@ -2284,10 +2288,10 @@
       <c r="A30" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="14" t="n">
+      <c r="B30" s="12" t="n">
         <v>80000</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="13" t="s">
         <v>51</v>
       </c>
       <c r="D30" s="3"/>
@@ -2300,10 +2304,10 @@
       <c r="A31" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="14" t="n">
+      <c r="B31" s="12" t="n">
         <v>1200</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="13" t="s">
         <v>53</v>
       </c>
       <c r="D31" s="3"/>
@@ -2316,10 +2320,10 @@
       <c r="A32" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="16" t="n">
+      <c r="B32" s="14" t="n">
         <v>0.12</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="C32" s="13" t="s">
         <v>55</v>
       </c>
       <c r="D32" s="3"/>
@@ -2332,10 +2336,10 @@
       <c r="A33" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="16" t="n">
+      <c r="B33" s="14" t="n">
         <v>0.2</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="13" t="s">
         <v>57</v>
       </c>
       <c r="D33" s="3"/>
@@ -2348,10 +2352,10 @@
       <c r="A34" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B34" s="16" t="n">
+      <c r="B34" s="14" t="n">
         <v>0.12</v>
       </c>
-      <c r="C34" s="15" t="s">
+      <c r="C34" s="13" t="s">
         <v>55</v>
       </c>
       <c r="D34" s="3"/>
@@ -2364,10 +2368,10 @@
       <c r="A35" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="16" t="n">
+      <c r="B35" s="14" t="n">
         <v>0.23</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="13" t="s">
         <v>60</v>
       </c>
       <c r="D35" s="3"/>
@@ -2395,9 +2399,11 @@
       <c r="H37" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="5" t="s">
         <v>62</v>
       </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -2405,9 +2411,11 @@
       <c r="H38" s="3"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="s">
+      <c r="A39" s="15" t="s">
         <v>63</v>
       </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -2415,9 +2423,11 @@
       <c r="H39" s="3"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="15" t="s">
         <v>64</v>
       </c>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -2425,9 +2435,11 @@
       <c r="H40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="4" t="s">
         <v>65</v>
       </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -2443,9 +2455,11 @@
       <c r="H42" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12" t="s">
+      <c r="A43" s="5" t="s">
         <v>66</v>
       </c>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -2453,9 +2467,11 @@
       <c r="H43" s="3"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
+      <c r="A44" s="4" t="s">
         <v>67</v>
       </c>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
@@ -2463,9 +2479,11 @@
       <c r="H44" s="3"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="13" t="s">
+      <c r="A45" s="4" t="s">
         <v>68</v>
       </c>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
@@ -2473,20 +2491,24 @@
       <c r="H45" s="3"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="16" t="s">
         <v>69</v>
       </c>
+      <c r="B46" s="16"/>
+      <c r="C46" s="16"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="17" t="s">
         <v>70</v>
       </c>
+      <c r="B47" s="17"/>
+      <c r="C47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B48" s="14" t="n">
+      <c r="B48" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C48" s="3" t="s">
@@ -2519,7 +2541,7 @@
       <c r="A51" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B51" s="14" t="n">
+      <c r="B51" s="12" t="n">
         <v>15</v>
       </c>
       <c r="C51" s="3" t="s">
@@ -2539,6 +2561,8 @@
       <c r="A54" s="20" t="s">
         <v>80</v>
       </c>
+      <c r="B54" s="20"/>
+      <c r="C54" s="20"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
@@ -2666,12 +2690,14 @@
       <c r="A67" s="20" t="s">
         <v>101</v>
       </c>
+      <c r="B67" s="20"/>
+      <c r="C67" s="20"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B68" s="14" t="n">
+      <c r="B68" s="12" t="n">
         <v>150</v>
       </c>
       <c r="C68" s="1" t="s">
@@ -2682,7 +2708,7 @@
       <c r="A69" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B69" s="14" t="n">
+      <c r="B69" s="12" t="n">
         <v>180000</v>
       </c>
       <c r="C69" s="1" t="s">
@@ -2693,7 +2719,7 @@
       <c r="A70" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B70" s="14" t="n">
+      <c r="B70" s="12" t="n">
         <v>12000</v>
       </c>
       <c r="C70" s="1" t="s">
@@ -2704,7 +2730,7 @@
       <c r="A71" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B71" s="14" t="n">
+      <c r="B71" s="12" t="n">
         <v>1200</v>
       </c>
       <c r="C71" s="1" t="s">
@@ -2715,7 +2741,7 @@
       <c r="A72" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B72" s="14" t="n">
+      <c r="B72" s="12" t="n">
         <v>10</v>
       </c>
       <c r="C72" s="1" t="s">
@@ -2726,7 +2752,7 @@
       <c r="A73" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B73" s="14" t="n">
+      <c r="B73" s="12" t="n">
         <v>5</v>
       </c>
       <c r="C73" s="1" t="s">
@@ -2737,7 +2763,7 @@
       <c r="A74" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B74" s="14" t="n">
+      <c r="B74" s="12" t="n">
         <v>40</v>
       </c>
       <c r="C74" s="1" t="s">
@@ -2748,7 +2774,7 @@
       <c r="A75" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B75" s="14" t="n">
+      <c r="B75" s="12" t="n">
         <v>290</v>
       </c>
       <c r="C75" s="1" t="s">
@@ -2759,7 +2785,7 @@
       <c r="A76" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B76" s="14" t="n">
+      <c r="B76" s="12" t="n">
         <v>0.12</v>
       </c>
       <c r="C76" s="1" t="s">
@@ -2770,7 +2796,7 @@
       <c r="A77" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B77" s="14" t="n">
+      <c r="B77" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C77" s="1" t="s">
@@ -2781,7 +2807,7 @@
       <c r="A78" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B78" s="14" t="n">
+      <c r="B78" s="12" t="n">
         <v>300</v>
       </c>
       <c r="C78" s="1" t="s">
@@ -2792,7 +2818,7 @@
       <c r="A79" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B79" s="14" t="n">
+      <c r="B79" s="12" t="n">
         <v>10</v>
       </c>
       <c r="C79" s="1" t="s">
@@ -2826,10 +2852,23 @@
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="16">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A40:C40"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A54:C54"/>
+    <mergeCell ref="A67:C67"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2867,6 +2906,7 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
       <c r="H1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2878,6 +2918,7 @@
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2889,6 +2930,7 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2909,6 +2951,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
       <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2953,7 +2996,7 @@
         <f aca="false">D7*Wyjaśnienia!$B$17</f>
         <v>13200</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="13" t="s">
         <v>136</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -2979,7 +3022,7 @@
         <f aca="false">D8*Wyjaśnienia!$B$17</f>
         <v>5280</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="13" t="s">
         <v>139</v>
       </c>
       <c r="G8" s="26" t="s">
@@ -3005,7 +3048,7 @@
         <f aca="false">D9*Wyjaśnienia!$B$17</f>
         <v>11000</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="13" t="s">
         <v>141</v>
       </c>
       <c r="G9" s="26" t="s">
@@ -3031,7 +3074,7 @@
         <f aca="false">D10*Wyjaśnienia!$B$17</f>
         <v>5060</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="13" t="s">
         <v>143</v>
       </c>
       <c r="G10" s="26" t="s">
@@ -3057,7 +3100,7 @@
         <f aca="false">D11*Wyjaśnienia!$B$17</f>
         <v>4400</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="13" t="s">
         <v>145</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -3083,7 +3126,7 @@
         <f aca="false">D12*Wyjaśnienia!$B$17</f>
         <v>4400</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="13" t="s">
         <v>147</v>
       </c>
       <c r="G12" s="26" t="s">
@@ -3109,7 +3152,7 @@
         <f aca="false">D13*Wyjaśnienia!$B$17</f>
         <v>8800</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="13" t="s">
         <v>149</v>
       </c>
       <c r="G13" s="26" t="s">
@@ -3135,7 +3178,7 @@
         <f aca="false">D14*Wyjaśnienia!$B$17</f>
         <v>5500</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="13" t="s">
         <v>152</v>
       </c>
       <c r="G14" s="26" t="s">
@@ -3161,7 +3204,7 @@
         <f aca="false">D15*Wyjaśnienia!$B$17</f>
         <v>5500</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="13" t="s">
         <v>154</v>
       </c>
       <c r="G15" s="26" t="s">
@@ -3187,7 +3230,7 @@
         <f aca="false">D16*Wyjaśnienia!$B$17</f>
         <v>8800</v>
       </c>
-      <c r="F16" s="15" t="s">
+      <c r="F16" s="13" t="s">
         <v>156</v>
       </c>
       <c r="G16" s="26" t="s">
@@ -3230,6 +3273,7 @@
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
       <c r="H19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3267,7 +3311,7 @@
         <f aca="false">B21*C21</f>
         <v>1200</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="13" t="s">
         <v>162</v>
       </c>
       <c r="F21" s="3"/>
@@ -3290,7 +3334,7 @@
         <f aca="false">B22*C22</f>
         <v>1500</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="13" t="s">
         <v>164</v>
       </c>
       <c r="F22" s="3"/>
@@ -3313,7 +3357,7 @@
         <f aca="false">B23*C23</f>
         <v>250</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="13" t="s">
         <v>166</v>
       </c>
       <c r="F23" s="3"/>
@@ -3336,7 +3380,7 @@
         <f aca="false">B24*C24</f>
         <v>32000</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="13" t="s">
         <v>168</v>
       </c>
       <c r="F24" s="3" t="s">
@@ -3361,7 +3405,7 @@
         <f aca="false">B25*C25</f>
         <v>0</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="13" t="s">
         <v>171</v>
       </c>
       <c r="F25" s="3"/>
@@ -3383,7 +3427,7 @@
         <f aca="false">B26*C26</f>
         <v>15000</v>
       </c>
-      <c r="E26" s="15" t="s">
+      <c r="E26" s="13" t="s">
         <v>173</v>
       </c>
       <c r="F26" s="3"/>
@@ -3407,7 +3451,7 @@
         <f aca="false">B27*C27</f>
         <v>12000</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="E27" s="13" t="s">
         <v>175</v>
       </c>
       <c r="F27" s="3"/>
@@ -3429,7 +3473,7 @@
         <f aca="false">B28*C28</f>
         <v>0</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="13" t="s">
         <v>177</v>
       </c>
       <c r="F28" s="3"/>
@@ -3452,7 +3496,7 @@
         <f aca="false">B29*C29</f>
         <v>10000</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="E29" s="13" t="s">
         <v>179</v>
       </c>
       <c r="F29" s="3"/>
@@ -3474,7 +3518,7 @@
         <f aca="false">B30*C30</f>
         <v>13333</v>
       </c>
-      <c r="E30" s="15" t="s">
+      <c r="E30" s="13" t="s">
         <v>181</v>
       </c>
       <c r="F30" s="3"/>
@@ -3493,7 +3537,7 @@
         <f aca="false">B31*C31</f>
         <v>3000</v>
       </c>
-      <c r="E31" s="15" t="s">
+      <c r="E31" s="13" t="s">
         <v>183</v>
       </c>
       <c r="F31" s="3"/>
@@ -3508,7 +3552,7 @@
         <f aca="false">SUM(D21:D31)</f>
         <v>88283</v>
       </c>
-      <c r="E32" s="15"/>
+      <c r="E32" s="13"/>
       <c r="F32" s="3"/>
       <c r="H32" s="3"/>
     </row>
@@ -3519,10 +3563,11 @@
       <c r="D33" s="29"/>
       <c r="E33" s="29"/>
       <c r="F33" s="29"/>
+      <c r="G33" s="29"/>
       <c r="H33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="30" t="s">
         <v>185</v>
       </c>
       <c r="H34" s="3"/>
@@ -3616,7 +3661,7 @@
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
-      <c r="D41" s="30" t="n">
+      <c r="D41" s="31" t="n">
         <f aca="false">D39+D40</f>
         <v>673806.0048</v>
       </c>
@@ -3690,12 +3735,12 @@
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A33:G33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3733,6 +3778,7 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
       <c r="H1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3744,6 +3790,7 @@
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3755,6 +3802,7 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3775,6 +3823,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
       <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3819,7 +3868,7 @@
         <f aca="false">D7*Wyjaśnienia!$B$17</f>
         <v>9900</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="13" t="s">
         <v>196</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -3845,7 +3894,7 @@
         <f aca="false">D8*Wyjaśnienia!$B$17</f>
         <v>8800</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="13" t="s">
         <v>198</v>
       </c>
       <c r="G8" s="26" t="s">
@@ -3871,7 +3920,7 @@
         <f aca="false">D9*Wyjaśnienia!$B$17</f>
         <v>2200</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="13" t="s">
         <v>200</v>
       </c>
       <c r="G9" s="26" t="s">
@@ -3885,8 +3934,8 @@
       <c r="C10" s="23"/>
       <c r="D10" s="24"/>
       <c r="E10" s="25"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="31"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="32"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3895,8 +3944,8 @@
       <c r="C11" s="23"/>
       <c r="D11" s="24"/>
       <c r="E11" s="25"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="31"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="32"/>
       <c r="H11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3905,8 +3954,8 @@
       <c r="C12" s="23"/>
       <c r="D12" s="24"/>
       <c r="E12" s="25"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="31"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="32"/>
       <c r="H12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3927,7 +3976,7 @@
         <f aca="false">D13*Wyjaśnienia!$B$17</f>
         <v>11000</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="13" t="s">
         <v>202</v>
       </c>
       <c r="G13" s="26" t="s">
@@ -3953,7 +4002,7 @@
         <f aca="false">D14*Wyjaśnienia!$B$17</f>
         <v>15840</v>
       </c>
-      <c r="F14" s="15"/>
+      <c r="F14" s="13"/>
       <c r="G14" s="26" t="s">
         <v>137</v>
       </c>
@@ -3993,6 +4042,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
       <c r="H17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4022,9 +4072,9 @@
       <c r="B19" s="28"/>
       <c r="C19" s="23"/>
       <c r="D19" s="25"/>
-      <c r="E19" s="15"/>
+      <c r="E19" s="13"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="31"/>
+      <c r="G19" s="32"/>
       <c r="H19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4032,9 +4082,9 @@
       <c r="B20" s="28"/>
       <c r="C20" s="23"/>
       <c r="D20" s="25"/>
-      <c r="E20" s="15"/>
+      <c r="E20" s="13"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="31"/>
+      <c r="G20" s="32"/>
       <c r="H20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4042,9 +4092,9 @@
       <c r="B21" s="28"/>
       <c r="C21" s="23"/>
       <c r="D21" s="25"/>
-      <c r="E21" s="15"/>
+      <c r="E21" s="13"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="31"/>
+      <c r="G21" s="32"/>
       <c r="H21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4061,7 +4111,7 @@
         <f aca="false">B22*C22</f>
         <v>40000</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="13" t="s">
         <v>205</v>
       </c>
       <c r="F22" s="3"/>
@@ -4084,7 +4134,7 @@
         <f aca="false">B23*C23</f>
         <v>4000</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="13" t="s">
         <v>207</v>
       </c>
       <c r="F23" s="3"/>
@@ -4107,7 +4157,7 @@
         <f aca="false">B24*C24</f>
         <v>3000</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="13" t="s">
         <v>209</v>
       </c>
       <c r="F24" s="3"/>
@@ -4130,7 +4180,7 @@
         <f aca="false">B25*C25</f>
         <v>4000</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="13" t="s">
         <v>211</v>
       </c>
       <c r="F25" s="3"/>
@@ -4153,7 +4203,7 @@
         <f aca="false">B26*C26</f>
         <v>0</v>
       </c>
-      <c r="E26" s="15" t="s">
+      <c r="E26" s="13" t="s">
         <v>213</v>
       </c>
       <c r="F26" s="3"/>
@@ -4167,9 +4217,9 @@
       <c r="B27" s="28"/>
       <c r="C27" s="23"/>
       <c r="D27" s="25"/>
-      <c r="E27" s="15"/>
+      <c r="E27" s="13"/>
       <c r="F27" s="3"/>
-      <c r="G27" s="31"/>
+      <c r="G27" s="32"/>
       <c r="H27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4177,9 +4227,9 @@
       <c r="B28" s="28"/>
       <c r="C28" s="23"/>
       <c r="D28" s="25"/>
-      <c r="E28" s="15"/>
+      <c r="E28" s="13"/>
       <c r="F28" s="3"/>
-      <c r="G28" s="31"/>
+      <c r="G28" s="32"/>
       <c r="H28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4187,27 +4237,27 @@
       <c r="B29" s="28"/>
       <c r="C29" s="23"/>
       <c r="D29" s="25"/>
-      <c r="E29" s="15"/>
+      <c r="E29" s="13"/>
       <c r="F29" s="3"/>
-      <c r="G29" s="31"/>
+      <c r="G29" s="32"/>
       <c r="H29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32"/>
+      <c r="A30" s="33"/>
       <c r="B30" s="18"/>
-      <c r="C30" s="33"/>
+      <c r="C30" s="34"/>
       <c r="D30" s="8"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="31"/>
+      <c r="F30" s="33"/>
+      <c r="G30" s="32"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="33" t="s">
         <v>214</v>
       </c>
       <c r="B31" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="33" t="n">
+      <c r="C31" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="8" t="n">
@@ -4217,19 +4267,19 @@
       <c r="E31" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F31" s="32"/>
+      <c r="F31" s="33"/>
       <c r="G31" s="26" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="32" t="s">
+      <c r="A32" s="33" t="s">
         <v>216</v>
       </c>
       <c r="B32" s="18" t="n">
         <v>40000</v>
       </c>
-      <c r="C32" s="33" t="n">
+      <c r="C32" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="8" t="n">
@@ -4239,20 +4289,21 @@
       <c r="E32" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="F32" s="32"/>
+      <c r="F32" s="33"/>
       <c r="G32" s="26" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="34" t="s">
+      <c r="A33" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="34"/>
-      <c r="E33" s="34"/>
-      <c r="F33" s="34"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
       <c r="H33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4262,10 +4313,11 @@
       <c r="D34" s="29"/>
       <c r="E34" s="29"/>
       <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
       <c r="H34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="30" t="s">
         <v>185</v>
       </c>
       <c r="H35" s="3"/>
@@ -4348,7 +4400,7 @@
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
-      <c r="D41" s="30" t="n">
+      <c r="D41" s="31" t="n">
         <f aca="false">D39+D40</f>
         <v>199459.26</v>
       </c>
@@ -4422,13 +4474,13 @@
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A34:G34"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4465,6 +4517,7 @@
       <c r="D1" s="29"/>
       <c r="E1" s="29"/>
       <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
@@ -4475,6 +4528,7 @@
       <c r="D2" s="29"/>
       <c r="E2" s="29"/>
       <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="29" t="s">
@@ -4485,6 +4539,7 @@
       <c r="D3" s="29"/>
       <c r="E3" s="29"/>
       <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="s">
@@ -4495,6 +4550,7 @@
       <c r="D5" s="29"/>
       <c r="E5" s="29"/>
       <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
@@ -4617,6 +4673,7 @@
       <c r="D13" s="29"/>
       <c r="E13" s="29"/>
       <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
@@ -4800,6 +4857,7 @@
       <c r="D24" s="29"/>
       <c r="E24" s="29"/>
       <c r="F24" s="29"/>
+      <c r="G24" s="29"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
@@ -4860,12 +4918,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A24:G24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4903,6 +4961,7 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
       <c r="H1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4914,6 +4973,7 @@
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4925,6 +4985,7 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4945,6 +5006,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
       <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4989,7 +5051,7 @@
         <f aca="false">D7*Wyjaśnienia!$B$17</f>
         <v>5500</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="13" t="s">
         <v>243</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -5013,7 +5075,7 @@
         <f aca="false">D8*Wyjaśnienia!$B$17</f>
         <v>8800</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="13" t="s">
         <v>245</v>
       </c>
       <c r="G8" s="26" t="s">
@@ -5037,7 +5099,7 @@
         <f aca="false">D9*Wyjaśnienia!$B$17</f>
         <v>6600</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="13" t="s">
         <v>247</v>
       </c>
       <c r="G9" s="26" t="s">
@@ -5061,7 +5123,7 @@
         <f aca="false">D10*Wyjaśnienia!$B$17</f>
         <v>4400</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="13" t="s">
         <v>249</v>
       </c>
       <c r="G10" s="26" t="s">
@@ -5085,7 +5147,7 @@
         <f aca="false">D11*Wyjaśnienia!$B$17</f>
         <v>11000</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="13" t="s">
         <v>251</v>
       </c>
       <c r="G11" s="26" t="s">
@@ -5130,6 +5192,7 @@
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
       <c r="H14" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5169,7 +5232,7 @@
         <f aca="false">B16*C16</f>
         <v>35000</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="13" t="s">
         <v>254</v>
       </c>
       <c r="F16" s="3"/>
@@ -5193,7 +5256,7 @@
         <f aca="false">B17*C17</f>
         <v>12000</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="13" t="s">
         <v>175</v>
       </c>
       <c r="F17" s="3"/>
@@ -5218,7 +5281,7 @@
         <f aca="false">B18*C18</f>
         <v>75000</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="E18" s="13" t="s">
         <v>256</v>
       </c>
       <c r="F18" s="3"/>
@@ -5242,7 +5305,7 @@
         <f aca="false">B19*C19</f>
         <v>80000</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="E19" s="13" t="s">
         <v>257</v>
       </c>
       <c r="F19" s="3"/>
@@ -5266,7 +5329,7 @@
         <f aca="false">B20*C20</f>
         <v>1200</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="13" t="s">
         <v>259</v>
       </c>
       <c r="F20" s="3"/>
@@ -5289,7 +5352,7 @@
         <f aca="false">B21*C21</f>
         <v>0</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="13" t="s">
         <v>261</v>
       </c>
       <c r="F21" s="3"/>
@@ -5312,7 +5375,7 @@
         <f aca="false">B22*C22</f>
         <v>0</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="13" t="s">
         <v>262</v>
       </c>
       <c r="F22" s="3"/>
@@ -5334,7 +5397,7 @@
         <f aca="false">B23*C23</f>
         <v>0</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="13" t="s">
         <v>264</v>
       </c>
       <c r="F23" s="3"/>
@@ -5344,13 +5407,13 @@
       <c r="H23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="s">
+      <c r="A24" s="33" t="s">
         <v>265</v>
       </c>
       <c r="B24" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="33" t="n">
+      <c r="C24" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8" t="n">
@@ -5360,7 +5423,7 @@
       <c r="E24" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="F24" s="32" t="s">
+      <c r="F24" s="33" t="s">
         <v>267</v>
       </c>
       <c r="G24" s="26" t="s">
@@ -5368,13 +5431,13 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="32" t="s">
+      <c r="A25" s="33" t="s">
         <v>268</v>
       </c>
       <c r="B25" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="33" t="n">
+      <c r="C25" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -5384,19 +5447,19 @@
       <c r="E25" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="F25" s="32"/>
+      <c r="F25" s="33"/>
       <c r="G25" s="26" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="33" t="s">
         <v>182</v>
       </c>
       <c r="B26" s="18" t="n">
         <v>3000</v>
       </c>
-      <c r="C26" s="33" t="n">
+      <c r="C26" s="34" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="8" t="n">
@@ -5406,7 +5469,7 @@
       <c r="E26" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="F26" s="32"/>
+      <c r="F26" s="33"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
@@ -5425,6 +5488,7 @@
       <c r="D28" s="29"/>
       <c r="E28" s="29"/>
       <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
       <c r="H28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5436,6 +5500,7 @@
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
       <c r="H29" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5528,7 +5593,7 @@
       </c>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
-      <c r="D36" s="30" t="n">
+      <c r="D36" s="31" t="n">
         <f aca="false">D34+D35</f>
         <v>327130.8</v>
       </c>
@@ -5607,13 +5672,13 @@
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A29:G29"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -5651,6 +5716,7 @@
       <c r="D1" s="36"/>
       <c r="E1" s="36"/>
       <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
@@ -5661,6 +5727,7 @@
       <c r="D2" s="29"/>
       <c r="E2" s="29"/>
       <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="29" t="s">
@@ -5671,6 +5738,7 @@
       <c r="D3" s="29"/>
       <c r="E3" s="29"/>
       <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="36" t="s">
@@ -5681,6 +5749,7 @@
       <c r="D5" s="36"/>
       <c r="E5" s="36"/>
       <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
@@ -5715,7 +5784,7 @@
       <c r="C7" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="D7" s="31" t="n">
+      <c r="D7" s="32" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$55/60</f>
         <v>25</v>
       </c>
@@ -5737,8 +5806,8 @@
       <c r="B8" s="21" t="n">
         <v>30</v>
       </c>
-      <c r="C8" s="31"/>
-      <c r="D8" s="31" t="n">
+      <c r="C8" s="32"/>
+      <c r="D8" s="32" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$55/60</f>
         <v>30</v>
       </c>
@@ -5760,8 +5829,8 @@
       <c r="B9" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31" t="n">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$55/60</f>
         <v>20</v>
       </c>
@@ -5783,8 +5852,8 @@
       <c r="B10" s="21" t="n">
         <v>35</v>
       </c>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31" t="n">
+      <c r="C10" s="32"/>
+      <c r="D10" s="32" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$55/60</f>
         <v>35</v>
       </c>
@@ -5806,8 +5875,8 @@
       <c r="B11" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31" t="n">
+      <c r="C11" s="32"/>
+      <c r="D11" s="32" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$55/60</f>
         <v>15</v>
       </c>
@@ -5829,8 +5898,8 @@
       <c r="B12" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="C12" s="31"/>
-      <c r="D12" s="31" t="n">
+      <c r="C12" s="32"/>
+      <c r="D12" s="32" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$55/60</f>
         <v>50</v>
       </c>
@@ -5852,8 +5921,8 @@
       <c r="B13" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31" t="n">
+      <c r="C13" s="32"/>
+      <c r="D13" s="32" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$55/60</f>
         <v>20</v>
       </c>
@@ -5893,6 +5962,7 @@
       <c r="D16" s="36"/>
       <c r="E16" s="36"/>
       <c r="F16" s="36"/>
+      <c r="G16" s="36"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
@@ -5922,7 +5992,7 @@
         <f aca="false">Wyjaśnienia!$B$56</f>
         <v>90000</v>
       </c>
-      <c r="C18" s="31" t="n">
+      <c r="C18" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="8" t="n">
@@ -5944,7 +6014,7 @@
         <f aca="false">Wyjaśnienia!$B$57</f>
         <v>12000</v>
       </c>
-      <c r="C19" s="31" t="n">
+      <c r="C19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="8" t="n">
@@ -5966,7 +6036,7 @@
         <f aca="false">Wyjaśnienia!$B$58</f>
         <v>1200</v>
       </c>
-      <c r="C20" s="31" t="n">
+      <c r="C20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
@@ -5987,7 +6057,7 @@
       <c r="B21" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C21" s="31" t="n">
+      <c r="C21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="8" t="n">
@@ -6008,7 +6078,7 @@
       <c r="B22" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="31" t="n">
+      <c r="C22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="8" t="n">
@@ -6030,7 +6100,7 @@
         <f aca="false">Wyjaśnienia!$B$63*2</f>
         <v>800</v>
       </c>
-      <c r="C23" s="31" t="n">
+      <c r="C23" s="32" t="n">
         <f aca="false">Wyjaśnienia!$B$62</f>
         <v>10</v>
       </c>
@@ -6053,7 +6123,7 @@
         <f aca="false">Wyjaśnienia!$B$64</f>
         <v>3000</v>
       </c>
-      <c r="C24" s="31" t="n">
+      <c r="C24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8" t="n">
@@ -6074,7 +6144,7 @@
       <c r="B25" s="18" t="n">
         <v>8000</v>
       </c>
-      <c r="C25" s="31" t="n">
+      <c r="C25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -6095,7 +6165,7 @@
       <c r="B26" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="31" t="n">
+      <c r="C26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="8" t="n">
@@ -6116,7 +6186,7 @@
       <c r="B27" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="31" t="n">
+      <c r="C27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="8" t="n">
@@ -6137,7 +6207,7 @@
       <c r="B28" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C28" s="31" t="n">
+      <c r="C28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="8" t="n">
@@ -6158,7 +6228,7 @@
       <c r="B29" s="18" t="n">
         <v>3000</v>
       </c>
-      <c r="C29" s="31" t="n">
+      <c r="C29" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="8" t="n">
@@ -6185,6 +6255,7 @@
       <c r="D31" s="29"/>
       <c r="E31" s="29"/>
       <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
@@ -6292,7 +6363,7 @@
       <c r="B44" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C44" s="31" t="n">
+      <c r="C44" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D44" s="8" t="n">
@@ -6311,7 +6382,7 @@
         <f aca="false">Wyjaśnienia!$B$17</f>
         <v>220</v>
       </c>
-      <c r="C45" s="31" t="n">
+      <c r="C45" s="32" t="n">
         <v>20</v>
       </c>
       <c r="D45" s="8" t="n">
@@ -6324,12 +6395,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A31:G31"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6367,6 +6438,7 @@
       <c r="D1" s="38"/>
       <c r="E1" s="38"/>
       <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="39" t="s">
@@ -6377,6 +6449,7 @@
       <c r="D2" s="39"/>
       <c r="E2" s="39"/>
       <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="39" t="s">
@@ -6387,147 +6460,150 @@
       <c r="D3" s="39"/>
       <c r="E3" s="39"/>
       <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="17" t="s">
         <v>308</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="41" t="s">
         <v>309</v>
       </c>
-      <c r="F6" s="41" t="s">
+      <c r="F6" s="40" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="33" t="s">
         <v>310</v>
       </c>
-      <c r="B7" s="43" t="n">
+      <c r="B7" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$18</f>
         <v>150</v>
       </c>
-      <c r="F7" s="32" t="s">
+      <c r="F7" s="33" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="33" t="s">
         <v>312</v>
       </c>
-      <c r="B8" s="43" t="n">
+      <c r="B8" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$48</f>
         <v>2</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F8" s="33" t="s">
         <v>313</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="40" t="s">
         <v>314</v>
       </c>
-      <c r="B9" s="44" t="n">
+      <c r="B9" s="43" t="n">
         <f aca="false">B7*B8</f>
         <v>300</v>
       </c>
-      <c r="F9" s="32" t="s">
+      <c r="F9" s="33" t="s">
         <v>315</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="32" t="s">
+      <c r="A10" s="33" t="s">
         <v>316</v>
       </c>
-      <c r="B10" s="43" t="n">
+      <c r="B10" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$68</f>
         <v>150</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="33" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="32" t="s">
+      <c r="A11" s="33" t="s">
         <v>318</v>
       </c>
-      <c r="B11" s="43" t="n">
+      <c r="B11" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$77</f>
         <v>2</v>
       </c>
-      <c r="F11" s="32" t="s">
+      <c r="F11" s="33" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="40" t="s">
         <v>320</v>
       </c>
-      <c r="B12" s="44" t="n">
+      <c r="B12" s="43" t="n">
         <f aca="false">B10*B11</f>
         <v>300</v>
       </c>
-      <c r="F12" s="32" t="s">
+      <c r="F12" s="33" t="s">
         <v>321</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="40" t="s">
+      <c r="A14" s="17" t="s">
         <v>322</v>
       </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="41" t="s">
+      <c r="A15" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="B15" s="42" t="s">
+      <c r="B15" s="41" t="s">
         <v>323</v>
       </c>
-      <c r="C15" s="42" t="s">
+      <c r="C15" s="41" t="s">
         <v>160</v>
       </c>
-      <c r="D15" s="42" t="s">
+      <c r="D15" s="41" t="s">
         <v>132</v>
       </c>
-      <c r="F15" s="41" t="s">
+      <c r="F15" s="40" t="s">
         <v>133</v>
       </c>
-      <c r="G15" s="41" t="s">
+      <c r="G15" s="40" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
+      <c r="A16" s="33" t="s">
         <v>324</v>
       </c>
-      <c r="B16" s="45" t="n">
+      <c r="B16" s="44" t="n">
         <f aca="false">Wyjaśnienia!$B$50</f>
         <v>2500</v>
       </c>
-      <c r="C16" s="43" t="n">
+      <c r="C16" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$51</f>
         <v>15</v>
       </c>
-      <c r="D16" s="45" t="n">
+      <c r="D16" s="44" t="n">
         <f aca="false">B16*C16</f>
         <v>37500</v>
       </c>
-      <c r="F16" s="32" t="s">
+      <c r="F16" s="33" t="s">
         <v>325</v>
       </c>
       <c r="G16" s="26" t="s">
@@ -6535,22 +6611,22 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="33" t="s">
         <v>326</v>
       </c>
-      <c r="B17" s="45" t="n">
+      <c r="B17" s="44" t="n">
         <f aca="false">Wyjaśnienia!$B$49</f>
         <v>500</v>
       </c>
-      <c r="C17" s="43" t="n">
+      <c r="C17" s="42" t="n">
         <f aca="false">ROUNDUP(B9/100,0)</f>
         <v>3</v>
       </c>
-      <c r="D17" s="45" t="n">
+      <c r="D17" s="44" t="n">
         <f aca="false">B17*C17</f>
         <v>1500</v>
       </c>
-      <c r="F17" s="32" t="s">
+      <c r="F17" s="33" t="s">
         <v>327</v>
       </c>
       <c r="G17" s="26" t="s">
@@ -6558,22 +6634,22 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="32" t="s">
+      <c r="A18" s="33" t="s">
         <v>328</v>
       </c>
-      <c r="B18" s="45" t="n">
+      <c r="B18" s="44" t="n">
         <f aca="false">Wyjaśnienia!$B$78</f>
         <v>300</v>
       </c>
-      <c r="C18" s="43" t="n">
+      <c r="C18" s="42" t="n">
         <f aca="false">B12</f>
         <v>300</v>
       </c>
-      <c r="D18" s="45" t="n">
+      <c r="D18" s="44" t="n">
         <f aca="false">B18*C18</f>
         <v>90000</v>
       </c>
-      <c r="F18" s="32" t="s">
+      <c r="F18" s="33" t="s">
         <v>329</v>
       </c>
       <c r="G18" s="26" t="s">
@@ -6581,59 +6657,60 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="41" t="s">
+      <c r="A19" s="40" t="s">
         <v>330</v>
       </c>
-      <c r="D19" s="46" t="n">
+      <c r="D19" s="45" t="n">
         <f aca="false">SUM(D16:D18)</f>
         <v>129000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="17" t="s">
         <v>158</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="41" t="s">
+      <c r="A22" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="41" t="s">
         <v>159</v>
       </c>
-      <c r="C22" s="42" t="s">
+      <c r="C22" s="41" t="s">
         <v>160</v>
       </c>
-      <c r="D22" s="42" t="s">
+      <c r="D22" s="41" t="s">
         <v>132</v>
       </c>
-      <c r="F22" s="41" t="s">
+      <c r="F22" s="40" t="s">
         <v>133</v>
       </c>
-      <c r="G22" s="41" t="s">
+      <c r="G22" s="40" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="33" t="s">
         <v>331</v>
       </c>
-      <c r="B23" s="45" t="n">
+      <c r="B23" s="44" t="n">
         <v>2000</v>
       </c>
-      <c r="C23" s="43" t="n">
+      <c r="C23" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="D23" s="45" t="n">
+      <c r="D23" s="44" t="n">
         <f aca="false">B23*C23</f>
         <v>2000</v>
       </c>
-      <c r="F23" s="32" t="s">
+      <c r="F23" s="33" t="s">
         <v>332</v>
       </c>
       <c r="G23" s="26" t="s">
@@ -6641,20 +6718,20 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="32" t="s">
+      <c r="A24" s="33" t="s">
         <v>333</v>
       </c>
-      <c r="B24" s="45" t="n">
+      <c r="B24" s="44" t="n">
         <v>3000</v>
       </c>
-      <c r="C24" s="43" t="n">
+      <c r="C24" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="45" t="n">
+      <c r="D24" s="44" t="n">
         <f aca="false">B24*C24</f>
         <v>3000</v>
       </c>
-      <c r="F24" s="32" t="s">
+      <c r="F24" s="33" t="s">
         <v>334</v>
       </c>
       <c r="G24" s="26" t="s">
@@ -6662,20 +6739,20 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="32" t="s">
+      <c r="A25" s="33" t="s">
         <v>335</v>
       </c>
-      <c r="B25" s="45" t="n">
+      <c r="B25" s="44" t="n">
         <v>5000</v>
       </c>
-      <c r="C25" s="43" t="n">
+      <c r="C25" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="D25" s="45" t="n">
+      <c r="D25" s="44" t="n">
         <f aca="false">B25*C25</f>
         <v>5000</v>
       </c>
-      <c r="F25" s="32" t="s">
+      <c r="F25" s="33" t="s">
         <v>336</v>
       </c>
       <c r="G25" s="26" t="s">
@@ -6683,20 +6760,20 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="32" t="s">
+      <c r="A26" s="33" t="s">
         <v>337</v>
       </c>
-      <c r="B26" s="45" t="n">
+      <c r="B26" s="44" t="n">
         <v>4000</v>
       </c>
-      <c r="C26" s="43" t="n">
+      <c r="C26" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="45" t="n">
+      <c r="D26" s="44" t="n">
         <f aca="false">B26*C26</f>
         <v>4000</v>
       </c>
-      <c r="F26" s="32" t="s">
+      <c r="F26" s="33" t="s">
         <v>338</v>
       </c>
       <c r="G26" s="26" t="s">
@@ -6704,87 +6781,89 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="41" t="s">
+      <c r="A27" s="40" t="s">
         <v>184</v>
       </c>
-      <c r="D27" s="46" t="n">
+      <c r="D27" s="45" t="n">
         <f aca="false">SUM(D23:D26)</f>
         <v>14000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="40" t="s">
+      <c r="A29" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="B29" s="40"/>
-      <c r="C29" s="40"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="40"/>
-      <c r="F29" s="40"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32" t="s">
+      <c r="A30" s="33" t="s">
         <v>339</v>
       </c>
-      <c r="D30" s="45" t="n">
+      <c r="D30" s="44" t="n">
         <f aca="false">D19</f>
         <v>129000</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="32" t="s">
+      <c r="A31" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="D31" s="45" t="n">
+      <c r="D31" s="44" t="n">
         <f aca="false">D27</f>
         <v>14000</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="32" t="s">
+      <c r="A32" s="33" t="s">
         <v>340</v>
       </c>
-      <c r="D32" s="45" t="n">
+      <c r="D32" s="44" t="n">
         <f aca="false">(D30+D31)*Wyjaśnienia!$B$32</f>
         <v>17160</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="41" t="s">
+      <c r="A33" s="40" t="s">
         <v>191</v>
       </c>
-      <c r="D33" s="46" t="n">
+      <c r="D33" s="45" t="n">
         <f aca="false">SUM(D30:D32)</f>
         <v>160160</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="32" t="s">
+      <c r="A34" s="33" t="s">
         <v>192</v>
       </c>
-      <c r="D34" s="45" t="n">
+      <c r="D34" s="44" t="n">
         <f aca="false">D33*Wyjaśnienia!$B$35</f>
         <v>36836.8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="41" t="s">
+      <c r="A35" s="40" t="s">
         <v>193</v>
       </c>
-      <c r="D35" s="46" t="n">
+      <c r="D35" s="45" t="n">
         <f aca="false">D33+D34</f>
         <v>196996.8</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="40" t="s">
+      <c r="A37" s="17" t="s">
         <v>341</v>
       </c>
-      <c r="B37" s="40"/>
-      <c r="C37" s="40"/>
-      <c r="D37" s="40"/>
-      <c r="E37" s="40"/>
-      <c r="F37" s="40"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="39" t="s">
@@ -6795,247 +6874,248 @@
       <c r="D38" s="39"/>
       <c r="E38" s="39"/>
       <c r="F38" s="39"/>
+      <c r="G38" s="39"/>
     </row>
     <row r="39" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="42" t="s">
+      <c r="A39" s="41" t="s">
         <v>343</v>
       </c>
-      <c r="B39" s="42" t="s">
+      <c r="B39" s="41" t="s">
         <v>344</v>
       </c>
-      <c r="C39" s="42" t="s">
+      <c r="C39" s="41" t="s">
         <v>345</v>
       </c>
-      <c r="D39" s="42" t="s">
+      <c r="D39" s="41" t="s">
         <v>346</v>
       </c>
-      <c r="E39" s="42" t="s">
+      <c r="E39" s="41" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="43" t="n">
+      <c r="A40" s="42" t="n">
         <v>150</v>
       </c>
-      <c r="B40" s="43" t="n">
+      <c r="B40" s="42" t="n">
         <f aca="false">A40*Wyjaśnienia!$B$48</f>
         <v>300</v>
       </c>
-      <c r="C40" s="43" t="n">
+      <c r="C40" s="42" t="n">
         <f aca="false">ROUNDUP(B40/100,0)</f>
         <v>3</v>
       </c>
-      <c r="D40" s="45" t="n">
+      <c r="D40" s="44" t="n">
         <f aca="false">C40*Wyjaśnienia!$B$49</f>
         <v>1500</v>
       </c>
-      <c r="E40" s="43" t="n">
+      <c r="E40" s="42" t="n">
         <f aca="false">ROUNDUP(B40*Wyjaśnienia!$B$52/60,0)</f>
         <v>150</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="43" t="n">
+      <c r="A41" s="42" t="n">
         <v>1000</v>
       </c>
-      <c r="B41" s="43" t="n">
+      <c r="B41" s="42" t="n">
         <f aca="false">A41*Wyjaśnienia!$B$48</f>
         <v>2000</v>
       </c>
-      <c r="C41" s="43" t="n">
+      <c r="C41" s="42" t="n">
         <f aca="false">ROUNDUP(B41/100,0)</f>
         <v>20</v>
       </c>
-      <c r="D41" s="45" t="n">
+      <c r="D41" s="44" t="n">
         <f aca="false">C41*Wyjaśnienia!$B$49</f>
         <v>10000</v>
       </c>
-      <c r="E41" s="43" t="n">
+      <c r="E41" s="42" t="n">
         <f aca="false">ROUNDUP(B41*Wyjaśnienia!$B$52/60,0)</f>
         <v>1000</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="43" t="n">
+      <c r="A42" s="42" t="n">
         <v>10000</v>
       </c>
-      <c r="B42" s="43" t="n">
+      <c r="B42" s="42" t="n">
         <f aca="false">A42*Wyjaśnienia!$B$48</f>
         <v>20000</v>
       </c>
-      <c r="C42" s="43" t="n">
+      <c r="C42" s="42" t="n">
         <f aca="false">ROUNDUP(B42/100,0)</f>
         <v>200</v>
       </c>
-      <c r="D42" s="45" t="n">
+      <c r="D42" s="44" t="n">
         <f aca="false">C42*Wyjaśnienia!$B$49</f>
         <v>100000</v>
       </c>
-      <c r="E42" s="43" t="n">
+      <c r="E42" s="42" t="n">
         <f aca="false">ROUNDUP(B42*Wyjaśnienia!$B$52/60,0)</f>
         <v>10000</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="43" t="n">
+      <c r="A43" s="42" t="n">
         <v>100000</v>
       </c>
-      <c r="B43" s="43" t="n">
+      <c r="B43" s="42" t="n">
         <f aca="false">A43*Wyjaśnienia!$B$48</f>
         <v>200000</v>
       </c>
-      <c r="C43" s="43" t="n">
+      <c r="C43" s="42" t="n">
         <f aca="false">ROUNDUP(B43/100,0)</f>
         <v>2000</v>
       </c>
-      <c r="D43" s="45" t="n">
+      <c r="D43" s="44" t="n">
         <f aca="false">C43*Wyjaśnienia!$B$49</f>
         <v>1000000</v>
       </c>
-      <c r="E43" s="43" t="n">
+      <c r="E43" s="42" t="n">
         <f aca="false">ROUNDUP(B43*Wyjaśnienia!$B$52/60,0)</f>
         <v>100000</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="43" t="n">
+      <c r="A44" s="42" t="n">
         <v>1000000</v>
       </c>
-      <c r="B44" s="43" t="n">
+      <c r="B44" s="42" t="n">
         <f aca="false">A44*Wyjaśnienia!$B$48</f>
         <v>2000000</v>
       </c>
-      <c r="C44" s="43" t="n">
+      <c r="C44" s="42" t="n">
         <f aca="false">ROUNDUP(B44/100,0)</f>
         <v>20000</v>
       </c>
-      <c r="D44" s="45" t="n">
+      <c r="D44" s="44" t="n">
         <f aca="false">C44*Wyjaśnienia!$B$49</f>
         <v>10000000</v>
       </c>
-      <c r="E44" s="43" t="n">
+      <c r="E44" s="42" t="n">
         <f aca="false">ROUNDUP(B44*Wyjaśnienia!$B$52/60,0)</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="42" t="s">
+      <c r="A46" s="41" t="s">
         <v>348</v>
       </c>
-      <c r="B46" s="42" t="s">
+      <c r="B46" s="41" t="s">
         <v>349</v>
       </c>
-      <c r="C46" s="42" t="s">
+      <c r="C46" s="41" t="s">
         <v>350</v>
       </c>
-      <c r="D46" s="42" t="s">
+      <c r="D46" s="41" t="s">
         <v>351</v>
       </c>
-      <c r="E46" s="42" t="s">
+      <c r="E46" s="41" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="43" t="n">
+      <c r="A47" s="42" t="n">
         <v>30</v>
       </c>
-      <c r="B47" s="43" t="n">
+      <c r="B47" s="42" t="n">
         <f aca="false">A47*Wyjaśnienia!$B$77</f>
         <v>60</v>
       </c>
-      <c r="C47" s="45" t="n">
+      <c r="C47" s="44" t="n">
         <f aca="false">B47*Wyjaśnienia!$B$78</f>
         <v>18000</v>
       </c>
-      <c r="D47" s="43" t="n">
+      <c r="D47" s="42" t="n">
         <f aca="false">B47*2</f>
         <v>120</v>
       </c>
-      <c r="E47" s="43" t="n">
+      <c r="E47" s="42" t="n">
         <f aca="false">ROUNDUP(B47/Wyjaśnienia!$B$79,0)</f>
         <v>6</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="43" t="n">
+      <c r="A48" s="42" t="n">
         <v>150</v>
       </c>
-      <c r="B48" s="43" t="n">
+      <c r="B48" s="42" t="n">
         <f aca="false">A48*Wyjaśnienia!$B$77</f>
         <v>300</v>
       </c>
-      <c r="C48" s="45" t="n">
+      <c r="C48" s="44" t="n">
         <f aca="false">B48*Wyjaśnienia!$B$78</f>
         <v>90000</v>
       </c>
-      <c r="D48" s="43" t="n">
+      <c r="D48" s="42" t="n">
         <f aca="false">B48*2</f>
         <v>600</v>
       </c>
-      <c r="E48" s="43" t="n">
+      <c r="E48" s="42" t="n">
         <f aca="false">ROUNDUP(B48/Wyjaśnienia!$B$79,0)</f>
         <v>30</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="43" t="n">
+      <c r="A49" s="42" t="n">
         <v>500</v>
       </c>
-      <c r="B49" s="43" t="n">
+      <c r="B49" s="42" t="n">
         <f aca="false">A49*Wyjaśnienia!$B$77</f>
         <v>1000</v>
       </c>
-      <c r="C49" s="45" t="n">
+      <c r="C49" s="44" t="n">
         <f aca="false">B49*Wyjaśnienia!$B$78</f>
         <v>300000</v>
       </c>
-      <c r="D49" s="43" t="n">
+      <c r="D49" s="42" t="n">
         <f aca="false">B49*2</f>
         <v>2000</v>
       </c>
-      <c r="E49" s="43" t="n">
+      <c r="E49" s="42" t="n">
         <f aca="false">ROUNDUP(B49/Wyjaśnienia!$B$79,0)</f>
         <v>100</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="43" t="n">
+      <c r="A50" s="42" t="n">
         <v>2000</v>
       </c>
-      <c r="B50" s="43" t="n">
+      <c r="B50" s="42" t="n">
         <f aca="false">A50*Wyjaśnienia!$B$77</f>
         <v>4000</v>
       </c>
-      <c r="C50" s="45" t="n">
+      <c r="C50" s="44" t="n">
         <f aca="false">B50*Wyjaśnienia!$B$78</f>
         <v>1200000</v>
       </c>
-      <c r="D50" s="43" t="n">
+      <c r="D50" s="42" t="n">
         <f aca="false">B50*2</f>
         <v>8000</v>
       </c>
-      <c r="E50" s="43" t="n">
+      <c r="E50" s="42" t="n">
         <f aca="false">ROUNDUP(B50/Wyjaśnienia!$B$79,0)</f>
         <v>400</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="43" t="n">
+      <c r="A51" s="42" t="n">
         <v>10000</v>
       </c>
-      <c r="B51" s="43" t="n">
+      <c r="B51" s="42" t="n">
         <f aca="false">A51*Wyjaśnienia!$B$77</f>
         <v>20000</v>
       </c>
-      <c r="C51" s="45" t="n">
+      <c r="C51" s="44" t="n">
         <f aca="false">B51*Wyjaśnienia!$B$78</f>
         <v>6000000</v>
       </c>
-      <c r="D51" s="43" t="n">
+      <c r="D51" s="42" t="n">
         <f aca="false">B51*2</f>
         <v>40000</v>
       </c>
-      <c r="E51" s="43" t="n">
+      <c r="E51" s="42" t="n">
         <f aca="false">ROUNDUP(B51/Wyjaśnienia!$B$79,0)</f>
         <v>2000</v>
       </c>
@@ -7049,9 +7129,10 @@
       <c r="D53" s="39"/>
       <c r="E53" s="39"/>
       <c r="F53" s="39"/>
+      <c r="G53" s="39"/>
     </row>
     <row r="55" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="17" t="s">
+      <c r="A55" s="46" t="s">
         <v>354</v>
       </c>
     </row>
@@ -7061,22 +7142,22 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="41" t="s">
+      <c r="A57" s="40" t="s">
         <v>128</v>
       </c>
-      <c r="B57" s="41" t="s">
+      <c r="B57" s="40" t="s">
         <v>323</v>
       </c>
-      <c r="C57" s="41" t="s">
+      <c r="C57" s="40" t="s">
         <v>160</v>
       </c>
-      <c r="D57" s="41" t="s">
+      <c r="D57" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="F57" s="41" t="s">
+      <c r="F57" s="40" t="s">
         <v>133</v>
       </c>
-      <c r="G57" s="41" t="s">
+      <c r="G57" s="40" t="s">
         <v>134</v>
       </c>
     </row>
@@ -7084,18 +7165,18 @@
       <c r="A58" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="B58" s="45" t="n">
+      <c r="B58" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="C58" s="43" t="n">
+      <c r="C58" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$24*2</f>
         <v>300</v>
       </c>
-      <c r="D58" s="45" t="n">
+      <c r="D58" s="44" t="n">
         <f aca="false">B58*C58</f>
         <v>0</v>
       </c>
-      <c r="F58" s="32" t="s">
+      <c r="F58" s="33" t="s">
         <v>357</v>
       </c>
       <c r="G58" s="26" t="s">
@@ -7106,18 +7187,18 @@
       <c r="A59" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="B59" s="45" t="n">
+      <c r="B59" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="C59" s="43" t="n">
+      <c r="C59" s="42" t="n">
         <f aca="false">Wyjaśnienia!$B$55*2</f>
         <v>300</v>
       </c>
-      <c r="D59" s="45" t="n">
+      <c r="D59" s="44" t="n">
         <f aca="false">B59*C59</f>
         <v>0</v>
       </c>
-      <c r="F59" s="32" t="s">
+      <c r="F59" s="33" t="s">
         <v>359</v>
       </c>
       <c r="G59" s="26" t="s">
@@ -7128,17 +7209,17 @@
       <c r="A60" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="B60" s="45" t="n">
+      <c r="B60" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="C60" s="43" t="s">
+      <c r="C60" s="42" t="s">
         <v>361</v>
       </c>
-      <c r="D60" s="45" t="n">
+      <c r="D60" s="44" t="n">
         <f aca="false">B60*C60</f>
         <v>0</v>
       </c>
-      <c r="F60" s="32" t="s">
+      <c r="F60" s="33" t="s">
         <v>362</v>
       </c>
       <c r="G60" s="26" t="s">
@@ -7149,17 +7230,17 @@
       <c r="A61" s="3" t="s">
         <v>363</v>
       </c>
-      <c r="B61" s="45" t="n">
+      <c r="B61" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="C61" s="43" t="s">
+      <c r="C61" s="42" t="s">
         <v>361</v>
       </c>
-      <c r="D61" s="45" t="n">
+      <c r="D61" s="44" t="n">
         <f aca="false">B61*C61</f>
         <v>0</v>
       </c>
-      <c r="F61" s="32" t="s">
+      <c r="F61" s="33" t="s">
         <v>364</v>
       </c>
       <c r="G61" s="26" t="s">
@@ -7167,26 +7248,26 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="41" t="s">
+      <c r="A62" s="40" t="s">
         <v>365</v>
       </c>
-      <c r="D62" s="46" t="n">
+      <c r="D62" s="45" t="n">
         <f aca="false">SUM(D58:D61)</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A53:G53"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7224,6 +7305,7 @@
       <c r="D1" s="36"/>
       <c r="E1" s="36"/>
       <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
@@ -7234,6 +7316,7 @@
       <c r="D2" s="29"/>
       <c r="E2" s="29"/>
       <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="29" t="s">
@@ -7244,6 +7327,7 @@
       <c r="D3" s="29"/>
       <c r="E3" s="29"/>
       <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="36" t="s">
@@ -7254,6 +7338,7 @@
       <c r="D5" s="36"/>
       <c r="E5" s="36"/>
       <c r="F5" s="36"/>
+      <c r="G5" s="36"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
@@ -7288,7 +7373,7 @@
       <c r="C7" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="D7" s="31" t="n">
+      <c r="D7" s="32" t="n">
         <f aca="false">B7+C7*Wyjaśnienia!$B$68/60</f>
         <v>30</v>
       </c>
@@ -7311,7 +7396,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="21"/>
-      <c r="D8" s="31" t="n">
+      <c r="D8" s="32" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$68/60</f>
         <v>25</v>
       </c>
@@ -7334,7 +7419,7 @@
         <v>60</v>
       </c>
       <c r="C9" s="21"/>
-      <c r="D9" s="31" t="n">
+      <c r="D9" s="32" t="n">
         <f aca="false">B9+C9*Wyjaśnienia!$B$68/60</f>
         <v>60</v>
       </c>
@@ -7357,7 +7442,7 @@
         <v>20</v>
       </c>
       <c r="C10" s="21"/>
-      <c r="D10" s="31" t="n">
+      <c r="D10" s="32" t="n">
         <f aca="false">B10+C10*Wyjaśnienia!$B$68/60</f>
         <v>20</v>
       </c>
@@ -7380,7 +7465,7 @@
         <v>40</v>
       </c>
       <c r="C11" s="21"/>
-      <c r="D11" s="31" t="n">
+      <c r="D11" s="32" t="n">
         <f aca="false">B11+C11*Wyjaśnienia!$B$68/60</f>
         <v>40</v>
       </c>
@@ -7403,7 +7488,7 @@
         <v>40</v>
       </c>
       <c r="C12" s="21"/>
-      <c r="D12" s="31" t="n">
+      <c r="D12" s="32" t="n">
         <f aca="false">B12+C12*Wyjaśnienia!$B$68/60</f>
         <v>40</v>
       </c>
@@ -7426,7 +7511,7 @@
         <v>25</v>
       </c>
       <c r="C13" s="21"/>
-      <c r="D13" s="31" t="n">
+      <c r="D13" s="32" t="n">
         <f aca="false">B13+C13*Wyjaśnienia!$B$68/60</f>
         <v>25</v>
       </c>
@@ -7449,7 +7534,7 @@
         <v>50</v>
       </c>
       <c r="C14" s="21"/>
-      <c r="D14" s="31" t="n">
+      <c r="D14" s="32" t="n">
         <f aca="false">B14+C14*Wyjaśnienia!$B$68/60</f>
         <v>50</v>
       </c>
@@ -7491,6 +7576,7 @@
       <c r="D17" s="36"/>
       <c r="E17" s="36"/>
       <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
@@ -7520,7 +7606,7 @@
         <f aca="false">Wyjaśnienia!$B$69</f>
         <v>180000</v>
       </c>
-      <c r="C19" s="31" t="n">
+      <c r="C19" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="8" t="n">
@@ -7542,7 +7628,7 @@
         <f aca="false">Wyjaśnienia!$B$70</f>
         <v>12000</v>
       </c>
-      <c r="C20" s="31" t="n">
+      <c r="C20" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="8" t="n">
@@ -7564,7 +7650,7 @@
         <f aca="false">Wyjaśnienia!$B$71</f>
         <v>1200</v>
       </c>
-      <c r="C21" s="31" t="n">
+      <c r="C21" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="8" t="n">
@@ -7585,7 +7671,7 @@
       <c r="B22" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C22" s="31" t="n">
+      <c r="C22" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="8" t="n">
@@ -7606,7 +7692,7 @@
       <c r="B23" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C23" s="31" t="n">
+      <c r="C23" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="8" t="n">
@@ -7627,7 +7713,7 @@
       <c r="B24" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C24" s="31" t="n">
+      <c r="C24" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="8" t="n">
@@ -7648,7 +7734,7 @@
       <c r="B25" s="8" t="n">
         <v>12000</v>
       </c>
-      <c r="C25" s="31" t="n">
+      <c r="C25" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="8" t="n">
@@ -7669,7 +7755,7 @@
       <c r="B26" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="31" t="n">
+      <c r="C26" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="8" t="n">
@@ -7690,7 +7776,7 @@
       <c r="B27" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="31" t="n">
+      <c r="C27" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="8" t="n">
@@ -7711,7 +7797,7 @@
       <c r="B28" s="8" t="n">
         <v>3000</v>
       </c>
-      <c r="C28" s="31" t="n">
+      <c r="C28" s="32" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="8" t="n">
@@ -7727,7 +7813,7 @@
         <v>184</v>
       </c>
       <c r="B29" s="8"/>
-      <c r="C29" s="31"/>
+      <c r="C29" s="32"/>
       <c r="D29" s="11" t="n">
         <f aca="false">SUM(D19:D28)</f>
         <v>208200</v>
@@ -7743,6 +7829,7 @@
       <c r="D31" s="36"/>
       <c r="E31" s="36"/>
       <c r="F31" s="36"/>
+      <c r="G31" s="36"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
@@ -7809,12 +7896,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A31:G31"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7852,6 +7939,7 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
       <c r="H1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7863,6 +7951,7 @@
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
       <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7874,6 +7963,7 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
       <c r="H3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7894,6 +7984,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
       <c r="H5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7938,7 +8029,7 @@
         <f aca="false">D7*Wyjaśnienia!$B$17</f>
         <v>9900</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="13" t="s">
         <v>397</v>
       </c>
       <c r="G7" s="26" t="s">
@@ -7981,6 +8072,7 @@
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
       <c r="H10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8019,7 +8111,7 @@
         <f aca="false">B12*C12</f>
         <v>8000</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="13" t="s">
         <v>399</v>
       </c>
       <c r="F12" s="3"/>
@@ -8042,7 +8134,7 @@
         <f aca="false">B13*C13</f>
         <v>1500</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="13" t="s">
         <v>401</v>
       </c>
       <c r="F13" s="3"/>
@@ -8065,7 +8157,7 @@
         <f aca="false">B14*C14</f>
         <v>4000</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="13" t="s">
         <v>403</v>
       </c>
       <c r="F14" s="3"/>
@@ -8088,7 +8180,7 @@
         <f aca="false">B15*C15</f>
         <v>32000</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="13" t="s">
         <v>405</v>
       </c>
       <c r="F15" s="3"/>
@@ -8111,7 +8203,7 @@
         <f aca="false">B16*C16</f>
         <v>0</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="13" t="s">
         <v>407</v>
       </c>
       <c r="G16" s="26" t="s">
@@ -8132,7 +8224,7 @@
         <f aca="false">B17*C17</f>
         <v>0</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="13" t="s">
         <v>409</v>
       </c>
       <c r="G17" s="26" t="s">
@@ -8153,7 +8245,7 @@
         <f aca="false">B18*C18</f>
         <v>0</v>
       </c>
-      <c r="E18" s="15" t="s">
+      <c r="E18" s="13" t="s">
         <v>411</v>
       </c>
       <c r="G18" s="26" t="s">
@@ -8174,7 +8266,7 @@
         <f aca="false">B19*C19</f>
         <v>0</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="E19" s="13" t="s">
         <v>413</v>
       </c>
       <c r="G19" s="26" t="s">
@@ -8208,6 +8300,7 @@
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
       <c r="H22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8282,7 +8375,7 @@
       </c>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
-      <c r="D28" s="30" t="n">
+      <c r="D28" s="31" t="n">
         <f aca="false">D26+D27</f>
         <v>76319.04</v>
       </c>
@@ -8369,12 +8462,12 @@
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A22:G22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Arkusz: zakładki Budżet Rozmowy z AI i Budżet Piosenki wielką literą
Nazwy dwóch zakładek pisane małą literą odstawały od pozostałych siedmiu.
Ujednolicone wraz z odmianą w opisach wewnątrz arkusza, w formułach i w
dokumentach powołujących się na te zakładki. Kotwice adresów bez zmian, bo
powstają z nazwy zapisanej małymi literami.

Sumy bez zmian: RAZEM 1 839 251,76 zł.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -9,8 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="Wyjaśnienia" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Budżet rozmowy z AI" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Budżet piosenki" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Budżet Rozmowy z AI" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Budżet Piosenki" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Budżet Plakatu" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Budżet Filmu" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Budżet Akademii" sheetId="6" state="visible" r:id="rId8"/>
@@ -48,13 +48,13 @@
     <t xml:space="preserve">Kwota netto</t>
   </si>
   <si>
-    <t xml:space="preserve">Budżet rozmowy z AI - nagrody, ocena i promocja</t>
+    <t xml:space="preserve">Budżet Rozmowy z AI - nagrody, ocena i promocja</t>
   </si>
   <si>
     <t xml:space="preserve">Fundator puli nagród</t>
   </si>
   <si>
-    <t xml:space="preserve">Budżet piosenki - plebiscyt na piosenkę</t>
+    <t xml:space="preserve">Budżet Piosenki - plebiscyt na piosenkę</t>
   </si>
   <si>
     <t xml:space="preserve">Sponsor plebiscytu</t>
@@ -189,10 +189,10 @@
     <t xml:space="preserve">Medal zwycięzcy i dyplomy piosenki (netto)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ten sam medal co w plebiscycie na rozmowę, cena jak w Budżecie rozmowy z AI.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rezerwa w Budżecie rozmowy z AI</t>
+    <t xml:space="preserve">Ten sam medal co w plebiscycie na rozmowę, cena jak w Budżecie Rozmowy z AI.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rezerwa w Budżecie Rozmowy z AI</t>
   </si>
   <si>
     <t xml:space="preserve">Narzut na nieprzewidziane.</t>
@@ -204,7 +204,7 @@
     <t xml:space="preserve">Narzut wynagrodzenia podmiotu, który wykona tę część, liczony wyłącznie od jego własnej pracy. Koszty zewnętrzne - notariusz, opłaty urzędowe, księgowość, agencja, druk, studio - wchodzą do budżetu w kwotach, jakie wystawi dostawca, bez narzutu. Rezerwa 10% liczona jest osobno, od pracy i kosztów razem, bo przekroczenie może wystąpić po obu stronach.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rezerwa w Budżecie piosenki</t>
+    <t xml:space="preserve">Rezerwa w Budżecie Piosenki</t>
   </si>
   <si>
     <t xml:space="preserve">Stawka VAT</t>
@@ -225,7 +225,7 @@
     <t xml:space="preserve">Realizacja części artystycznej gali</t>
   </si>
   <si>
-    <t xml:space="preserve">Po wpisaniu tych kwot rosną Budżet piosenki, Budżet Plakatu i Budżet Filmu. W Budżecie Plakatu czekają na wycenę cztery pozycje, w Budżecie Filmu pięć - wszystkie opisane w kolumnie Uwagi.</t>
+    <t xml:space="preserve">Po wpisaniu tych kwot rosną Budżet Piosenki, Budżet Plakatu i Budżet Filmu. W Budżecie Plakatu czekają na wycenę cztery pozycje, w Budżecie Filmu pięć - wszystkie opisane w kolumnie Uwagi.</t>
   </si>
   <si>
     <t xml:space="preserve">JAK CZYTAĆ BUDŻETY</t>
@@ -258,7 +258,7 @@
     <t xml:space="preserve">Honorarium podstawowe czytelnika (netto)</t>
   </si>
   <si>
-    <t xml:space="preserve">Przeniesione z Budżetu rozmowy z AI. Voucher jest dodatkiem, nie zamiennikiem.</t>
+    <t xml:space="preserve">Przeniesione z Budżetu Rozmowy z AI. Voucher jest dodatkiem, nie zamiennikiem.</t>
   </si>
   <si>
     <t xml:space="preserve">Liczba czytelników w pierwszej edycji</t>
@@ -948,7 +948,7 @@
     <t xml:space="preserve">Honorarium podstawowe czytelników rozmów</t>
   </si>
   <si>
-    <t xml:space="preserve">przeniesione z Budżetu rozmowy z AI</t>
+    <t xml:space="preserve">przeniesione z Budżetu Rozmowy z AI</t>
   </si>
   <si>
     <t xml:space="preserve">Vouchery za oceniane rozmowy</t>
@@ -1940,7 +1940,7 @@
         <v>7</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">'Budżet rozmowy z AI'!$D$39</f>
+        <f aca="false">'Budżet Rozmowy z AI'!$D$39</f>
         <v>547809.76</v>
       </c>
       <c r="D6" s="3"/>
@@ -1957,7 +1957,7 @@
         <v>9</v>
       </c>
       <c r="C7" s="8" t="n">
-        <f aca="false">'Budżet piosenki'!$D$34</f>
+        <f aca="false">'Budżet Piosenki'!$D$34</f>
         <v>265960</v>
       </c>
       <c r="D7" s="3"/>
@@ -2053,7 +2053,7 @@
         <v>22</v>
       </c>
       <c r="C14" s="11" t="n">
-        <f aca="false">'Budżet rozmowy z AI'!$D$39+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$39+'Budżet Uruchomienia'!$D$28+'Budżet piosenki'!$D$34+'Budżet Plakatu'!$D$37+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$36</f>
+        <f aca="false">'Budżet Rozmowy z AI'!$D$39+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$39+'Budżet Uruchomienia'!$D$28+'Budżet Piosenki'!$D$34+'Budżet Plakatu'!$D$37+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$36</f>
         <v>1839251.76</v>
       </c>
       <c r="D14" s="3"/>

</xml_diff>

<commit_message>
Oferta filmowa: weryfikacja historii filmu rozliczana od liczby zgłoszeń
Pozycja stała w kosztorysie jako ryczałt 25 godzin, choć skaluje się z liczbą
zgłoszeń dokładnie tak jak kontrola formalna. Teraz ma 5 godzin na metodę i
narzędzie oraz 8 minut na zgłoszenie: przy 150 zgłoszeniach wychodzi te same 25
godzin, przy 15 - siedem. Razem z kontrolą formalną obie pozycje zależne od
frekwencji schodzą wtedy z 55 godzin do 10.

Kwota oferty bez zmian, 281 600 zł netto. Arkusz liczył tę kolumnę od początku,
wiersz miał tylko wpisany ryczałt w kolumnie godzin stałych.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -5363,9 +5363,11 @@
         <v>263</v>
       </c>
       <c r="B8" s="21" t="n">
-        <v>25</v>
-      </c>
-      <c r="C8" s="21"/>
+        <v>5</v>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="D8" s="34" t="n">
         <f aca="false">B8+C8*Wyjaśnienia!$B$68/60</f>
         <v>25</v>

</xml_diff>

<commit_message>
Budżet Filmu: podsumowanie wróciło pod swoje etykiety
Przy wstawianiu wierszy kopii archiwalnej formuły podsumowania trafiły o wiersz
niżej niż ich nazwy, więc na stronie przy "Pracy organizatora" stała kwota
nagród, przy "RAZEM NETTO" rezerwa, a prawdziwa kwota brutto wisiała w wierszu
bez etykiety. Formuły przesunięte na swoje miejsca, odwołania w Wyjaśnieniach
poprawione.

Wartości bez zmian: praca 69 850 zł, rezerwa 11 226 zł, RAZEM NETTO 296 776 zł,
brutto 365 034,48 zł, suma całości 1 880 187,76 zł.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/budzet-edycji-pierwszej.xlsx
+++ b/budzet-edycji-pierwszej.xlsx
@@ -2006,7 +2006,7 @@
         <v>13</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">'Budżet Filmu'!$D$39</f>
+        <f aca="false">'Budżet Filmu'!$D$38</f>
         <v>296776</v>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
         <v>22</v>
       </c>
       <c r="C14" s="11" t="n">
-        <f aca="false">'Budżet Rozmowy z AI'!$D$39+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$39+'Budżet Uruchomienia'!$D$28+'Budżet Piosenki'!$D$34+'Budżet Plakatu'!$D$37+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$39</f>
+        <f aca="false">'Budżet Rozmowy z AI'!$D$39+'Budżet Gali'!$D$26+'Budżet Antologii'!$D$39+'Budżet Uruchomienia'!$D$28+'Budżet Piosenki'!$D$34+'Budżet Plakatu'!$D$37+'Budżet Akademii'!$D$33+'Budżet Filmu'!$D$38</f>
         <v>1880187.76</v>
       </c>
       <c r="D14" s="3"/>
@@ -5882,8 +5882,8 @@
         <v>188</v>
       </c>
       <c r="D35" s="8" t="n">
-        <f aca="false">Wyjaśnienia!$B$69+Wyjaśnienia!$B$70</f>
-        <v>192000</v>
+        <f aca="false">E16</f>
+        <v>69850</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5891,8 +5891,8 @@
         <v>224</v>
       </c>
       <c r="D36" s="8" t="n">
-        <f aca="false">E16</f>
-        <v>69850</v>
+        <f aca="false">D31-D34</f>
+        <v>23700</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5900,8 +5900,8 @@
         <v>190</v>
       </c>
       <c r="D37" s="8" t="n">
-        <f aca="false">D31-D35</f>
-        <v>23700</v>
+        <f aca="false">(D35+D36)*Wyjaśnienia!$B$76</f>
+        <v>11226</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5909,8 +5909,8 @@
         <v>192</v>
       </c>
       <c r="D38" s="11" t="n">
-        <f aca="false">(D36+D37)*Wyjaśnienia!$B$76</f>
-        <v>11226</v>
+        <f aca="false">SUM(D34:D37)</f>
+        <v>296776</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5918,8 +5918,8 @@
         <v>193</v>
       </c>
       <c r="D39" s="8" t="n">
-        <f aca="false">SUM(D35:D38)</f>
-        <v>296776</v>
+        <f aca="false">D38*Wyjaśnienia!$B$35</f>
+        <v>68258.48</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5927,16 +5927,11 @@
         <v>194</v>
       </c>
       <c r="D40" s="11" t="n">
-        <f aca="false">D39*Wyjaśnienia!$B$35</f>
-        <v>68258.48</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D41" s="3" t="n">
-        <f aca="false">D39+D40</f>
+        <f aca="false">D38+D39</f>
         <v>365034.48</v>
       </c>
     </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:G1"/>

</xml_diff>